<commit_message>
Fix Set 2 domain length to 640 nm and tidy notes after audit
Set 2 renders show 640/lambda stripes, not 1280/lambda, so waves, c min and
c max now use L = 640 (conflict with sine.m flagged on the Notes sheet).
Also: correct the c min/c max wording, the worked delta example and the
'unrounded' claim, make the .vtk name column General so the formula survives
editing, and add a do-not-sort warning for the floating renders.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011WnE18kmcTTQHQwwBdKitt
</commit_message>
<xml_diff>
--- a/CM_Sweep_Sets_1_2.xlsx
+++ b/CM_Sweep_Sets_1_2.xlsx
@@ -83,7 +83,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">avg - amp when the domain holds &gt;= 0.75 waves, otherwise the sine value at the end of the domain (sine.m starts at phase 0 at y = 0). Closed-form estimate; see Notes.</t>
+          <t xml:space="preserve">avg - amp when the domain holds &gt;= 0.75 waves. With fewer waves, the lowest value reached: avg (at y = 0) or the sine value at the end of the domain, whichever is lower. Closed-form estimate of the sine.m field; see Notes.</t>
         </r>
       </text>
     </comment>
@@ -95,7 +95,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">avg + amp when the domain holds &gt;= 0.25 waves, otherwise the sine value at the end of the domain. See Notes.</t>
+          <t xml:space="preserve">avg + amp when the domain holds &gt;= 0.25 waves, otherwise the sine value at the end of the domain (the highest value reached). See Notes.</t>
         </r>
       </text>
     </comment>
@@ -107,7 +107,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, unrounded. Units not stated in the source file.</t>
+          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, kept at full precision (15 significant digits). Units not stated in the source file.</t>
         </r>
       </text>
     </comment>
@@ -131,7 +131,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, unrounded. Units not stated in the source file.</t>
+          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, kept at full precision (15 significant digits). Units not stated in the source file.</t>
         </r>
       </text>
     </comment>
@@ -143,7 +143,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, unrounded. Units not stated in the source file.</t>
+          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, kept at full precision (15 significant digits). Units not stated in the source file.</t>
         </r>
       </text>
     </comment>
@@ -155,7 +155,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, unrounded. Units not stated in the source file.</t>
+          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, kept at full precision (15 significant digits). Units not stated in the source file.</t>
         </r>
       </text>
     </comment>
@@ -191,7 +191,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Inferred from sine.m / write_vtk (set2_pt7.vtk). Edit if your file names differ.</t>
+          <t xml:space="preserve">Formula: set&lt;N&gt;_pt&lt;point&gt;.vtk, inferred from sine.m / write_vtk (set2_pt7.vtk). Overwrite with the real file name if yours differ.</t>
         </r>
       </text>
     </comment>
@@ -261,7 +261,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">avg - amp when the domain holds &gt;= 0.75 waves, otherwise the sine value at the end of the domain (sine.m starts at phase 0 at y = 0). Closed-form estimate; see Notes.</t>
+          <t xml:space="preserve">avg - amp when the domain holds &gt;= 0.75 waves. With fewer waves, the lowest value reached: avg (at y = 0) or the sine value at the end of the domain, whichever is lower. Closed-form estimate of the sine.m field; see Notes.</t>
         </r>
       </text>
     </comment>
@@ -273,7 +273,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">avg + amp when the domain holds &gt;= 0.25 waves, otherwise the sine value at the end of the domain. See Notes.</t>
+          <t xml:space="preserve">avg + amp when the domain holds &gt;= 0.25 waves, otherwise the sine value at the end of the domain (the highest value reached). See Notes.</t>
         </r>
       </text>
     </comment>
@@ -285,7 +285,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, unrounded. Units not stated in the source file.</t>
+          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, kept at full precision (15 significant digits). Units not stated in the source file.</t>
         </r>
       </text>
     </comment>
@@ -309,7 +309,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, unrounded. Units not stated in the source file.</t>
+          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, kept at full precision (15 significant digits). Units not stated in the source file.</t>
         </r>
       </text>
     </comment>
@@ -321,7 +321,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, unrounded. Units not stated in the source file.</t>
+          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, kept at full precision (15 significant digits). Units not stated in the source file.</t>
         </r>
       </text>
     </comment>
@@ -333,7 +333,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, unrounded. Units not stated in the source file.</t>
+          <t xml:space="preserve">Shanghai ML prediction, from the set CSV, kept at full precision (15 significant digits). Units not stated in the source file.</t>
         </r>
       </text>
     </comment>
@@ -369,7 +369,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Inferred from sine.m / write_vtk (set2_pt7.vtk). Edit if your file names differ.</t>
+          <t xml:space="preserve">Formula: set&lt;N&gt;_pt&lt;point&gt;.vtk, inferred from sine.m / write_vtk (set2_pt7.vtk). Overwrite with the real file name if yours differ.</t>
         </r>
       </text>
     </comment>
@@ -378,7 +378,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="66">
   <si>
     <t xml:space="preserve">Point</t>
   </si>
@@ -467,13 +467,13 @@
     <t xml:space="preserve">Set 1 domain length L (nm)</t>
   </si>
   <si>
-    <t xml:space="preserve">Assumption: taken from the 'waves / 640 nm' column header in Aum's 2D sweep sheet. Confirm for the 3D set 1 runs.</t>
+    <t xml:space="preserve">Assumption: taken from the 'waves / 640 nm' header in Aum's 2D sweep sheet; the Set 1 renders agree (stripe count = 640/λ).</t>
   </si>
   <si>
     <t xml:space="preserve">Set 2 domain length L (nm)</t>
   </si>
   <si>
-    <t xml:space="preserve">Assumption: sine.m uses Ny = 1280 grid points along y (1 nm spacing assumed) for set2_pt7. Confirm it is the same for all 10 set 2 points.</t>
+    <t xml:space="preserve">Assumption: set to 640 because all 10 Set 2 renders show 640/λ waves (e.g. λ = 640 shows one wave, λ = 80 shows eight). sine.m (Ny = 1280, wv = 1280 for set2_pt7) points to 1280 instead, so the two disagree. Confirm which grid set 2 used; changing this cell updates waves, c min and c max.</t>
   </si>
   <si>
     <t xml:space="preserve">Legend</t>
@@ -497,6 +497,12 @@
     <t xml:space="preserve">Cell to fill in: the SIM columns. Everything that depends on them (Δ columns, loop ratio, loop rank Δ) fills itself in.</t>
   </si>
   <si>
+    <t xml:space="preserve">Do not sort or filter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The renders are floating pictures anchored to rows 2–11, so they will not follow their rows if the table is sorted. Copy the values elsewhere to sort.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Column definitions</t>
   </si>
   <si>
@@ -515,13 +521,13 @@
     <t xml:space="preserve">c min, c max</t>
   </si>
   <si>
-    <t xml:space="preserve">avg ∓ amp when the domain holds enough of a wave to reach the peak/trough, otherwise the sine value at the end of the domain. Closed-form estimate of the field built in sine.m (c = avg + amp·sin(2πy/λ)). For set 1 point 2 (960 nm in 640 nm, 0.67 waves) this gives c min = 50.550; Aum's sheet lists 50.558. The 0.008 difference is probably grid sampling; every other point matches.</t>
+    <t xml:space="preserve">c min = avg − amp once the domain holds 0.75 waves; with fewer, the lowest value reached (avg at y = 0, or the sine value at the end of the domain if that is lower). c max = avg + amp once the domain holds 0.25 waves. Closed-form estimate of the field built in sine.m (c = avg + amp·sin(2πy/λ)). For set 1 point 2 (960 nm in 640 nm, 0.67 waves) this gives c min = 50.550; Aum's sheet lists 50.558, which a coarser 5 nm grid reproduces, so his 2D grid is probably coarser. Every other set 1 point matches.</t>
   </si>
   <si>
     <t xml:space="preserve">ML V1 / V3 stress, strain range, loop area</t>
   </si>
   <si>
-    <t xml:space="preserve">Shanghai ML predictions, copied unrounded from the CSVs. Units are not stated in the source files.</t>
+    <t xml:space="preserve">Shanghai ML predictions, copied from the CSVs at full precision (15 significant digits). Units are not stated in the source files.</t>
   </si>
   <si>
     <t xml:space="preserve">SIM columns</t>
@@ -533,7 +539,7 @@
     <t xml:space="preserve">Δ V1, Δ V3, Δ strain (pp)</t>
   </si>
   <si>
-    <t xml:space="preserve">SIM − ML. Blank until the SIM value is filled in. (Check against Aum's sample: 572 − 1421 = −850 after rounding.)</t>
+    <t xml:space="preserve">SIM − ML on the stored values. Blank until the SIM value is filled in. Aum's displayed Δ values come from unrounded SIM numbers, so typing his rounded values can differ by 1 (572 − 1421.16 = −849, his sheet shows −850).</t>
   </si>
   <si>
     <t xml:space="preserve">ML loop area ÷ SIM loop area.</t>
@@ -588,10 +594,9 @@
   </numFmts>
   <fonts count="10">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
@@ -792,7 +797,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2720,7 +2725,7 @@
       </c>
       <c r="E1" s="1" t="str">
         <f aca="false">"waves / "&amp;Notes!$B$5&amp;" nm"</f>
-        <v>waves / 1280 nm</v>
+        <v>waves / 640 nm</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>4</v>
@@ -2799,7 +2804,7 @@
       </c>
       <c r="E2" s="5" t="n">
         <f aca="false">Notes!$B$5/D2</f>
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F2" s="4" t="n">
         <v>0.88</v>
@@ -2870,7 +2875,7 @@
       </c>
       <c r="E3" s="5" t="n">
         <f aca="false">Notes!$B$5/D3</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F3" s="4" t="n">
         <v>0.92</v>
@@ -2941,7 +2946,7 @@
       </c>
       <c r="E4" s="5" t="n">
         <f aca="false">Notes!$B$5/D4</f>
-        <v>5.33333333333333</v>
+        <v>2.66666666666667</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>0.8</v>
@@ -3012,7 +3017,7 @@
       </c>
       <c r="E5" s="5" t="n">
         <f aca="false">Notes!$B$5/D5</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>1</v>
@@ -3083,7 +3088,7 @@
       </c>
       <c r="E6" s="5" t="n">
         <f aca="false">Notes!$B$5/D6</f>
-        <v>2.66666666666667</v>
+        <v>1.33333333333333</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>0.92</v>
@@ -3154,7 +3159,7 @@
       </c>
       <c r="E7" s="5" t="n">
         <f aca="false">Notes!$B$5/D7</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>0.8</v>
@@ -3225,14 +3230,14 @@
       </c>
       <c r="E8" s="5" t="n">
         <f aca="false">Notes!$B$5/D8</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>0.68</v>
       </c>
       <c r="G8" s="6" t="n">
         <f aca="false">C8+F8*IF(E8&gt;=0.75,-1,MIN(0,SIN(2*PI()*E8)))</f>
-        <v>49.87</v>
+        <v>50.55</v>
       </c>
       <c r="H8" s="6" t="n">
         <f aca="false">C8+F8*IF(E8&gt;=0.25,1,SIN(2*PI()*E8))</f>
@@ -3296,14 +3301,14 @@
       </c>
       <c r="E9" s="5" t="n">
         <f aca="false">Notes!$B$5/D9</f>
-        <v>1.23076923076923</v>
+        <v>0.615384615384615</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>0.56</v>
       </c>
       <c r="G9" s="6" t="n">
         <f aca="false">C9+F9*IF(E9&gt;=0.75,-1,MIN(0,SIN(2*PI()*E9)))</f>
-        <v>49.99</v>
+        <v>50.1786513113852</v>
       </c>
       <c r="H9" s="6" t="n">
         <f aca="false">C9+F9*IF(E9&gt;=0.25,1,SIN(2*PI()*E9))</f>
@@ -3367,7 +3372,7 @@
       </c>
       <c r="E10" s="5" t="n">
         <f aca="false">Notes!$B$5/D10</f>
-        <v>1.77777777777778</v>
+        <v>0.888888888888889</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>0.6</v>
@@ -3438,7 +3443,7 @@
       </c>
       <c r="E11" s="5" t="n">
         <f aca="false">Notes!$B$5/D11</f>
-        <v>1.77777777777778</v>
+        <v>0.888888888888889</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>0.04</v>
@@ -3515,7 +3520,7 @@
     <tabColor rgb="FF7F7F7F"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -3549,12 +3554,12 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
         <v>30</v>
       </c>
       <c r="B5" s="21" t="n">
-        <v>1280</v>
+        <v>640</v>
       </c>
       <c r="C5" s="20" t="s">
         <v>31</v>
@@ -3589,20 +3594,20 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
+    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="20" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="25" t="s">
+      <c r="C11" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="20" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="19" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="25" t="s">
         <v>42</v>
       </c>
@@ -3610,7 +3615,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="25" t="s">
         <v>44</v>
       </c>
@@ -3618,7 +3623,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="25" t="s">
         <v>46</v>
       </c>
@@ -3642,134 +3647,142 @@
         <v>51</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="20" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="25" t="s">
+      <c r="C20" s="20" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="20" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="25" t="s">
-        <v>24</v>
-      </c>
       <c r="C21" s="20" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C22" s="20" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="19" t="s">
-        <v>56</v>
+      <c r="C23" s="20" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="C25" s="20" t="s">
+      <c r="A25" s="19" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="B26" s="26" t="n">
-        <v>572</v>
+        <v>59</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B27" s="26" t="n">
-        <v>796</v>
+        <v>572</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="B28" s="27" t="n">
-        <v>4.95</v>
+        <v>11</v>
+      </c>
+      <c r="B28" s="26" t="n">
+        <v>796</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B29" s="27" t="n">
-        <v>5.57</v>
+        <v>4.95</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="B30" s="28" t="n">
-        <v>0.931</v>
+        <v>17</v>
+      </c>
+      <c r="B30" s="27" t="n">
+        <v>5.57</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B31" s="28" t="n">
-        <v>0.618</v>
+        <v>0.931</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B32" s="28" t="n">
+        <v>0.618</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="B32" s="29" t="n">
+      <c r="B33" s="29" t="n">
         <v>0.000178</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="19" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="C35" s="20" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="19" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="20" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C36" s="20" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="20" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="20" t="s">
-        <v>60</v>
-      </c>
       <c r="C37" s="20" t="s">
-        <v>63</v>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="C38" s="20" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Combined and Charts tabs, fix comment-box anchors
Combined stacks both sets (all cells link to the Set sheets) with a Pearson r
table, ML vs SIM, per set and overall. Charts holds four ML vs SIM scatter
plots that fill in as SIM values are entered. Header comments now pop up beside
their own cell instead of in one fixed spot.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011WnE18kmcTTQHQwwBdKitt
</commit_message>
<xml_diff>
--- a/CM_Sweep_Sets_1_2.xlsx
+++ b/CM_Sweep_Sets_1_2.xlsx
@@ -10,7 +10,9 @@
   <sheets>
     <sheet name="Set 1" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Set 2" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Notes" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Combined" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Charts" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Notes" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -378,7 +380,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="89">
   <si>
     <t xml:space="preserve">Point</t>
   </si>
@@ -455,6 +457,60 @@
     <t xml:space="preserve">CM field (.vtk)</t>
   </si>
   <si>
+    <t xml:space="preserve">Set</t>
+  </si>
+  <si>
+    <t xml:space="preserve">waves / L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pearson r, ML vs SIM (blank until at least 3 points have a SIM value)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n Set 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">r Set 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n Set 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">r Set 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n all</t>
+  </si>
+  <si>
+    <t xml:space="preserve">r all</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V1 stress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V3 stress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strain range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loop area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ML vs SIM scatter plots</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Points appear as SIM values are filled in on the Set sheets. Stress-strain curves will be added once the raw cycle data is available.</t>
+  </si>
+  <si>
     <t xml:space="preserve">CM sweep, Sets 1 and 2: notes, assumptions and legend</t>
   </si>
   <si>
@@ -551,6 +607,18 @@
     <t xml:space="preserve">set&lt;N&gt;_pt&lt;point&gt;.vtk, inferred from the write_vtk call in sine.m ('set2_pt7.vtk'). Aum's sheet uses a longer path pattern.</t>
   </si>
   <si>
+    <t xml:space="preserve">Combined sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sets 1 and 2 stacked into 20 rows. Every cell is a link to the Set sheets (green text), so nothing is typed here. SIM-dependent cells stay blank until the SIM values exist. Below the table, Pearson r between each ML metric and its SIM value, per set and for all 20 points; it needs at least 3 points with a SIM value. With so few points r is only indicative.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charts sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scatter plots of ML (x) against SIM (y) for V1, V3, strain range and loop area, one series per set. They read the Set sheets directly, so points appear as SIM values are filled in. Stress-strain curves are not here yet; they need the raw cycle data.</t>
+  </si>
+  <si>
     <t xml:space="preserve">ParaView renders from VTK_Field_Report.xlsx, one per point. They appear to be auto-scaled to each field's own range, so amplitude differences between points are not visible.</t>
   </si>
   <si>
@@ -576,6 +644,9 @@
   </si>
   <si>
     <t xml:space="preserve">Confirm the domain lengths above and the .vtk naming.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stress-strain curves and any 2D / pseudo-2D comparison tabs are not built: they need the raw cycle data and 2D results.</t>
   </si>
 </sst>
 </file>
@@ -592,7 +663,7 @@
     <numFmt numFmtId="170" formatCode="0.000000"/>
     <numFmt numFmtId="171" formatCode="@"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="15">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -642,11 +713,45 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="12"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -732,7 +837,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -801,7 +906,59 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -809,7 +966,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -833,7 +990,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -887,7 +1044,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -904,14 +1061,14 @@
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF2E75B6"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FFC55A11"/>
       <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF878787"/>
       <rgbColor rgb="FF1F3864"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
@@ -923,6 +1080,1882 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>V1 stress: ML vs SIM</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Set 1"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Set 1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="1f3864"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1f3864"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Set 1'!$I$2:$I$11</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>1421.15811288509</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1380.32366821806</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1408.29891867377</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1409.06706888271</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1407.499351274</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1407.29955396803</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1409.21728292278</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1402.53857129639</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1403.69923690996</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1404.60593589585</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Set 1'!$J$2:$J$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Set 2"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Set 2</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="c55a11"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="diamond"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="c55a11"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Set 2'!$I$2:$I$11</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>252.941476967729</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>252.932975417789</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>252.941476967729</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>244.381588889695</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>244.510942148903</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>244.518491839956</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>312.794696376031</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>312.794696376031</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>365.193909930287</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>365.193909930287</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Set 2'!$J$2:$J$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:axId val="49179135"/>
+        <c:axId val="92601320"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="49179135"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>ML V1 stress</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="92601320"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="92601320"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>SIM V1 stress</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="49179135"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>V3 stress: ML vs SIM</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Set 1"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Set 1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="1f3864"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1f3864"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Set 1'!$L$2:$L$11</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>1746.44105539347</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1744.46534440925</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1745.71301367738</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1746.41676186042</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1746.37860154084</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1745.65194202208</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1746.53707486242</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1746.17439480164</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1749.6312767733</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1749.65293005789</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Set 1'!$M$2:$M$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Set 2"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Set 2</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="c55a11"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="diamond"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="c55a11"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Set 2'!$L$2:$L$11</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>1272.77675106126</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1271.95778259744</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1274.36021618533</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1240.57518622454</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1241.43819349573</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1244.01182011071</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1161.08798987177</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1161.74939305885</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1153.32150850965</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1147.99922817314</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Set 2'!$M$2:$M$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:axId val="67022920"/>
+        <c:axId val="86970286"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="67022920"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>ML V3 stress</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="86970286"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="86970286"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>SIM V3 stress</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="67022920"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Strain range: ML vs SIM</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Set 1"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Set 1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="1f3864"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1f3864"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Set 1'!$O$2:$O$11</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>7.550116</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>7.61353533333333</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7.63308399999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7.62935699999999</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>7.63384199999999</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7.64592499999999</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.64266299999999</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7.64895899999999</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>7.64311299999999</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>7.64497699999999</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Set 1'!$P$2:$P$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Set 2"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Set 2</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="c55a11"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="diamond"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="c55a11"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Set 2'!$O$2:$O$11</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>7.51738999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>7.51647999999999</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7.51820299999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7.54008299999999</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>7.54310199999999</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7.54482499999999</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.66023</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7.660533</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>7.677769</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>7.680507</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Set 2'!$P$2:$P$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:axId val="31666765"/>
+        <c:axId val="42321796"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="31666765"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>ML strain range</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="42321796"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="42321796"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>SIM strain range</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="31666765"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Loop area: ML vs SIM</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Set 1"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Set 1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="1f3864"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1f3864"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Set 1'!$R$2:$R$11</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>263.959090135506</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>543.22722833229</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>632.07201334017</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>650.201104432882</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>656.430712583907</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>661.922490247295</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>722.735643650416</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>731.734711525745</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>741.859239328738</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>749.678589646605</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Set 1'!$S$2:$S$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Set 2"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Set 2</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="c55a11"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="diamond"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="c55a11"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Set 2'!$R$2:$R$11</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>194.037396072618</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>194.398322200401</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>195.04844034153</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>265.165023707051</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>265.45253270235</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>266.130053765627</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>612.727627704531</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>613.002453735894</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>646.382176644298</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>655.711579058753</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Set 2'!$S$2:$S$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:axId val="13051780"/>
+        <c:axId val="47218477"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="13051780"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>ML loop area</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="47218477"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="47218477"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>SIM loop area</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="13051780"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1675,6 +3708,131 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>4680</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>170640</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="20" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="571680"/>
+        <a:ext cx="6119640" cy="3599640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>4320</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>170640</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="21" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="6114960" y="571680"/>
+        <a:ext cx="6119640" cy="3599640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>4680</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>170640</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="22" name="Chart 3"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="4762440"/>
+        <a:ext cx="6119640" cy="3599640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>4320</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>170640</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="23" name="Chart 4"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="6114960" y="4762440"/>
+        <a:ext cx="6119640" cy="3599640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
@@ -3517,10 +5675,1986 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
+    <tabColor rgb="FF2E75B6"/>
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:U29"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="3" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="18" t="n">
+        <f aca="false">'Set 1'!A2</f>
+        <v>1</v>
+      </c>
+      <c r="C2" s="19" t="n">
+        <f aca="false">'Set 1'!C2</f>
+        <v>51</v>
+      </c>
+      <c r="D2" s="18" t="n">
+        <f aca="false">'Set 1'!D2</f>
+        <v>400</v>
+      </c>
+      <c r="E2" s="19" t="n">
+        <f aca="false">'Set 1'!E2</f>
+        <v>1.6</v>
+      </c>
+      <c r="F2" s="19" t="n">
+        <f aca="false">'Set 1'!F2</f>
+        <v>0.56</v>
+      </c>
+      <c r="G2" s="18" t="n">
+        <f aca="false">'Set 1'!I2</f>
+        <v>1421.15811288509</v>
+      </c>
+      <c r="H2" s="18" t="str">
+        <f aca="false">IF('Set 1'!J2="","",'Set 1'!J2)</f>
+        <v/>
+      </c>
+      <c r="I2" s="18" t="str">
+        <f aca="false">IF('Set 1'!K2="","",'Set 1'!K2)</f>
+        <v/>
+      </c>
+      <c r="J2" s="18" t="n">
+        <f aca="false">'Set 1'!L2</f>
+        <v>1746.44105539347</v>
+      </c>
+      <c r="K2" s="18" t="str">
+        <f aca="false">IF('Set 1'!M2="","",'Set 1'!M2)</f>
+        <v/>
+      </c>
+      <c r="L2" s="18" t="str">
+        <f aca="false">IF('Set 1'!N2="","",'Set 1'!N2)</f>
+        <v/>
+      </c>
+      <c r="M2" s="19" t="n">
+        <f aca="false">'Set 1'!O2</f>
+        <v>7.550116</v>
+      </c>
+      <c r="N2" s="19" t="str">
+        <f aca="false">IF('Set 1'!P2="","",'Set 1'!P2)</f>
+        <v/>
+      </c>
+      <c r="O2" s="19" t="str">
+        <f aca="false">IF('Set 1'!Q2="","",'Set 1'!Q2)</f>
+        <v/>
+      </c>
+      <c r="P2" s="20" t="n">
+        <f aca="false">'Set 1'!R2</f>
+        <v>263.959090135506</v>
+      </c>
+      <c r="Q2" s="19" t="str">
+        <f aca="false">IF('Set 1'!S2="","",'Set 1'!S2)</f>
+        <v/>
+      </c>
+      <c r="R2" s="20" t="str">
+        <f aca="false">IF('Set 1'!T2="","",'Set 1'!T2)</f>
+        <v/>
+      </c>
+      <c r="S2" s="21" t="str">
+        <f aca="false">IF('Set 1'!V2="","",'Set 1'!V2)</f>
+        <v/>
+      </c>
+      <c r="T2" s="21" t="str">
+        <f aca="false">IF('Set 1'!W2="","",'Set 1'!W2)</f>
+        <v/>
+      </c>
+      <c r="U2" s="22" t="str">
+        <f aca="false">IF('Set 1'!X2="","",'Set 1'!X2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="18" t="n">
+        <f aca="false">'Set 1'!A3</f>
+        <v>2</v>
+      </c>
+      <c r="C3" s="19" t="n">
+        <f aca="false">'Set 1'!C3</f>
+        <v>51</v>
+      </c>
+      <c r="D3" s="18" t="n">
+        <f aca="false">'Set 1'!D3</f>
+        <v>960</v>
+      </c>
+      <c r="E3" s="19" t="n">
+        <f aca="false">'Set 1'!E3</f>
+        <v>0.666666666666667</v>
+      </c>
+      <c r="F3" s="19" t="n">
+        <f aca="false">'Set 1'!F3</f>
+        <v>0.52</v>
+      </c>
+      <c r="G3" s="18" t="n">
+        <f aca="false">'Set 1'!I3</f>
+        <v>1380.32366821806</v>
+      </c>
+      <c r="H3" s="18" t="str">
+        <f aca="false">IF('Set 1'!J3="","",'Set 1'!J3)</f>
+        <v/>
+      </c>
+      <c r="I3" s="18" t="str">
+        <f aca="false">IF('Set 1'!K3="","",'Set 1'!K3)</f>
+        <v/>
+      </c>
+      <c r="J3" s="18" t="n">
+        <f aca="false">'Set 1'!L3</f>
+        <v>1744.46534440925</v>
+      </c>
+      <c r="K3" s="18" t="str">
+        <f aca="false">IF('Set 1'!M3="","",'Set 1'!M3)</f>
+        <v/>
+      </c>
+      <c r="L3" s="18" t="str">
+        <f aca="false">IF('Set 1'!N3="","",'Set 1'!N3)</f>
+        <v/>
+      </c>
+      <c r="M3" s="19" t="n">
+        <f aca="false">'Set 1'!O3</f>
+        <v>7.61353533333333</v>
+      </c>
+      <c r="N3" s="19" t="str">
+        <f aca="false">IF('Set 1'!P3="","",'Set 1'!P3)</f>
+        <v/>
+      </c>
+      <c r="O3" s="19" t="str">
+        <f aca="false">IF('Set 1'!Q3="","",'Set 1'!Q3)</f>
+        <v/>
+      </c>
+      <c r="P3" s="20" t="n">
+        <f aca="false">'Set 1'!R3</f>
+        <v>543.22722833229</v>
+      </c>
+      <c r="Q3" s="19" t="str">
+        <f aca="false">IF('Set 1'!S3="","",'Set 1'!S3)</f>
+        <v/>
+      </c>
+      <c r="R3" s="20" t="str">
+        <f aca="false">IF('Set 1'!T3="","",'Set 1'!T3)</f>
+        <v/>
+      </c>
+      <c r="S3" s="21" t="str">
+        <f aca="false">IF('Set 1'!V3="","",'Set 1'!V3)</f>
+        <v/>
+      </c>
+      <c r="T3" s="21" t="str">
+        <f aca="false">IF('Set 1'!W3="","",'Set 1'!W3)</f>
+        <v/>
+      </c>
+      <c r="U3" s="22" t="str">
+        <f aca="false">IF('Set 1'!X3="","",'Set 1'!X3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="18" t="n">
+        <f aca="false">'Set 1'!A4</f>
+        <v>3</v>
+      </c>
+      <c r="C4" s="19" t="n">
+        <f aca="false">'Set 1'!C4</f>
+        <v>51</v>
+      </c>
+      <c r="D4" s="18" t="n">
+        <f aca="false">'Set 1'!D4</f>
+        <v>480</v>
+      </c>
+      <c r="E4" s="19" t="n">
+        <f aca="false">'Set 1'!E4</f>
+        <v>1.33333333333333</v>
+      </c>
+      <c r="F4" s="19" t="n">
+        <f aca="false">'Set 1'!F4</f>
+        <v>0.52</v>
+      </c>
+      <c r="G4" s="18" t="n">
+        <f aca="false">'Set 1'!I4</f>
+        <v>1408.29891867377</v>
+      </c>
+      <c r="H4" s="18" t="str">
+        <f aca="false">IF('Set 1'!J4="","",'Set 1'!J4)</f>
+        <v/>
+      </c>
+      <c r="I4" s="18" t="str">
+        <f aca="false">IF('Set 1'!K4="","",'Set 1'!K4)</f>
+        <v/>
+      </c>
+      <c r="J4" s="18" t="n">
+        <f aca="false">'Set 1'!L4</f>
+        <v>1745.71301367738</v>
+      </c>
+      <c r="K4" s="18" t="str">
+        <f aca="false">IF('Set 1'!M4="","",'Set 1'!M4)</f>
+        <v/>
+      </c>
+      <c r="L4" s="18" t="str">
+        <f aca="false">IF('Set 1'!N4="","",'Set 1'!N4)</f>
+        <v/>
+      </c>
+      <c r="M4" s="19" t="n">
+        <f aca="false">'Set 1'!O4</f>
+        <v>7.63308399999999</v>
+      </c>
+      <c r="N4" s="19" t="str">
+        <f aca="false">IF('Set 1'!P4="","",'Set 1'!P4)</f>
+        <v/>
+      </c>
+      <c r="O4" s="19" t="str">
+        <f aca="false">IF('Set 1'!Q4="","",'Set 1'!Q4)</f>
+        <v/>
+      </c>
+      <c r="P4" s="20" t="n">
+        <f aca="false">'Set 1'!R4</f>
+        <v>632.07201334017</v>
+      </c>
+      <c r="Q4" s="19" t="str">
+        <f aca="false">IF('Set 1'!S4="","",'Set 1'!S4)</f>
+        <v/>
+      </c>
+      <c r="R4" s="20" t="str">
+        <f aca="false">IF('Set 1'!T4="","",'Set 1'!T4)</f>
+        <v/>
+      </c>
+      <c r="S4" s="21" t="str">
+        <f aca="false">IF('Set 1'!V4="","",'Set 1'!V4)</f>
+        <v/>
+      </c>
+      <c r="T4" s="21" t="str">
+        <f aca="false">IF('Set 1'!W4="","",'Set 1'!W4)</f>
+        <v/>
+      </c>
+      <c r="U4" s="22" t="str">
+        <f aca="false">IF('Set 1'!X4="","",'Set 1'!X4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="18" t="n">
+        <f aca="false">'Set 1'!A5</f>
+        <v>4</v>
+      </c>
+      <c r="C5" s="19" t="n">
+        <f aca="false">'Set 1'!C5</f>
+        <v>51</v>
+      </c>
+      <c r="D5" s="18" t="n">
+        <f aca="false">'Set 1'!D5</f>
+        <v>240</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <f aca="false">'Set 1'!E5</f>
+        <v>2.66666666666667</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <f aca="false">'Set 1'!F5</f>
+        <v>0.52</v>
+      </c>
+      <c r="G5" s="18" t="n">
+        <f aca="false">'Set 1'!I5</f>
+        <v>1409.06706888271</v>
+      </c>
+      <c r="H5" s="18" t="str">
+        <f aca="false">IF('Set 1'!J5="","",'Set 1'!J5)</f>
+        <v/>
+      </c>
+      <c r="I5" s="18" t="str">
+        <f aca="false">IF('Set 1'!K5="","",'Set 1'!K5)</f>
+        <v/>
+      </c>
+      <c r="J5" s="18" t="n">
+        <f aca="false">'Set 1'!L5</f>
+        <v>1746.41676186042</v>
+      </c>
+      <c r="K5" s="18" t="str">
+        <f aca="false">IF('Set 1'!M5="","",'Set 1'!M5)</f>
+        <v/>
+      </c>
+      <c r="L5" s="18" t="str">
+        <f aca="false">IF('Set 1'!N5="","",'Set 1'!N5)</f>
+        <v/>
+      </c>
+      <c r="M5" s="19" t="n">
+        <f aca="false">'Set 1'!O5</f>
+        <v>7.62935699999999</v>
+      </c>
+      <c r="N5" s="19" t="str">
+        <f aca="false">IF('Set 1'!P5="","",'Set 1'!P5)</f>
+        <v/>
+      </c>
+      <c r="O5" s="19" t="str">
+        <f aca="false">IF('Set 1'!Q5="","",'Set 1'!Q5)</f>
+        <v/>
+      </c>
+      <c r="P5" s="20" t="n">
+        <f aca="false">'Set 1'!R5</f>
+        <v>650.201104432882</v>
+      </c>
+      <c r="Q5" s="19" t="str">
+        <f aca="false">IF('Set 1'!S5="","",'Set 1'!S5)</f>
+        <v/>
+      </c>
+      <c r="R5" s="20" t="str">
+        <f aca="false">IF('Set 1'!T5="","",'Set 1'!T5)</f>
+        <v/>
+      </c>
+      <c r="S5" s="21" t="str">
+        <f aca="false">IF('Set 1'!V5="","",'Set 1'!V5)</f>
+        <v/>
+      </c>
+      <c r="T5" s="21" t="str">
+        <f aca="false">IF('Set 1'!W5="","",'Set 1'!W5)</f>
+        <v/>
+      </c>
+      <c r="U5" s="22" t="str">
+        <f aca="false">IF('Set 1'!X5="","",'Set 1'!X5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="18" t="n">
+        <f aca="false">'Set 1'!A6</f>
+        <v>5</v>
+      </c>
+      <c r="C6" s="19" t="n">
+        <f aca="false">'Set 1'!C6</f>
+        <v>50.95</v>
+      </c>
+      <c r="D6" s="18" t="n">
+        <f aca="false">'Set 1'!D6</f>
+        <v>240</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <f aca="false">'Set 1'!E6</f>
+        <v>2.66666666666667</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <f aca="false">'Set 1'!F6</f>
+        <v>0.52</v>
+      </c>
+      <c r="G6" s="18" t="n">
+        <f aca="false">'Set 1'!I6</f>
+        <v>1407.499351274</v>
+      </c>
+      <c r="H6" s="18" t="str">
+        <f aca="false">IF('Set 1'!J6="","",'Set 1'!J6)</f>
+        <v/>
+      </c>
+      <c r="I6" s="18" t="str">
+        <f aca="false">IF('Set 1'!K6="","",'Set 1'!K6)</f>
+        <v/>
+      </c>
+      <c r="J6" s="18" t="n">
+        <f aca="false">'Set 1'!L6</f>
+        <v>1746.37860154084</v>
+      </c>
+      <c r="K6" s="18" t="str">
+        <f aca="false">IF('Set 1'!M6="","",'Set 1'!M6)</f>
+        <v/>
+      </c>
+      <c r="L6" s="18" t="str">
+        <f aca="false">IF('Set 1'!N6="","",'Set 1'!N6)</f>
+        <v/>
+      </c>
+      <c r="M6" s="19" t="n">
+        <f aca="false">'Set 1'!O6</f>
+        <v>7.63384199999999</v>
+      </c>
+      <c r="N6" s="19" t="str">
+        <f aca="false">IF('Set 1'!P6="","",'Set 1'!P6)</f>
+        <v/>
+      </c>
+      <c r="O6" s="19" t="str">
+        <f aca="false">IF('Set 1'!Q6="","",'Set 1'!Q6)</f>
+        <v/>
+      </c>
+      <c r="P6" s="20" t="n">
+        <f aca="false">'Set 1'!R6</f>
+        <v>656.430712583907</v>
+      </c>
+      <c r="Q6" s="19" t="str">
+        <f aca="false">IF('Set 1'!S6="","",'Set 1'!S6)</f>
+        <v/>
+      </c>
+      <c r="R6" s="20" t="str">
+        <f aca="false">IF('Set 1'!T6="","",'Set 1'!T6)</f>
+        <v/>
+      </c>
+      <c r="S6" s="21" t="str">
+        <f aca="false">IF('Set 1'!V6="","",'Set 1'!V6)</f>
+        <v/>
+      </c>
+      <c r="T6" s="21" t="str">
+        <f aca="false">IF('Set 1'!W6="","",'Set 1'!W6)</f>
+        <v/>
+      </c>
+      <c r="U6" s="22" t="str">
+        <f aca="false">IF('Set 1'!X6="","",'Set 1'!X6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="18" t="n">
+        <f aca="false">'Set 1'!A7</f>
+        <v>6</v>
+      </c>
+      <c r="C7" s="19" t="n">
+        <f aca="false">'Set 1'!C7</f>
+        <v>50.95</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <f aca="false">'Set 1'!D7</f>
+        <v>320</v>
+      </c>
+      <c r="E7" s="19" t="n">
+        <f aca="false">'Set 1'!E7</f>
+        <v>2</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <f aca="false">'Set 1'!F7</f>
+        <v>0.52</v>
+      </c>
+      <c r="G7" s="18" t="n">
+        <f aca="false">'Set 1'!I7</f>
+        <v>1407.29955396803</v>
+      </c>
+      <c r="H7" s="18" t="str">
+        <f aca="false">IF('Set 1'!J7="","",'Set 1'!J7)</f>
+        <v/>
+      </c>
+      <c r="I7" s="18" t="str">
+        <f aca="false">IF('Set 1'!K7="","",'Set 1'!K7)</f>
+        <v/>
+      </c>
+      <c r="J7" s="18" t="n">
+        <f aca="false">'Set 1'!L7</f>
+        <v>1745.65194202208</v>
+      </c>
+      <c r="K7" s="18" t="str">
+        <f aca="false">IF('Set 1'!M7="","",'Set 1'!M7)</f>
+        <v/>
+      </c>
+      <c r="L7" s="18" t="str">
+        <f aca="false">IF('Set 1'!N7="","",'Set 1'!N7)</f>
+        <v/>
+      </c>
+      <c r="M7" s="19" t="n">
+        <f aca="false">'Set 1'!O7</f>
+        <v>7.64592499999999</v>
+      </c>
+      <c r="N7" s="19" t="str">
+        <f aca="false">IF('Set 1'!P7="","",'Set 1'!P7)</f>
+        <v/>
+      </c>
+      <c r="O7" s="19" t="str">
+        <f aca="false">IF('Set 1'!Q7="","",'Set 1'!Q7)</f>
+        <v/>
+      </c>
+      <c r="P7" s="20" t="n">
+        <f aca="false">'Set 1'!R7</f>
+        <v>661.922490247295</v>
+      </c>
+      <c r="Q7" s="19" t="str">
+        <f aca="false">IF('Set 1'!S7="","",'Set 1'!S7)</f>
+        <v/>
+      </c>
+      <c r="R7" s="20" t="str">
+        <f aca="false">IF('Set 1'!T7="","",'Set 1'!T7)</f>
+        <v/>
+      </c>
+      <c r="S7" s="21" t="str">
+        <f aca="false">IF('Set 1'!V7="","",'Set 1'!V7)</f>
+        <v/>
+      </c>
+      <c r="T7" s="21" t="str">
+        <f aca="false">IF('Set 1'!W7="","",'Set 1'!W7)</f>
+        <v/>
+      </c>
+      <c r="U7" s="22" t="str">
+        <f aca="false">IF('Set 1'!X7="","",'Set 1'!X7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="18" t="n">
+        <f aca="false">'Set 1'!A8</f>
+        <v>7</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <f aca="false">'Set 1'!C8</f>
+        <v>51</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <f aca="false">'Set 1'!D8</f>
+        <v>240</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <f aca="false">'Set 1'!E8</f>
+        <v>2.66666666666667</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <f aca="false">'Set 1'!F8</f>
+        <v>0.4</v>
+      </c>
+      <c r="G8" s="18" t="n">
+        <f aca="false">'Set 1'!I8</f>
+        <v>1409.21728292278</v>
+      </c>
+      <c r="H8" s="18" t="str">
+        <f aca="false">IF('Set 1'!J8="","",'Set 1'!J8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="18" t="str">
+        <f aca="false">IF('Set 1'!K8="","",'Set 1'!K8)</f>
+        <v/>
+      </c>
+      <c r="J8" s="18" t="n">
+        <f aca="false">'Set 1'!L8</f>
+        <v>1746.53707486242</v>
+      </c>
+      <c r="K8" s="18" t="str">
+        <f aca="false">IF('Set 1'!M8="","",'Set 1'!M8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="18" t="str">
+        <f aca="false">IF('Set 1'!N8="","",'Set 1'!N8)</f>
+        <v/>
+      </c>
+      <c r="M8" s="19" t="n">
+        <f aca="false">'Set 1'!O8</f>
+        <v>7.64266299999999</v>
+      </c>
+      <c r="N8" s="19" t="str">
+        <f aca="false">IF('Set 1'!P8="","",'Set 1'!P8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="19" t="str">
+        <f aca="false">IF('Set 1'!Q8="","",'Set 1'!Q8)</f>
+        <v/>
+      </c>
+      <c r="P8" s="20" t="n">
+        <f aca="false">'Set 1'!R8</f>
+        <v>722.735643650416</v>
+      </c>
+      <c r="Q8" s="19" t="str">
+        <f aca="false">IF('Set 1'!S8="","",'Set 1'!S8)</f>
+        <v/>
+      </c>
+      <c r="R8" s="20" t="str">
+        <f aca="false">IF('Set 1'!T8="","",'Set 1'!T8)</f>
+        <v/>
+      </c>
+      <c r="S8" s="21" t="str">
+        <f aca="false">IF('Set 1'!V8="","",'Set 1'!V8)</f>
+        <v/>
+      </c>
+      <c r="T8" s="21" t="str">
+        <f aca="false">IF('Set 1'!W8="","",'Set 1'!W8)</f>
+        <v/>
+      </c>
+      <c r="U8" s="22" t="str">
+        <f aca="false">IF('Set 1'!X8="","",'Set 1'!X8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="18" t="n">
+        <f aca="false">'Set 1'!A9</f>
+        <v>8</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <f aca="false">'Set 1'!C9</f>
+        <v>50.95</v>
+      </c>
+      <c r="D9" s="18" t="n">
+        <f aca="false">'Set 1'!D9</f>
+        <v>240</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <f aca="false">'Set 1'!E9</f>
+        <v>2.66666666666667</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <f aca="false">'Set 1'!F9</f>
+        <v>0.48</v>
+      </c>
+      <c r="G9" s="18" t="n">
+        <f aca="false">'Set 1'!I9</f>
+        <v>1402.53857129639</v>
+      </c>
+      <c r="H9" s="18" t="str">
+        <f aca="false">IF('Set 1'!J9="","",'Set 1'!J9)</f>
+        <v/>
+      </c>
+      <c r="I9" s="18" t="str">
+        <f aca="false">IF('Set 1'!K9="","",'Set 1'!K9)</f>
+        <v/>
+      </c>
+      <c r="J9" s="18" t="n">
+        <f aca="false">'Set 1'!L9</f>
+        <v>1746.17439480164</v>
+      </c>
+      <c r="K9" s="18" t="str">
+        <f aca="false">IF('Set 1'!M9="","",'Set 1'!M9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="18" t="str">
+        <f aca="false">IF('Set 1'!N9="","",'Set 1'!N9)</f>
+        <v/>
+      </c>
+      <c r="M9" s="19" t="n">
+        <f aca="false">'Set 1'!O9</f>
+        <v>7.64895899999999</v>
+      </c>
+      <c r="N9" s="19" t="str">
+        <f aca="false">IF('Set 1'!P9="","",'Set 1'!P9)</f>
+        <v/>
+      </c>
+      <c r="O9" s="19" t="str">
+        <f aca="false">IF('Set 1'!Q9="","",'Set 1'!Q9)</f>
+        <v/>
+      </c>
+      <c r="P9" s="20" t="n">
+        <f aca="false">'Set 1'!R9</f>
+        <v>731.734711525745</v>
+      </c>
+      <c r="Q9" s="19" t="str">
+        <f aca="false">IF('Set 1'!S9="","",'Set 1'!S9)</f>
+        <v/>
+      </c>
+      <c r="R9" s="20" t="str">
+        <f aca="false">IF('Set 1'!T9="","",'Set 1'!T9)</f>
+        <v/>
+      </c>
+      <c r="S9" s="21" t="str">
+        <f aca="false">IF('Set 1'!V9="","",'Set 1'!V9)</f>
+        <v/>
+      </c>
+      <c r="T9" s="21" t="str">
+        <f aca="false">IF('Set 1'!W9="","",'Set 1'!W9)</f>
+        <v/>
+      </c>
+      <c r="U9" s="22" t="str">
+        <f aca="false">IF('Set 1'!X9="","",'Set 1'!X9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="18" t="n">
+        <f aca="false">'Set 1'!A10</f>
+        <v>9</v>
+      </c>
+      <c r="C10" s="19" t="n">
+        <f aca="false">'Set 1'!C10</f>
+        <v>51</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <f aca="false">'Set 1'!D10</f>
+        <v>160</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <f aca="false">'Set 1'!E10</f>
+        <v>4</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <f aca="false">'Set 1'!F10</f>
+        <v>0.48</v>
+      </c>
+      <c r="G10" s="18" t="n">
+        <f aca="false">'Set 1'!I10</f>
+        <v>1403.69923690996</v>
+      </c>
+      <c r="H10" s="18" t="str">
+        <f aca="false">IF('Set 1'!J10="","",'Set 1'!J10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="18" t="str">
+        <f aca="false">IF('Set 1'!K10="","",'Set 1'!K10)</f>
+        <v/>
+      </c>
+      <c r="J10" s="18" t="n">
+        <f aca="false">'Set 1'!L10</f>
+        <v>1749.6312767733</v>
+      </c>
+      <c r="K10" s="18" t="str">
+        <f aca="false">IF('Set 1'!M10="","",'Set 1'!M10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="18" t="str">
+        <f aca="false">IF('Set 1'!N10="","",'Set 1'!N10)</f>
+        <v/>
+      </c>
+      <c r="M10" s="19" t="n">
+        <f aca="false">'Set 1'!O10</f>
+        <v>7.64311299999999</v>
+      </c>
+      <c r="N10" s="19" t="str">
+        <f aca="false">IF('Set 1'!P10="","",'Set 1'!P10)</f>
+        <v/>
+      </c>
+      <c r="O10" s="19" t="str">
+        <f aca="false">IF('Set 1'!Q10="","",'Set 1'!Q10)</f>
+        <v/>
+      </c>
+      <c r="P10" s="20" t="n">
+        <f aca="false">'Set 1'!R10</f>
+        <v>741.859239328738</v>
+      </c>
+      <c r="Q10" s="19" t="str">
+        <f aca="false">IF('Set 1'!S10="","",'Set 1'!S10)</f>
+        <v/>
+      </c>
+      <c r="R10" s="20" t="str">
+        <f aca="false">IF('Set 1'!T10="","",'Set 1'!T10)</f>
+        <v/>
+      </c>
+      <c r="S10" s="21" t="str">
+        <f aca="false">IF('Set 1'!V10="","",'Set 1'!V10)</f>
+        <v/>
+      </c>
+      <c r="T10" s="21" t="str">
+        <f aca="false">IF('Set 1'!W10="","",'Set 1'!W10)</f>
+        <v/>
+      </c>
+      <c r="U10" s="22" t="str">
+        <f aca="false">IF('Set 1'!X10="","",'Set 1'!X10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="18" t="n">
+        <f aca="false">'Set 1'!A11</f>
+        <v>10</v>
+      </c>
+      <c r="C11" s="19" t="n">
+        <f aca="false">'Set 1'!C11</f>
+        <v>51</v>
+      </c>
+      <c r="D11" s="18" t="n">
+        <f aca="false">'Set 1'!D11</f>
+        <v>160</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <f aca="false">'Set 1'!E11</f>
+        <v>4</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <f aca="false">'Set 1'!F11</f>
+        <v>0.44</v>
+      </c>
+      <c r="G11" s="18" t="n">
+        <f aca="false">'Set 1'!I11</f>
+        <v>1404.60593589585</v>
+      </c>
+      <c r="H11" s="18" t="str">
+        <f aca="false">IF('Set 1'!J11="","",'Set 1'!J11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="18" t="str">
+        <f aca="false">IF('Set 1'!K11="","",'Set 1'!K11)</f>
+        <v/>
+      </c>
+      <c r="J11" s="18" t="n">
+        <f aca="false">'Set 1'!L11</f>
+        <v>1749.65293005789</v>
+      </c>
+      <c r="K11" s="18" t="str">
+        <f aca="false">IF('Set 1'!M11="","",'Set 1'!M11)</f>
+        <v/>
+      </c>
+      <c r="L11" s="18" t="str">
+        <f aca="false">IF('Set 1'!N11="","",'Set 1'!N11)</f>
+        <v/>
+      </c>
+      <c r="M11" s="19" t="n">
+        <f aca="false">'Set 1'!O11</f>
+        <v>7.64497699999999</v>
+      </c>
+      <c r="N11" s="19" t="str">
+        <f aca="false">IF('Set 1'!P11="","",'Set 1'!P11)</f>
+        <v/>
+      </c>
+      <c r="O11" s="19" t="str">
+        <f aca="false">IF('Set 1'!Q11="","",'Set 1'!Q11)</f>
+        <v/>
+      </c>
+      <c r="P11" s="20" t="n">
+        <f aca="false">'Set 1'!R11</f>
+        <v>749.678589646605</v>
+      </c>
+      <c r="Q11" s="19" t="str">
+        <f aca="false">IF('Set 1'!S11="","",'Set 1'!S11)</f>
+        <v/>
+      </c>
+      <c r="R11" s="20" t="str">
+        <f aca="false">IF('Set 1'!T11="","",'Set 1'!T11)</f>
+        <v/>
+      </c>
+      <c r="S11" s="21" t="str">
+        <f aca="false">IF('Set 1'!V11="","",'Set 1'!V11)</f>
+        <v/>
+      </c>
+      <c r="T11" s="21" t="str">
+        <f aca="false">IF('Set 1'!W11="","",'Set 1'!W11)</f>
+        <v/>
+      </c>
+      <c r="U11" s="22" t="str">
+        <f aca="false">IF('Set 1'!X11="","",'Set 1'!X11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="18" t="n">
+        <f aca="false">'Set 2'!A2</f>
+        <v>1</v>
+      </c>
+      <c r="C12" s="19" t="n">
+        <f aca="false">'Set 2'!C2</f>
+        <v>50.55</v>
+      </c>
+      <c r="D12" s="18" t="n">
+        <f aca="false">'Set 2'!D2</f>
+        <v>80</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <f aca="false">'Set 2'!E2</f>
+        <v>8</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <f aca="false">'Set 2'!F2</f>
+        <v>0.88</v>
+      </c>
+      <c r="G12" s="18" t="n">
+        <f aca="false">'Set 2'!I2</f>
+        <v>252.941476967729</v>
+      </c>
+      <c r="H12" s="18" t="str">
+        <f aca="false">IF('Set 2'!J2="","",'Set 2'!J2)</f>
+        <v/>
+      </c>
+      <c r="I12" s="18" t="str">
+        <f aca="false">IF('Set 2'!K2="","",'Set 2'!K2)</f>
+        <v/>
+      </c>
+      <c r="J12" s="18" t="n">
+        <f aca="false">'Set 2'!L2</f>
+        <v>1272.77675106126</v>
+      </c>
+      <c r="K12" s="18" t="str">
+        <f aca="false">IF('Set 2'!M2="","",'Set 2'!M2)</f>
+        <v/>
+      </c>
+      <c r="L12" s="18" t="str">
+        <f aca="false">IF('Set 2'!N2="","",'Set 2'!N2)</f>
+        <v/>
+      </c>
+      <c r="M12" s="19" t="n">
+        <f aca="false">'Set 2'!O2</f>
+        <v>7.51738999999999</v>
+      </c>
+      <c r="N12" s="19" t="str">
+        <f aca="false">IF('Set 2'!P2="","",'Set 2'!P2)</f>
+        <v/>
+      </c>
+      <c r="O12" s="19" t="str">
+        <f aca="false">IF('Set 2'!Q2="","",'Set 2'!Q2)</f>
+        <v/>
+      </c>
+      <c r="P12" s="20" t="n">
+        <f aca="false">'Set 2'!R2</f>
+        <v>194.037396072618</v>
+      </c>
+      <c r="Q12" s="19" t="str">
+        <f aca="false">IF('Set 2'!S2="","",'Set 2'!S2)</f>
+        <v/>
+      </c>
+      <c r="R12" s="20" t="str">
+        <f aca="false">IF('Set 2'!T2="","",'Set 2'!T2)</f>
+        <v/>
+      </c>
+      <c r="S12" s="21" t="str">
+        <f aca="false">IF('Set 2'!V2="","",'Set 2'!V2)</f>
+        <v/>
+      </c>
+      <c r="T12" s="21" t="str">
+        <f aca="false">IF('Set 2'!W2="","",'Set 2'!W2)</f>
+        <v/>
+      </c>
+      <c r="U12" s="22" t="str">
+        <f aca="false">IF('Set 2'!X2="","",'Set 2'!X2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="18" t="n">
+        <f aca="false">'Set 2'!A3</f>
+        <v>2</v>
+      </c>
+      <c r="C13" s="19" t="n">
+        <f aca="false">'Set 2'!C3</f>
+        <v>50.55</v>
+      </c>
+      <c r="D13" s="18" t="n">
+        <f aca="false">'Set 2'!D3</f>
+        <v>320</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <f aca="false">'Set 2'!E3</f>
+        <v>2</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <f aca="false">'Set 2'!F3</f>
+        <v>0.92</v>
+      </c>
+      <c r="G13" s="18" t="n">
+        <f aca="false">'Set 2'!I3</f>
+        <v>252.932975417789</v>
+      </c>
+      <c r="H13" s="18" t="str">
+        <f aca="false">IF('Set 2'!J3="","",'Set 2'!J3)</f>
+        <v/>
+      </c>
+      <c r="I13" s="18" t="str">
+        <f aca="false">IF('Set 2'!K3="","",'Set 2'!K3)</f>
+        <v/>
+      </c>
+      <c r="J13" s="18" t="n">
+        <f aca="false">'Set 2'!L3</f>
+        <v>1271.95778259744</v>
+      </c>
+      <c r="K13" s="18" t="str">
+        <f aca="false">IF('Set 2'!M3="","",'Set 2'!M3)</f>
+        <v/>
+      </c>
+      <c r="L13" s="18" t="str">
+        <f aca="false">IF('Set 2'!N3="","",'Set 2'!N3)</f>
+        <v/>
+      </c>
+      <c r="M13" s="19" t="n">
+        <f aca="false">'Set 2'!O3</f>
+        <v>7.51647999999999</v>
+      </c>
+      <c r="N13" s="19" t="str">
+        <f aca="false">IF('Set 2'!P3="","",'Set 2'!P3)</f>
+        <v/>
+      </c>
+      <c r="O13" s="19" t="str">
+        <f aca="false">IF('Set 2'!Q3="","",'Set 2'!Q3)</f>
+        <v/>
+      </c>
+      <c r="P13" s="20" t="n">
+        <f aca="false">'Set 2'!R3</f>
+        <v>194.398322200401</v>
+      </c>
+      <c r="Q13" s="19" t="str">
+        <f aca="false">IF('Set 2'!S3="","",'Set 2'!S3)</f>
+        <v/>
+      </c>
+      <c r="R13" s="20" t="str">
+        <f aca="false">IF('Set 2'!T3="","",'Set 2'!T3)</f>
+        <v/>
+      </c>
+      <c r="S13" s="21" t="str">
+        <f aca="false">IF('Set 2'!V3="","",'Set 2'!V3)</f>
+        <v/>
+      </c>
+      <c r="T13" s="21" t="str">
+        <f aca="false">IF('Set 2'!W3="","",'Set 2'!W3)</f>
+        <v/>
+      </c>
+      <c r="U13" s="22" t="str">
+        <f aca="false">IF('Set 2'!X3="","",'Set 2'!X3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="18" t="n">
+        <f aca="false">'Set 2'!A4</f>
+        <v>3</v>
+      </c>
+      <c r="C14" s="19" t="n">
+        <f aca="false">'Set 2'!C4</f>
+        <v>50.55</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <f aca="false">'Set 2'!D4</f>
+        <v>240</v>
+      </c>
+      <c r="E14" s="19" t="n">
+        <f aca="false">'Set 2'!E4</f>
+        <v>2.66666666666667</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <f aca="false">'Set 2'!F4</f>
+        <v>0.8</v>
+      </c>
+      <c r="G14" s="18" t="n">
+        <f aca="false">'Set 2'!I4</f>
+        <v>252.941476967729</v>
+      </c>
+      <c r="H14" s="18" t="str">
+        <f aca="false">IF('Set 2'!J4="","",'Set 2'!J4)</f>
+        <v/>
+      </c>
+      <c r="I14" s="18" t="str">
+        <f aca="false">IF('Set 2'!K4="","",'Set 2'!K4)</f>
+        <v/>
+      </c>
+      <c r="J14" s="18" t="n">
+        <f aca="false">'Set 2'!L4</f>
+        <v>1274.36021618533</v>
+      </c>
+      <c r="K14" s="18" t="str">
+        <f aca="false">IF('Set 2'!M4="","",'Set 2'!M4)</f>
+        <v/>
+      </c>
+      <c r="L14" s="18" t="str">
+        <f aca="false">IF('Set 2'!N4="","",'Set 2'!N4)</f>
+        <v/>
+      </c>
+      <c r="M14" s="19" t="n">
+        <f aca="false">'Set 2'!O4</f>
+        <v>7.51820299999999</v>
+      </c>
+      <c r="N14" s="19" t="str">
+        <f aca="false">IF('Set 2'!P4="","",'Set 2'!P4)</f>
+        <v/>
+      </c>
+      <c r="O14" s="19" t="str">
+        <f aca="false">IF('Set 2'!Q4="","",'Set 2'!Q4)</f>
+        <v/>
+      </c>
+      <c r="P14" s="20" t="n">
+        <f aca="false">'Set 2'!R4</f>
+        <v>195.04844034153</v>
+      </c>
+      <c r="Q14" s="19" t="str">
+        <f aca="false">IF('Set 2'!S4="","",'Set 2'!S4)</f>
+        <v/>
+      </c>
+      <c r="R14" s="20" t="str">
+        <f aca="false">IF('Set 2'!T4="","",'Set 2'!T4)</f>
+        <v/>
+      </c>
+      <c r="S14" s="21" t="str">
+        <f aca="false">IF('Set 2'!V4="","",'Set 2'!V4)</f>
+        <v/>
+      </c>
+      <c r="T14" s="21" t="str">
+        <f aca="false">IF('Set 2'!W4="","",'Set 2'!W4)</f>
+        <v/>
+      </c>
+      <c r="U14" s="22" t="str">
+        <f aca="false">IF('Set 2'!X4="","",'Set 2'!X4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="18" t="n">
+        <f aca="false">'Set 2'!A5</f>
+        <v>4</v>
+      </c>
+      <c r="C15" s="19" t="n">
+        <f aca="false">'Set 2'!C5</f>
+        <v>50.55</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <f aca="false">'Set 2'!D5</f>
+        <v>640</v>
+      </c>
+      <c r="E15" s="19" t="n">
+        <f aca="false">'Set 2'!E5</f>
+        <v>1</v>
+      </c>
+      <c r="F15" s="19" t="n">
+        <f aca="false">'Set 2'!F5</f>
+        <v>1</v>
+      </c>
+      <c r="G15" s="18" t="n">
+        <f aca="false">'Set 2'!I5</f>
+        <v>244.381588889695</v>
+      </c>
+      <c r="H15" s="18" t="str">
+        <f aca="false">IF('Set 2'!J5="","",'Set 2'!J5)</f>
+        <v/>
+      </c>
+      <c r="I15" s="18" t="str">
+        <f aca="false">IF('Set 2'!K5="","",'Set 2'!K5)</f>
+        <v/>
+      </c>
+      <c r="J15" s="18" t="n">
+        <f aca="false">'Set 2'!L5</f>
+        <v>1240.57518622454</v>
+      </c>
+      <c r="K15" s="18" t="str">
+        <f aca="false">IF('Set 2'!M5="","",'Set 2'!M5)</f>
+        <v/>
+      </c>
+      <c r="L15" s="18" t="str">
+        <f aca="false">IF('Set 2'!N5="","",'Set 2'!N5)</f>
+        <v/>
+      </c>
+      <c r="M15" s="19" t="n">
+        <f aca="false">'Set 2'!O5</f>
+        <v>7.54008299999999</v>
+      </c>
+      <c r="N15" s="19" t="str">
+        <f aca="false">IF('Set 2'!P5="","",'Set 2'!P5)</f>
+        <v/>
+      </c>
+      <c r="O15" s="19" t="str">
+        <f aca="false">IF('Set 2'!Q5="","",'Set 2'!Q5)</f>
+        <v/>
+      </c>
+      <c r="P15" s="20" t="n">
+        <f aca="false">'Set 2'!R5</f>
+        <v>265.165023707051</v>
+      </c>
+      <c r="Q15" s="19" t="str">
+        <f aca="false">IF('Set 2'!S5="","",'Set 2'!S5)</f>
+        <v/>
+      </c>
+      <c r="R15" s="20" t="str">
+        <f aca="false">IF('Set 2'!T5="","",'Set 2'!T5)</f>
+        <v/>
+      </c>
+      <c r="S15" s="21" t="str">
+        <f aca="false">IF('Set 2'!V5="","",'Set 2'!V5)</f>
+        <v/>
+      </c>
+      <c r="T15" s="21" t="str">
+        <f aca="false">IF('Set 2'!W5="","",'Set 2'!W5)</f>
+        <v/>
+      </c>
+      <c r="U15" s="22" t="str">
+        <f aca="false">IF('Set 2'!X5="","",'Set 2'!X5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="18" t="n">
+        <f aca="false">'Set 2'!A6</f>
+        <v>5</v>
+      </c>
+      <c r="C16" s="19" t="n">
+        <f aca="false">'Set 2'!C6</f>
+        <v>50.55</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <f aca="false">'Set 2'!D6</f>
+        <v>480</v>
+      </c>
+      <c r="E16" s="19" t="n">
+        <f aca="false">'Set 2'!E6</f>
+        <v>1.33333333333333</v>
+      </c>
+      <c r="F16" s="19" t="n">
+        <f aca="false">'Set 2'!F6</f>
+        <v>0.92</v>
+      </c>
+      <c r="G16" s="18" t="n">
+        <f aca="false">'Set 2'!I6</f>
+        <v>244.510942148903</v>
+      </c>
+      <c r="H16" s="18" t="str">
+        <f aca="false">IF('Set 2'!J6="","",'Set 2'!J6)</f>
+        <v/>
+      </c>
+      <c r="I16" s="18" t="str">
+        <f aca="false">IF('Set 2'!K6="","",'Set 2'!K6)</f>
+        <v/>
+      </c>
+      <c r="J16" s="18" t="n">
+        <f aca="false">'Set 2'!L6</f>
+        <v>1241.43819349573</v>
+      </c>
+      <c r="K16" s="18" t="str">
+        <f aca="false">IF('Set 2'!M6="","",'Set 2'!M6)</f>
+        <v/>
+      </c>
+      <c r="L16" s="18" t="str">
+        <f aca="false">IF('Set 2'!N6="","",'Set 2'!N6)</f>
+        <v/>
+      </c>
+      <c r="M16" s="19" t="n">
+        <f aca="false">'Set 2'!O6</f>
+        <v>7.54310199999999</v>
+      </c>
+      <c r="N16" s="19" t="str">
+        <f aca="false">IF('Set 2'!P6="","",'Set 2'!P6)</f>
+        <v/>
+      </c>
+      <c r="O16" s="19" t="str">
+        <f aca="false">IF('Set 2'!Q6="","",'Set 2'!Q6)</f>
+        <v/>
+      </c>
+      <c r="P16" s="20" t="n">
+        <f aca="false">'Set 2'!R6</f>
+        <v>265.45253270235</v>
+      </c>
+      <c r="Q16" s="19" t="str">
+        <f aca="false">IF('Set 2'!S6="","",'Set 2'!S6)</f>
+        <v/>
+      </c>
+      <c r="R16" s="20" t="str">
+        <f aca="false">IF('Set 2'!T6="","",'Set 2'!T6)</f>
+        <v/>
+      </c>
+      <c r="S16" s="21" t="str">
+        <f aca="false">IF('Set 2'!V6="","",'Set 2'!V6)</f>
+        <v/>
+      </c>
+      <c r="T16" s="21" t="str">
+        <f aca="false">IF('Set 2'!W6="","",'Set 2'!W6)</f>
+        <v/>
+      </c>
+      <c r="U16" s="22" t="str">
+        <f aca="false">IF('Set 2'!X6="","",'Set 2'!X6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="18" t="n">
+        <f aca="false">'Set 2'!A7</f>
+        <v>6</v>
+      </c>
+      <c r="C17" s="19" t="n">
+        <f aca="false">'Set 2'!C7</f>
+        <v>50.55</v>
+      </c>
+      <c r="D17" s="18" t="n">
+        <f aca="false">'Set 2'!D7</f>
+        <v>640</v>
+      </c>
+      <c r="E17" s="19" t="n">
+        <f aca="false">'Set 2'!E7</f>
+        <v>1</v>
+      </c>
+      <c r="F17" s="19" t="n">
+        <f aca="false">'Set 2'!F7</f>
+        <v>0.8</v>
+      </c>
+      <c r="G17" s="18" t="n">
+        <f aca="false">'Set 2'!I7</f>
+        <v>244.518491839956</v>
+      </c>
+      <c r="H17" s="18" t="str">
+        <f aca="false">IF('Set 2'!J7="","",'Set 2'!J7)</f>
+        <v/>
+      </c>
+      <c r="I17" s="18" t="str">
+        <f aca="false">IF('Set 2'!K7="","",'Set 2'!K7)</f>
+        <v/>
+      </c>
+      <c r="J17" s="18" t="n">
+        <f aca="false">'Set 2'!L7</f>
+        <v>1244.01182011071</v>
+      </c>
+      <c r="K17" s="18" t="str">
+        <f aca="false">IF('Set 2'!M7="","",'Set 2'!M7)</f>
+        <v/>
+      </c>
+      <c r="L17" s="18" t="str">
+        <f aca="false">IF('Set 2'!N7="","",'Set 2'!N7)</f>
+        <v/>
+      </c>
+      <c r="M17" s="19" t="n">
+        <f aca="false">'Set 2'!O7</f>
+        <v>7.54482499999999</v>
+      </c>
+      <c r="N17" s="19" t="str">
+        <f aca="false">IF('Set 2'!P7="","",'Set 2'!P7)</f>
+        <v/>
+      </c>
+      <c r="O17" s="19" t="str">
+        <f aca="false">IF('Set 2'!Q7="","",'Set 2'!Q7)</f>
+        <v/>
+      </c>
+      <c r="P17" s="20" t="n">
+        <f aca="false">'Set 2'!R7</f>
+        <v>266.130053765627</v>
+      </c>
+      <c r="Q17" s="19" t="str">
+        <f aca="false">IF('Set 2'!S7="","",'Set 2'!S7)</f>
+        <v/>
+      </c>
+      <c r="R17" s="20" t="str">
+        <f aca="false">IF('Set 2'!T7="","",'Set 2'!T7)</f>
+        <v/>
+      </c>
+      <c r="S17" s="21" t="str">
+        <f aca="false">IF('Set 2'!V7="","",'Set 2'!V7)</f>
+        <v/>
+      </c>
+      <c r="T17" s="21" t="str">
+        <f aca="false">IF('Set 2'!W7="","",'Set 2'!W7)</f>
+        <v/>
+      </c>
+      <c r="U17" s="22" t="str">
+        <f aca="false">IF('Set 2'!X7="","",'Set 2'!X7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" s="18" t="n">
+        <f aca="false">'Set 2'!A8</f>
+        <v>7</v>
+      </c>
+      <c r="C18" s="19" t="n">
+        <f aca="false">'Set 2'!C8</f>
+        <v>50.55</v>
+      </c>
+      <c r="D18" s="18" t="n">
+        <f aca="false">'Set 2'!D8</f>
+        <v>1280</v>
+      </c>
+      <c r="E18" s="19" t="n">
+        <f aca="false">'Set 2'!E8</f>
+        <v>0.5</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <f aca="false">'Set 2'!F8</f>
+        <v>0.68</v>
+      </c>
+      <c r="G18" s="18" t="n">
+        <f aca="false">'Set 2'!I8</f>
+        <v>312.794696376031</v>
+      </c>
+      <c r="H18" s="18" t="str">
+        <f aca="false">IF('Set 2'!J8="","",'Set 2'!J8)</f>
+        <v/>
+      </c>
+      <c r="I18" s="18" t="str">
+        <f aca="false">IF('Set 2'!K8="","",'Set 2'!K8)</f>
+        <v/>
+      </c>
+      <c r="J18" s="18" t="n">
+        <f aca="false">'Set 2'!L8</f>
+        <v>1161.08798987177</v>
+      </c>
+      <c r="K18" s="18" t="str">
+        <f aca="false">IF('Set 2'!M8="","",'Set 2'!M8)</f>
+        <v/>
+      </c>
+      <c r="L18" s="18" t="str">
+        <f aca="false">IF('Set 2'!N8="","",'Set 2'!N8)</f>
+        <v/>
+      </c>
+      <c r="M18" s="19" t="n">
+        <f aca="false">'Set 2'!O8</f>
+        <v>7.66023</v>
+      </c>
+      <c r="N18" s="19" t="str">
+        <f aca="false">IF('Set 2'!P8="","",'Set 2'!P8)</f>
+        <v/>
+      </c>
+      <c r="O18" s="19" t="str">
+        <f aca="false">IF('Set 2'!Q8="","",'Set 2'!Q8)</f>
+        <v/>
+      </c>
+      <c r="P18" s="20" t="n">
+        <f aca="false">'Set 2'!R8</f>
+        <v>612.727627704531</v>
+      </c>
+      <c r="Q18" s="19" t="str">
+        <f aca="false">IF('Set 2'!S8="","",'Set 2'!S8)</f>
+        <v/>
+      </c>
+      <c r="R18" s="20" t="str">
+        <f aca="false">IF('Set 2'!T8="","",'Set 2'!T8)</f>
+        <v/>
+      </c>
+      <c r="S18" s="21" t="str">
+        <f aca="false">IF('Set 2'!V8="","",'Set 2'!V8)</f>
+        <v/>
+      </c>
+      <c r="T18" s="21" t="str">
+        <f aca="false">IF('Set 2'!W8="","",'Set 2'!W8)</f>
+        <v/>
+      </c>
+      <c r="U18" s="22" t="str">
+        <f aca="false">IF('Set 2'!X8="","",'Set 2'!X8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="18" t="n">
+        <f aca="false">'Set 2'!A9</f>
+        <v>8</v>
+      </c>
+      <c r="C19" s="19" t="n">
+        <f aca="false">'Set 2'!C9</f>
+        <v>50.55</v>
+      </c>
+      <c r="D19" s="18" t="n">
+        <f aca="false">'Set 2'!D9</f>
+        <v>1040</v>
+      </c>
+      <c r="E19" s="19" t="n">
+        <f aca="false">'Set 2'!E9</f>
+        <v>0.615384615384615</v>
+      </c>
+      <c r="F19" s="19" t="n">
+        <f aca="false">'Set 2'!F9</f>
+        <v>0.56</v>
+      </c>
+      <c r="G19" s="18" t="n">
+        <f aca="false">'Set 2'!I9</f>
+        <v>312.794696376031</v>
+      </c>
+      <c r="H19" s="18" t="str">
+        <f aca="false">IF('Set 2'!J9="","",'Set 2'!J9)</f>
+        <v/>
+      </c>
+      <c r="I19" s="18" t="str">
+        <f aca="false">IF('Set 2'!K9="","",'Set 2'!K9)</f>
+        <v/>
+      </c>
+      <c r="J19" s="18" t="n">
+        <f aca="false">'Set 2'!L9</f>
+        <v>1161.74939305885</v>
+      </c>
+      <c r="K19" s="18" t="str">
+        <f aca="false">IF('Set 2'!M9="","",'Set 2'!M9)</f>
+        <v/>
+      </c>
+      <c r="L19" s="18" t="str">
+        <f aca="false">IF('Set 2'!N9="","",'Set 2'!N9)</f>
+        <v/>
+      </c>
+      <c r="M19" s="19" t="n">
+        <f aca="false">'Set 2'!O9</f>
+        <v>7.660533</v>
+      </c>
+      <c r="N19" s="19" t="str">
+        <f aca="false">IF('Set 2'!P9="","",'Set 2'!P9)</f>
+        <v/>
+      </c>
+      <c r="O19" s="19" t="str">
+        <f aca="false">IF('Set 2'!Q9="","",'Set 2'!Q9)</f>
+        <v/>
+      </c>
+      <c r="P19" s="20" t="n">
+        <f aca="false">'Set 2'!R9</f>
+        <v>613.002453735894</v>
+      </c>
+      <c r="Q19" s="19" t="str">
+        <f aca="false">IF('Set 2'!S9="","",'Set 2'!S9)</f>
+        <v/>
+      </c>
+      <c r="R19" s="20" t="str">
+        <f aca="false">IF('Set 2'!T9="","",'Set 2'!T9)</f>
+        <v/>
+      </c>
+      <c r="S19" s="21" t="str">
+        <f aca="false">IF('Set 2'!V9="","",'Set 2'!V9)</f>
+        <v/>
+      </c>
+      <c r="T19" s="21" t="str">
+        <f aca="false">IF('Set 2'!W9="","",'Set 2'!W9)</f>
+        <v/>
+      </c>
+      <c r="U19" s="22" t="str">
+        <f aca="false">IF('Set 2'!X9="","",'Set 2'!X9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="18" t="n">
+        <f aca="false">'Set 2'!A10</f>
+        <v>9</v>
+      </c>
+      <c r="C20" s="19" t="n">
+        <f aca="false">'Set 2'!C10</f>
+        <v>50.55</v>
+      </c>
+      <c r="D20" s="18" t="n">
+        <f aca="false">'Set 2'!D10</f>
+        <v>720</v>
+      </c>
+      <c r="E20" s="19" t="n">
+        <f aca="false">'Set 2'!E10</f>
+        <v>0.888888888888889</v>
+      </c>
+      <c r="F20" s="19" t="n">
+        <f aca="false">'Set 2'!F10</f>
+        <v>0.6</v>
+      </c>
+      <c r="G20" s="18" t="n">
+        <f aca="false">'Set 2'!I10</f>
+        <v>365.193909930287</v>
+      </c>
+      <c r="H20" s="18" t="str">
+        <f aca="false">IF('Set 2'!J10="","",'Set 2'!J10)</f>
+        <v/>
+      </c>
+      <c r="I20" s="18" t="str">
+        <f aca="false">IF('Set 2'!K10="","",'Set 2'!K10)</f>
+        <v/>
+      </c>
+      <c r="J20" s="18" t="n">
+        <f aca="false">'Set 2'!L10</f>
+        <v>1153.32150850965</v>
+      </c>
+      <c r="K20" s="18" t="str">
+        <f aca="false">IF('Set 2'!M10="","",'Set 2'!M10)</f>
+        <v/>
+      </c>
+      <c r="L20" s="18" t="str">
+        <f aca="false">IF('Set 2'!N10="","",'Set 2'!N10)</f>
+        <v/>
+      </c>
+      <c r="M20" s="19" t="n">
+        <f aca="false">'Set 2'!O10</f>
+        <v>7.677769</v>
+      </c>
+      <c r="N20" s="19" t="str">
+        <f aca="false">IF('Set 2'!P10="","",'Set 2'!P10)</f>
+        <v/>
+      </c>
+      <c r="O20" s="19" t="str">
+        <f aca="false">IF('Set 2'!Q10="","",'Set 2'!Q10)</f>
+        <v/>
+      </c>
+      <c r="P20" s="20" t="n">
+        <f aca="false">'Set 2'!R10</f>
+        <v>646.382176644298</v>
+      </c>
+      <c r="Q20" s="19" t="str">
+        <f aca="false">IF('Set 2'!S10="","",'Set 2'!S10)</f>
+        <v/>
+      </c>
+      <c r="R20" s="20" t="str">
+        <f aca="false">IF('Set 2'!T10="","",'Set 2'!T10)</f>
+        <v/>
+      </c>
+      <c r="S20" s="21" t="str">
+        <f aca="false">IF('Set 2'!V10="","",'Set 2'!V10)</f>
+        <v/>
+      </c>
+      <c r="T20" s="21" t="str">
+        <f aca="false">IF('Set 2'!W10="","",'Set 2'!W10)</f>
+        <v/>
+      </c>
+      <c r="U20" s="22" t="str">
+        <f aca="false">IF('Set 2'!X10="","",'Set 2'!X10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="18" t="n">
+        <f aca="false">'Set 2'!A11</f>
+        <v>10</v>
+      </c>
+      <c r="C21" s="19" t="n">
+        <f aca="false">'Set 2'!C11</f>
+        <v>50.55</v>
+      </c>
+      <c r="D21" s="18" t="n">
+        <f aca="false">'Set 2'!D11</f>
+        <v>720</v>
+      </c>
+      <c r="E21" s="19" t="n">
+        <f aca="false">'Set 2'!E11</f>
+        <v>0.888888888888889</v>
+      </c>
+      <c r="F21" s="19" t="n">
+        <f aca="false">'Set 2'!F11</f>
+        <v>0.04</v>
+      </c>
+      <c r="G21" s="18" t="n">
+        <f aca="false">'Set 2'!I11</f>
+        <v>365.193909930287</v>
+      </c>
+      <c r="H21" s="18" t="str">
+        <f aca="false">IF('Set 2'!J11="","",'Set 2'!J11)</f>
+        <v/>
+      </c>
+      <c r="I21" s="18" t="str">
+        <f aca="false">IF('Set 2'!K11="","",'Set 2'!K11)</f>
+        <v/>
+      </c>
+      <c r="J21" s="18" t="n">
+        <f aca="false">'Set 2'!L11</f>
+        <v>1147.99922817314</v>
+      </c>
+      <c r="K21" s="18" t="str">
+        <f aca="false">IF('Set 2'!M11="","",'Set 2'!M11)</f>
+        <v/>
+      </c>
+      <c r="L21" s="18" t="str">
+        <f aca="false">IF('Set 2'!N11="","",'Set 2'!N11)</f>
+        <v/>
+      </c>
+      <c r="M21" s="19" t="n">
+        <f aca="false">'Set 2'!O11</f>
+        <v>7.680507</v>
+      </c>
+      <c r="N21" s="19" t="str">
+        <f aca="false">IF('Set 2'!P11="","",'Set 2'!P11)</f>
+        <v/>
+      </c>
+      <c r="O21" s="19" t="str">
+        <f aca="false">IF('Set 2'!Q11="","",'Set 2'!Q11)</f>
+        <v/>
+      </c>
+      <c r="P21" s="20" t="n">
+        <f aca="false">'Set 2'!R11</f>
+        <v>655.711579058753</v>
+      </c>
+      <c r="Q21" s="19" t="str">
+        <f aca="false">IF('Set 2'!S11="","",'Set 2'!S11)</f>
+        <v/>
+      </c>
+      <c r="R21" s="20" t="str">
+        <f aca="false">IF('Set 2'!T11="","",'Set 2'!T11)</f>
+        <v/>
+      </c>
+      <c r="S21" s="21" t="str">
+        <f aca="false">IF('Set 2'!V11="","",'Set 2'!V11)</f>
+        <v/>
+      </c>
+      <c r="T21" s="21" t="str">
+        <f aca="false">IF('Set 2'!W11="","",'Set 2'!W11)</f>
+        <v/>
+      </c>
+      <c r="U21" s="22" t="str">
+        <f aca="false">IF('Set 2'!X11="","",'Set 2'!X11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="23" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25" s="24"/>
+      <c r="C25" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="D25" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="E25" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="F25" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="G25" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="H25" s="24" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" s="25"/>
+      <c r="C26" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(G$2:G$11)*ISNUMBER(H$2:H$11))</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="27" t="str">
+        <f aca="false">IF(C26&gt;=3,IFERROR(CORREL(G$2:G$11,H$2:H$11),""),"")</f>
+        <v/>
+      </c>
+      <c r="E26" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(G$12:G$21)*ISNUMBER(H$12:H$21))</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="27" t="str">
+        <f aca="false">IF(E26&gt;=3,IFERROR(CORREL(G$12:G$21,H$12:H$21),""),"")</f>
+        <v/>
+      </c>
+      <c r="G26" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(G$2:G$21)*ISNUMBER(H$2:H$21))</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="27" t="str">
+        <f aca="false">IF(G26&gt;=3,IFERROR(CORREL(G$2:G$21,H$2:H$21),""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="25"/>
+      <c r="C27" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(J$2:J$11)*ISNUMBER(K$2:K$11))</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="27" t="str">
+        <f aca="false">IF(C27&gt;=3,IFERROR(CORREL(J$2:J$11,K$2:K$11),""),"")</f>
+        <v/>
+      </c>
+      <c r="E27" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(J$12:J$21)*ISNUMBER(K$12:K$21))</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="27" t="str">
+        <f aca="false">IF(E27&gt;=3,IFERROR(CORREL(J$12:J$21,K$12:K$21),""),"")</f>
+        <v/>
+      </c>
+      <c r="G27" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(J$2:J$21)*ISNUMBER(K$2:K$21))</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="27" t="str">
+        <f aca="false">IF(G27&gt;=3,IFERROR(CORREL(J$2:J$21,K$2:K$21),""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(M$2:M$11)*ISNUMBER(N$2:N$11))</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="27" t="str">
+        <f aca="false">IF(C28&gt;=3,IFERROR(CORREL(M$2:M$11,N$2:N$11),""),"")</f>
+        <v/>
+      </c>
+      <c r="E28" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(M$12:M$21)*ISNUMBER(N$12:N$21))</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="27" t="str">
+        <f aca="false">IF(E28&gt;=3,IFERROR(CORREL(M$12:M$21,N$12:N$21),""),"")</f>
+        <v/>
+      </c>
+      <c r="G28" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(M$2:M$21)*ISNUMBER(N$2:N$21))</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="27" t="str">
+        <f aca="false">IF(G28&gt;=3,IFERROR(CORREL(M$2:M$21,N$2:N$21),""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29" s="25"/>
+      <c r="C29" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(P$2:P$11)*ISNUMBER(Q$2:Q$11))</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="27" t="str">
+        <f aca="false">IF(C29&gt;=3,IFERROR(CORREL(P$2:P$11,Q$2:Q$11),""),"")</f>
+        <v/>
+      </c>
+      <c r="E29" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(P$12:P$21)*ISNUMBER(Q$12:Q$21))</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="27" t="str">
+        <f aca="false">IF(E29&gt;=3,IFERROR(CORREL(P$12:P$21,Q$12:Q$21),""),"")</f>
+        <v/>
+      </c>
+      <c r="G29" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(P$2:P$21)*ISNUMBER(Q$2:Q$21))</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="27" t="str">
+        <f aca="false">IF(G29&gt;=3,IFERROR(CORREL(P$2:P$21,Q$2:Q$21),""),"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FF2E75B6"/>
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="28" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="29" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
     <tabColor rgb="FF7F7F7F"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -3529,260 +7663,284 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>25</v>
+      <c r="A1" s="30" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
-        <v>26</v>
+      <c r="A2" s="31" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
-        <v>27</v>
+      <c r="A3" s="32" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="21" t="n">
+      <c r="A4" s="33" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="34" t="n">
         <v>640</v>
       </c>
-      <c r="C4" s="20" t="s">
-        <v>29</v>
+      <c r="C4" s="33" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="B5" s="21" t="n">
+      <c r="A5" s="33" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="34" t="n">
         <v>640</v>
       </c>
-      <c r="C5" s="20" t="s">
-        <v>31</v>
+      <c r="C5" s="33" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
-        <v>32</v>
+      <c r="A7" s="32" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>34</v>
+      <c r="A8" s="35" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="33" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>36</v>
+      <c r="A9" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="33" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="24" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>38</v>
+      <c r="A10" s="37" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="33" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>40</v>
+      <c r="A11" s="33" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" s="33" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
-        <v>41</v>
+      <c r="A13" s="32" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="25" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>43</v>
+      <c r="A14" s="38" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" s="33" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="C15" s="20" t="s">
-        <v>45</v>
+      <c r="A15" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="33" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="25" t="s">
-        <v>46</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>47</v>
+      <c r="A16" s="38" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" s="33" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="25" t="s">
-        <v>48</v>
-      </c>
-      <c r="C17" s="20" t="s">
-        <v>49</v>
+      <c r="A17" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" s="33" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="25" t="s">
-        <v>50</v>
-      </c>
-      <c r="C18" s="20" t="s">
-        <v>51</v>
+      <c r="A18" s="38" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" s="33" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>53</v>
+      <c r="A19" s="38" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="33" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="25" t="s">
+      <c r="A20" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="20" t="s">
-        <v>54</v>
+      <c r="C20" s="33" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="25" t="s">
+      <c r="A21" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="20" t="s">
-        <v>55</v>
+      <c r="C21" s="33" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="25" t="s">
+      <c r="A22" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="C22" s="20" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="25" t="s">
+      <c r="C22" s="33" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="38" t="s">
+        <v>75</v>
+      </c>
+      <c r="C23" s="33" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="38" t="s">
+        <v>77</v>
+      </c>
+      <c r="C24" s="33" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="C23" s="20" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="C26" s="20" t="s">
-        <v>60</v>
+      <c r="C25" s="33" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="20" t="s">
+      <c r="A27" s="32" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="C28" s="33" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="B27" s="26" t="n">
+      <c r="B29" s="39" t="n">
         <v>572</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="26" t="n">
+      <c r="B30" s="39" t="n">
         <v>796</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B29" s="27" t="n">
+      <c r="B31" s="40" t="n">
         <v>4.95</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="B30" s="27" t="n">
+      <c r="B32" s="40" t="n">
         <v>5.57</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="B31" s="28" t="n">
+      <c r="B33" s="41" t="n">
         <v>0.931</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="B32" s="28" t="n">
+      <c r="B34" s="41" t="n">
         <v>0.618</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="20" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="B33" s="29" t="n">
+      <c r="B35" s="42" t="n">
         <v>0.000178</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="19" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="C36" s="20" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="C37" s="20" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="C38" s="20" t="s">
-        <v>65</v>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="32" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="C38" s="33" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="C39" s="33" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="C40" s="33" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="C41" s="33" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Harden Combined links and tidy notes after second audit
Combined now passes only numeric SIM values through, so a typed =NA() or text
cannot blank the correlation table. Notes: fix the 'every cell is a link' claim,
add the green-text legend and a leave-SIM-cells-empty warning. Comment boxes
wrap text.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011WnE18kmcTTQHQwwBdKitt
</commit_message>
<xml_diff>
--- a/CM_Sweep_Sets_1_2.xlsx
+++ b/CM_Sweep_Sets_1_2.xlsx
@@ -380,7 +380,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="91">
   <si>
     <t xml:space="preserve">Point</t>
   </si>
@@ -550,7 +550,13 @@
     <t xml:space="preserve">Blue text, yellow fill</t>
   </si>
   <si>
-    <t xml:space="preserve">Cell to fill in: the SIM columns. Everything that depends on them (Δ columns, loop ratio, loop rank Δ) fills itself in.</t>
+    <t xml:space="preserve">Cell to fill in: the SIM columns. Everything that depends on them (Δ columns, loop ratio, loop rank Δ, Combined, Charts) fills itself in. Leave a cell empty if there is no value: text such as n/a can plot as 0 in Excel charts, and Combined only passes numbers through.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Green text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Link to another sheet (the Combined tab). Do not overwrite.</t>
   </si>
   <si>
     <t xml:space="preserve">Do not sort or filter</t>
@@ -610,7 +616,7 @@
     <t xml:space="preserve">Combined sheet</t>
   </si>
   <si>
-    <t xml:space="preserve">Sets 1 and 2 stacked into 20 rows. Every cell is a link to the Set sheets (green text), so nothing is typed here. SIM-dependent cells stay blank until the SIM values exist. Below the table, Pearson r between each ML metric and its SIM value, per set and for all 20 points; it needs at least 3 points with a SIM value. With so few points r is only indicative.</t>
+    <t xml:space="preserve">Sets 1 and 2 stacked into 20 rows. Columns B–U of the 20-row table are links to the Set sheets (green text); only the Set label in column A is typed. SIM-dependent cells stay blank until a numeric SIM value exists (text or error values are ignored). The Pearson block is calculated. Below the table, Pearson r between each ML metric and its SIM value, per set and for all 20 points; it needs at least 3 points with a SIM value. With so few points r is only indicative.</t>
   </si>
   <si>
     <t xml:space="preserve">Charts sheet</t>
@@ -837,7 +843,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -990,6 +996,10 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1338,11 +1348,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="49179135"/>
-        <c:axId val="92601320"/>
+        <c:axId val="78884795"/>
+        <c:axId val="7905892"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="49179135"/>
+        <c:axId val="78884795"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1418,12 +1428,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92601320"/>
+        <c:crossAx val="7905892"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="92601320"/>
+        <c:axId val="7905892"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1499,7 +1509,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49179135"/>
+        <c:crossAx val="78884795"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1807,11 +1817,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="67022920"/>
-        <c:axId val="86970286"/>
+        <c:axId val="37380373"/>
+        <c:axId val="47674793"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="67022920"/>
+        <c:axId val="37380373"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1887,12 +1897,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86970286"/>
+        <c:crossAx val="47674793"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="86970286"/>
+        <c:axId val="47674793"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1968,7 +1978,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67022920"/>
+        <c:crossAx val="37380373"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2276,11 +2286,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="31666765"/>
-        <c:axId val="42321796"/>
+        <c:axId val="51108273"/>
+        <c:axId val="66932665"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="31666765"/>
+        <c:axId val="51108273"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2356,12 +2366,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42321796"/>
+        <c:crossAx val="66932665"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="42321796"/>
+        <c:axId val="66932665"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2437,7 +2447,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31666765"/>
+        <c:crossAx val="51108273"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2745,11 +2755,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="13051780"/>
-        <c:axId val="47218477"/>
+        <c:axId val="52103404"/>
+        <c:axId val="47569270"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="13051780"/>
+        <c:axId val="52103404"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2825,12 +2835,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47218477"/>
+        <c:crossAx val="47569270"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="47218477"/>
+        <c:axId val="47569270"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2906,7 +2916,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13051780"/>
+        <c:crossAx val="52103404"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5779,11 +5789,11 @@
         <v>1421.15811288509</v>
       </c>
       <c r="H2" s="18" t="str">
-        <f aca="false">IF('Set 1'!J2="","",'Set 1'!J2)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!J2),'Set 1'!J2,"")</f>
         <v/>
       </c>
       <c r="I2" s="18" t="str">
-        <f aca="false">IF('Set 1'!K2="","",'Set 1'!K2)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!K2),'Set 1'!K2,"")</f>
         <v/>
       </c>
       <c r="J2" s="18" t="n">
@@ -5791,11 +5801,11 @@
         <v>1746.44105539347</v>
       </c>
       <c r="K2" s="18" t="str">
-        <f aca="false">IF('Set 1'!M2="","",'Set 1'!M2)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!M2),'Set 1'!M2,"")</f>
         <v/>
       </c>
       <c r="L2" s="18" t="str">
-        <f aca="false">IF('Set 1'!N2="","",'Set 1'!N2)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!N2),'Set 1'!N2,"")</f>
         <v/>
       </c>
       <c r="M2" s="19" t="n">
@@ -5803,11 +5813,11 @@
         <v>7.550116</v>
       </c>
       <c r="N2" s="19" t="str">
-        <f aca="false">IF('Set 1'!P2="","",'Set 1'!P2)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!P2),'Set 1'!P2,"")</f>
         <v/>
       </c>
       <c r="O2" s="19" t="str">
-        <f aca="false">IF('Set 1'!Q2="","",'Set 1'!Q2)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!Q2),'Set 1'!Q2,"")</f>
         <v/>
       </c>
       <c r="P2" s="20" t="n">
@@ -5815,23 +5825,23 @@
         <v>263.959090135506</v>
       </c>
       <c r="Q2" s="19" t="str">
-        <f aca="false">IF('Set 1'!S2="","",'Set 1'!S2)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!S2),'Set 1'!S2,"")</f>
         <v/>
       </c>
       <c r="R2" s="20" t="str">
-        <f aca="false">IF('Set 1'!T2="","",'Set 1'!T2)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!T2),'Set 1'!T2,"")</f>
         <v/>
       </c>
       <c r="S2" s="21" t="str">
-        <f aca="false">IF('Set 1'!V2="","",'Set 1'!V2)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!V2),'Set 1'!V2,"")</f>
         <v/>
       </c>
       <c r="T2" s="21" t="str">
-        <f aca="false">IF('Set 1'!W2="","",'Set 1'!W2)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!W2),'Set 1'!W2,"")</f>
         <v/>
       </c>
       <c r="U2" s="22" t="str">
-        <f aca="false">IF('Set 1'!X2="","",'Set 1'!X2)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!X2),'Set 1'!X2,"")</f>
         <v/>
       </c>
     </row>
@@ -5864,11 +5874,11 @@
         <v>1380.32366821806</v>
       </c>
       <c r="H3" s="18" t="str">
-        <f aca="false">IF('Set 1'!J3="","",'Set 1'!J3)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!J3),'Set 1'!J3,"")</f>
         <v/>
       </c>
       <c r="I3" s="18" t="str">
-        <f aca="false">IF('Set 1'!K3="","",'Set 1'!K3)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!K3),'Set 1'!K3,"")</f>
         <v/>
       </c>
       <c r="J3" s="18" t="n">
@@ -5876,11 +5886,11 @@
         <v>1744.46534440925</v>
       </c>
       <c r="K3" s="18" t="str">
-        <f aca="false">IF('Set 1'!M3="","",'Set 1'!M3)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!M3),'Set 1'!M3,"")</f>
         <v/>
       </c>
       <c r="L3" s="18" t="str">
-        <f aca="false">IF('Set 1'!N3="","",'Set 1'!N3)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!N3),'Set 1'!N3,"")</f>
         <v/>
       </c>
       <c r="M3" s="19" t="n">
@@ -5888,11 +5898,11 @@
         <v>7.61353533333333</v>
       </c>
       <c r="N3" s="19" t="str">
-        <f aca="false">IF('Set 1'!P3="","",'Set 1'!P3)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!P3),'Set 1'!P3,"")</f>
         <v/>
       </c>
       <c r="O3" s="19" t="str">
-        <f aca="false">IF('Set 1'!Q3="","",'Set 1'!Q3)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!Q3),'Set 1'!Q3,"")</f>
         <v/>
       </c>
       <c r="P3" s="20" t="n">
@@ -5900,23 +5910,23 @@
         <v>543.22722833229</v>
       </c>
       <c r="Q3" s="19" t="str">
-        <f aca="false">IF('Set 1'!S3="","",'Set 1'!S3)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!S3),'Set 1'!S3,"")</f>
         <v/>
       </c>
       <c r="R3" s="20" t="str">
-        <f aca="false">IF('Set 1'!T3="","",'Set 1'!T3)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!T3),'Set 1'!T3,"")</f>
         <v/>
       </c>
       <c r="S3" s="21" t="str">
-        <f aca="false">IF('Set 1'!V3="","",'Set 1'!V3)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!V3),'Set 1'!V3,"")</f>
         <v/>
       </c>
       <c r="T3" s="21" t="str">
-        <f aca="false">IF('Set 1'!W3="","",'Set 1'!W3)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!W3),'Set 1'!W3,"")</f>
         <v/>
       </c>
       <c r="U3" s="22" t="str">
-        <f aca="false">IF('Set 1'!X3="","",'Set 1'!X3)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!X3),'Set 1'!X3,"")</f>
         <v/>
       </c>
     </row>
@@ -5949,11 +5959,11 @@
         <v>1408.29891867377</v>
       </c>
       <c r="H4" s="18" t="str">
-        <f aca="false">IF('Set 1'!J4="","",'Set 1'!J4)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!J4),'Set 1'!J4,"")</f>
         <v/>
       </c>
       <c r="I4" s="18" t="str">
-        <f aca="false">IF('Set 1'!K4="","",'Set 1'!K4)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!K4),'Set 1'!K4,"")</f>
         <v/>
       </c>
       <c r="J4" s="18" t="n">
@@ -5961,11 +5971,11 @@
         <v>1745.71301367738</v>
       </c>
       <c r="K4" s="18" t="str">
-        <f aca="false">IF('Set 1'!M4="","",'Set 1'!M4)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!M4),'Set 1'!M4,"")</f>
         <v/>
       </c>
       <c r="L4" s="18" t="str">
-        <f aca="false">IF('Set 1'!N4="","",'Set 1'!N4)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!N4),'Set 1'!N4,"")</f>
         <v/>
       </c>
       <c r="M4" s="19" t="n">
@@ -5973,11 +5983,11 @@
         <v>7.63308399999999</v>
       </c>
       <c r="N4" s="19" t="str">
-        <f aca="false">IF('Set 1'!P4="","",'Set 1'!P4)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!P4),'Set 1'!P4,"")</f>
         <v/>
       </c>
       <c r="O4" s="19" t="str">
-        <f aca="false">IF('Set 1'!Q4="","",'Set 1'!Q4)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!Q4),'Set 1'!Q4,"")</f>
         <v/>
       </c>
       <c r="P4" s="20" t="n">
@@ -5985,23 +5995,23 @@
         <v>632.07201334017</v>
       </c>
       <c r="Q4" s="19" t="str">
-        <f aca="false">IF('Set 1'!S4="","",'Set 1'!S4)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!S4),'Set 1'!S4,"")</f>
         <v/>
       </c>
       <c r="R4" s="20" t="str">
-        <f aca="false">IF('Set 1'!T4="","",'Set 1'!T4)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!T4),'Set 1'!T4,"")</f>
         <v/>
       </c>
       <c r="S4" s="21" t="str">
-        <f aca="false">IF('Set 1'!V4="","",'Set 1'!V4)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!V4),'Set 1'!V4,"")</f>
         <v/>
       </c>
       <c r="T4" s="21" t="str">
-        <f aca="false">IF('Set 1'!W4="","",'Set 1'!W4)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!W4),'Set 1'!W4,"")</f>
         <v/>
       </c>
       <c r="U4" s="22" t="str">
-        <f aca="false">IF('Set 1'!X4="","",'Set 1'!X4)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!X4),'Set 1'!X4,"")</f>
         <v/>
       </c>
     </row>
@@ -6034,11 +6044,11 @@
         <v>1409.06706888271</v>
       </c>
       <c r="H5" s="18" t="str">
-        <f aca="false">IF('Set 1'!J5="","",'Set 1'!J5)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!J5),'Set 1'!J5,"")</f>
         <v/>
       </c>
       <c r="I5" s="18" t="str">
-        <f aca="false">IF('Set 1'!K5="","",'Set 1'!K5)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!K5),'Set 1'!K5,"")</f>
         <v/>
       </c>
       <c r="J5" s="18" t="n">
@@ -6046,11 +6056,11 @@
         <v>1746.41676186042</v>
       </c>
       <c r="K5" s="18" t="str">
-        <f aca="false">IF('Set 1'!M5="","",'Set 1'!M5)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!M5),'Set 1'!M5,"")</f>
         <v/>
       </c>
       <c r="L5" s="18" t="str">
-        <f aca="false">IF('Set 1'!N5="","",'Set 1'!N5)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!N5),'Set 1'!N5,"")</f>
         <v/>
       </c>
       <c r="M5" s="19" t="n">
@@ -6058,11 +6068,11 @@
         <v>7.62935699999999</v>
       </c>
       <c r="N5" s="19" t="str">
-        <f aca="false">IF('Set 1'!P5="","",'Set 1'!P5)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!P5),'Set 1'!P5,"")</f>
         <v/>
       </c>
       <c r="O5" s="19" t="str">
-        <f aca="false">IF('Set 1'!Q5="","",'Set 1'!Q5)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!Q5),'Set 1'!Q5,"")</f>
         <v/>
       </c>
       <c r="P5" s="20" t="n">
@@ -6070,23 +6080,23 @@
         <v>650.201104432882</v>
       </c>
       <c r="Q5" s="19" t="str">
-        <f aca="false">IF('Set 1'!S5="","",'Set 1'!S5)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!S5),'Set 1'!S5,"")</f>
         <v/>
       </c>
       <c r="R5" s="20" t="str">
-        <f aca="false">IF('Set 1'!T5="","",'Set 1'!T5)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!T5),'Set 1'!T5,"")</f>
         <v/>
       </c>
       <c r="S5" s="21" t="str">
-        <f aca="false">IF('Set 1'!V5="","",'Set 1'!V5)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!V5),'Set 1'!V5,"")</f>
         <v/>
       </c>
       <c r="T5" s="21" t="str">
-        <f aca="false">IF('Set 1'!W5="","",'Set 1'!W5)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!W5),'Set 1'!W5,"")</f>
         <v/>
       </c>
       <c r="U5" s="22" t="str">
-        <f aca="false">IF('Set 1'!X5="","",'Set 1'!X5)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!X5),'Set 1'!X5,"")</f>
         <v/>
       </c>
     </row>
@@ -6119,11 +6129,11 @@
         <v>1407.499351274</v>
       </c>
       <c r="H6" s="18" t="str">
-        <f aca="false">IF('Set 1'!J6="","",'Set 1'!J6)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!J6),'Set 1'!J6,"")</f>
         <v/>
       </c>
       <c r="I6" s="18" t="str">
-        <f aca="false">IF('Set 1'!K6="","",'Set 1'!K6)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!K6),'Set 1'!K6,"")</f>
         <v/>
       </c>
       <c r="J6" s="18" t="n">
@@ -6131,11 +6141,11 @@
         <v>1746.37860154084</v>
       </c>
       <c r="K6" s="18" t="str">
-        <f aca="false">IF('Set 1'!M6="","",'Set 1'!M6)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!M6),'Set 1'!M6,"")</f>
         <v/>
       </c>
       <c r="L6" s="18" t="str">
-        <f aca="false">IF('Set 1'!N6="","",'Set 1'!N6)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!N6),'Set 1'!N6,"")</f>
         <v/>
       </c>
       <c r="M6" s="19" t="n">
@@ -6143,11 +6153,11 @@
         <v>7.63384199999999</v>
       </c>
       <c r="N6" s="19" t="str">
-        <f aca="false">IF('Set 1'!P6="","",'Set 1'!P6)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!P6),'Set 1'!P6,"")</f>
         <v/>
       </c>
       <c r="O6" s="19" t="str">
-        <f aca="false">IF('Set 1'!Q6="","",'Set 1'!Q6)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!Q6),'Set 1'!Q6,"")</f>
         <v/>
       </c>
       <c r="P6" s="20" t="n">
@@ -6155,23 +6165,23 @@
         <v>656.430712583907</v>
       </c>
       <c r="Q6" s="19" t="str">
-        <f aca="false">IF('Set 1'!S6="","",'Set 1'!S6)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!S6),'Set 1'!S6,"")</f>
         <v/>
       </c>
       <c r="R6" s="20" t="str">
-        <f aca="false">IF('Set 1'!T6="","",'Set 1'!T6)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!T6),'Set 1'!T6,"")</f>
         <v/>
       </c>
       <c r="S6" s="21" t="str">
-        <f aca="false">IF('Set 1'!V6="","",'Set 1'!V6)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!V6),'Set 1'!V6,"")</f>
         <v/>
       </c>
       <c r="T6" s="21" t="str">
-        <f aca="false">IF('Set 1'!W6="","",'Set 1'!W6)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!W6),'Set 1'!W6,"")</f>
         <v/>
       </c>
       <c r="U6" s="22" t="str">
-        <f aca="false">IF('Set 1'!X6="","",'Set 1'!X6)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!X6),'Set 1'!X6,"")</f>
         <v/>
       </c>
     </row>
@@ -6204,11 +6214,11 @@
         <v>1407.29955396803</v>
       </c>
       <c r="H7" s="18" t="str">
-        <f aca="false">IF('Set 1'!J7="","",'Set 1'!J7)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!J7),'Set 1'!J7,"")</f>
         <v/>
       </c>
       <c r="I7" s="18" t="str">
-        <f aca="false">IF('Set 1'!K7="","",'Set 1'!K7)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!K7),'Set 1'!K7,"")</f>
         <v/>
       </c>
       <c r="J7" s="18" t="n">
@@ -6216,11 +6226,11 @@
         <v>1745.65194202208</v>
       </c>
       <c r="K7" s="18" t="str">
-        <f aca="false">IF('Set 1'!M7="","",'Set 1'!M7)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!M7),'Set 1'!M7,"")</f>
         <v/>
       </c>
       <c r="L7" s="18" t="str">
-        <f aca="false">IF('Set 1'!N7="","",'Set 1'!N7)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!N7),'Set 1'!N7,"")</f>
         <v/>
       </c>
       <c r="M7" s="19" t="n">
@@ -6228,11 +6238,11 @@
         <v>7.64592499999999</v>
       </c>
       <c r="N7" s="19" t="str">
-        <f aca="false">IF('Set 1'!P7="","",'Set 1'!P7)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!P7),'Set 1'!P7,"")</f>
         <v/>
       </c>
       <c r="O7" s="19" t="str">
-        <f aca="false">IF('Set 1'!Q7="","",'Set 1'!Q7)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!Q7),'Set 1'!Q7,"")</f>
         <v/>
       </c>
       <c r="P7" s="20" t="n">
@@ -6240,23 +6250,23 @@
         <v>661.922490247295</v>
       </c>
       <c r="Q7" s="19" t="str">
-        <f aca="false">IF('Set 1'!S7="","",'Set 1'!S7)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!S7),'Set 1'!S7,"")</f>
         <v/>
       </c>
       <c r="R7" s="20" t="str">
-        <f aca="false">IF('Set 1'!T7="","",'Set 1'!T7)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!T7),'Set 1'!T7,"")</f>
         <v/>
       </c>
       <c r="S7" s="21" t="str">
-        <f aca="false">IF('Set 1'!V7="","",'Set 1'!V7)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!V7),'Set 1'!V7,"")</f>
         <v/>
       </c>
       <c r="T7" s="21" t="str">
-        <f aca="false">IF('Set 1'!W7="","",'Set 1'!W7)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!W7),'Set 1'!W7,"")</f>
         <v/>
       </c>
       <c r="U7" s="22" t="str">
-        <f aca="false">IF('Set 1'!X7="","",'Set 1'!X7)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!X7),'Set 1'!X7,"")</f>
         <v/>
       </c>
     </row>
@@ -6289,11 +6299,11 @@
         <v>1409.21728292278</v>
       </c>
       <c r="H8" s="18" t="str">
-        <f aca="false">IF('Set 1'!J8="","",'Set 1'!J8)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!J8),'Set 1'!J8,"")</f>
         <v/>
       </c>
       <c r="I8" s="18" t="str">
-        <f aca="false">IF('Set 1'!K8="","",'Set 1'!K8)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!K8),'Set 1'!K8,"")</f>
         <v/>
       </c>
       <c r="J8" s="18" t="n">
@@ -6301,11 +6311,11 @@
         <v>1746.53707486242</v>
       </c>
       <c r="K8" s="18" t="str">
-        <f aca="false">IF('Set 1'!M8="","",'Set 1'!M8)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!M8),'Set 1'!M8,"")</f>
         <v/>
       </c>
       <c r="L8" s="18" t="str">
-        <f aca="false">IF('Set 1'!N8="","",'Set 1'!N8)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!N8),'Set 1'!N8,"")</f>
         <v/>
       </c>
       <c r="M8" s="19" t="n">
@@ -6313,11 +6323,11 @@
         <v>7.64266299999999</v>
       </c>
       <c r="N8" s="19" t="str">
-        <f aca="false">IF('Set 1'!P8="","",'Set 1'!P8)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!P8),'Set 1'!P8,"")</f>
         <v/>
       </c>
       <c r="O8" s="19" t="str">
-        <f aca="false">IF('Set 1'!Q8="","",'Set 1'!Q8)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!Q8),'Set 1'!Q8,"")</f>
         <v/>
       </c>
       <c r="P8" s="20" t="n">
@@ -6325,23 +6335,23 @@
         <v>722.735643650416</v>
       </c>
       <c r="Q8" s="19" t="str">
-        <f aca="false">IF('Set 1'!S8="","",'Set 1'!S8)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!S8),'Set 1'!S8,"")</f>
         <v/>
       </c>
       <c r="R8" s="20" t="str">
-        <f aca="false">IF('Set 1'!T8="","",'Set 1'!T8)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!T8),'Set 1'!T8,"")</f>
         <v/>
       </c>
       <c r="S8" s="21" t="str">
-        <f aca="false">IF('Set 1'!V8="","",'Set 1'!V8)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!V8),'Set 1'!V8,"")</f>
         <v/>
       </c>
       <c r="T8" s="21" t="str">
-        <f aca="false">IF('Set 1'!W8="","",'Set 1'!W8)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!W8),'Set 1'!W8,"")</f>
         <v/>
       </c>
       <c r="U8" s="22" t="str">
-        <f aca="false">IF('Set 1'!X8="","",'Set 1'!X8)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!X8),'Set 1'!X8,"")</f>
         <v/>
       </c>
     </row>
@@ -6374,11 +6384,11 @@
         <v>1402.53857129639</v>
       </c>
       <c r="H9" s="18" t="str">
-        <f aca="false">IF('Set 1'!J9="","",'Set 1'!J9)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!J9),'Set 1'!J9,"")</f>
         <v/>
       </c>
       <c r="I9" s="18" t="str">
-        <f aca="false">IF('Set 1'!K9="","",'Set 1'!K9)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!K9),'Set 1'!K9,"")</f>
         <v/>
       </c>
       <c r="J9" s="18" t="n">
@@ -6386,11 +6396,11 @@
         <v>1746.17439480164</v>
       </c>
       <c r="K9" s="18" t="str">
-        <f aca="false">IF('Set 1'!M9="","",'Set 1'!M9)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!M9),'Set 1'!M9,"")</f>
         <v/>
       </c>
       <c r="L9" s="18" t="str">
-        <f aca="false">IF('Set 1'!N9="","",'Set 1'!N9)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!N9),'Set 1'!N9,"")</f>
         <v/>
       </c>
       <c r="M9" s="19" t="n">
@@ -6398,11 +6408,11 @@
         <v>7.64895899999999</v>
       </c>
       <c r="N9" s="19" t="str">
-        <f aca="false">IF('Set 1'!P9="","",'Set 1'!P9)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!P9),'Set 1'!P9,"")</f>
         <v/>
       </c>
       <c r="O9" s="19" t="str">
-        <f aca="false">IF('Set 1'!Q9="","",'Set 1'!Q9)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!Q9),'Set 1'!Q9,"")</f>
         <v/>
       </c>
       <c r="P9" s="20" t="n">
@@ -6410,23 +6420,23 @@
         <v>731.734711525745</v>
       </c>
       <c r="Q9" s="19" t="str">
-        <f aca="false">IF('Set 1'!S9="","",'Set 1'!S9)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!S9),'Set 1'!S9,"")</f>
         <v/>
       </c>
       <c r="R9" s="20" t="str">
-        <f aca="false">IF('Set 1'!T9="","",'Set 1'!T9)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!T9),'Set 1'!T9,"")</f>
         <v/>
       </c>
       <c r="S9" s="21" t="str">
-        <f aca="false">IF('Set 1'!V9="","",'Set 1'!V9)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!V9),'Set 1'!V9,"")</f>
         <v/>
       </c>
       <c r="T9" s="21" t="str">
-        <f aca="false">IF('Set 1'!W9="","",'Set 1'!W9)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!W9),'Set 1'!W9,"")</f>
         <v/>
       </c>
       <c r="U9" s="22" t="str">
-        <f aca="false">IF('Set 1'!X9="","",'Set 1'!X9)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!X9),'Set 1'!X9,"")</f>
         <v/>
       </c>
     </row>
@@ -6459,11 +6469,11 @@
         <v>1403.69923690996</v>
       </c>
       <c r="H10" s="18" t="str">
-        <f aca="false">IF('Set 1'!J10="","",'Set 1'!J10)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!J10),'Set 1'!J10,"")</f>
         <v/>
       </c>
       <c r="I10" s="18" t="str">
-        <f aca="false">IF('Set 1'!K10="","",'Set 1'!K10)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!K10),'Set 1'!K10,"")</f>
         <v/>
       </c>
       <c r="J10" s="18" t="n">
@@ -6471,11 +6481,11 @@
         <v>1749.6312767733</v>
       </c>
       <c r="K10" s="18" t="str">
-        <f aca="false">IF('Set 1'!M10="","",'Set 1'!M10)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!M10),'Set 1'!M10,"")</f>
         <v/>
       </c>
       <c r="L10" s="18" t="str">
-        <f aca="false">IF('Set 1'!N10="","",'Set 1'!N10)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!N10),'Set 1'!N10,"")</f>
         <v/>
       </c>
       <c r="M10" s="19" t="n">
@@ -6483,11 +6493,11 @@
         <v>7.64311299999999</v>
       </c>
       <c r="N10" s="19" t="str">
-        <f aca="false">IF('Set 1'!P10="","",'Set 1'!P10)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!P10),'Set 1'!P10,"")</f>
         <v/>
       </c>
       <c r="O10" s="19" t="str">
-        <f aca="false">IF('Set 1'!Q10="","",'Set 1'!Q10)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!Q10),'Set 1'!Q10,"")</f>
         <v/>
       </c>
       <c r="P10" s="20" t="n">
@@ -6495,23 +6505,23 @@
         <v>741.859239328738</v>
       </c>
       <c r="Q10" s="19" t="str">
-        <f aca="false">IF('Set 1'!S10="","",'Set 1'!S10)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!S10),'Set 1'!S10,"")</f>
         <v/>
       </c>
       <c r="R10" s="20" t="str">
-        <f aca="false">IF('Set 1'!T10="","",'Set 1'!T10)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!T10),'Set 1'!T10,"")</f>
         <v/>
       </c>
       <c r="S10" s="21" t="str">
-        <f aca="false">IF('Set 1'!V10="","",'Set 1'!V10)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!V10),'Set 1'!V10,"")</f>
         <v/>
       </c>
       <c r="T10" s="21" t="str">
-        <f aca="false">IF('Set 1'!W10="","",'Set 1'!W10)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!W10),'Set 1'!W10,"")</f>
         <v/>
       </c>
       <c r="U10" s="22" t="str">
-        <f aca="false">IF('Set 1'!X10="","",'Set 1'!X10)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!X10),'Set 1'!X10,"")</f>
         <v/>
       </c>
     </row>
@@ -6544,11 +6554,11 @@
         <v>1404.60593589585</v>
       </c>
       <c r="H11" s="18" t="str">
-        <f aca="false">IF('Set 1'!J11="","",'Set 1'!J11)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!J11),'Set 1'!J11,"")</f>
         <v/>
       </c>
       <c r="I11" s="18" t="str">
-        <f aca="false">IF('Set 1'!K11="","",'Set 1'!K11)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!K11),'Set 1'!K11,"")</f>
         <v/>
       </c>
       <c r="J11" s="18" t="n">
@@ -6556,11 +6566,11 @@
         <v>1749.65293005789</v>
       </c>
       <c r="K11" s="18" t="str">
-        <f aca="false">IF('Set 1'!M11="","",'Set 1'!M11)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!M11),'Set 1'!M11,"")</f>
         <v/>
       </c>
       <c r="L11" s="18" t="str">
-        <f aca="false">IF('Set 1'!N11="","",'Set 1'!N11)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!N11),'Set 1'!N11,"")</f>
         <v/>
       </c>
       <c r="M11" s="19" t="n">
@@ -6568,11 +6578,11 @@
         <v>7.64497699999999</v>
       </c>
       <c r="N11" s="19" t="str">
-        <f aca="false">IF('Set 1'!P11="","",'Set 1'!P11)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!P11),'Set 1'!P11,"")</f>
         <v/>
       </c>
       <c r="O11" s="19" t="str">
-        <f aca="false">IF('Set 1'!Q11="","",'Set 1'!Q11)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!Q11),'Set 1'!Q11,"")</f>
         <v/>
       </c>
       <c r="P11" s="20" t="n">
@@ -6580,23 +6590,23 @@
         <v>749.678589646605</v>
       </c>
       <c r="Q11" s="19" t="str">
-        <f aca="false">IF('Set 1'!S11="","",'Set 1'!S11)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!S11),'Set 1'!S11,"")</f>
         <v/>
       </c>
       <c r="R11" s="20" t="str">
-        <f aca="false">IF('Set 1'!T11="","",'Set 1'!T11)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!T11),'Set 1'!T11,"")</f>
         <v/>
       </c>
       <c r="S11" s="21" t="str">
-        <f aca="false">IF('Set 1'!V11="","",'Set 1'!V11)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!V11),'Set 1'!V11,"")</f>
         <v/>
       </c>
       <c r="T11" s="21" t="str">
-        <f aca="false">IF('Set 1'!W11="","",'Set 1'!W11)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!W11),'Set 1'!W11,"")</f>
         <v/>
       </c>
       <c r="U11" s="22" t="str">
-        <f aca="false">IF('Set 1'!X11="","",'Set 1'!X11)</f>
+        <f aca="false">IF(ISNUMBER('Set 1'!X11),'Set 1'!X11,"")</f>
         <v/>
       </c>
     </row>
@@ -6629,11 +6639,11 @@
         <v>252.941476967729</v>
       </c>
       <c r="H12" s="18" t="str">
-        <f aca="false">IF('Set 2'!J2="","",'Set 2'!J2)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!J2),'Set 2'!J2,"")</f>
         <v/>
       </c>
       <c r="I12" s="18" t="str">
-        <f aca="false">IF('Set 2'!K2="","",'Set 2'!K2)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!K2),'Set 2'!K2,"")</f>
         <v/>
       </c>
       <c r="J12" s="18" t="n">
@@ -6641,11 +6651,11 @@
         <v>1272.77675106126</v>
       </c>
       <c r="K12" s="18" t="str">
-        <f aca="false">IF('Set 2'!M2="","",'Set 2'!M2)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!M2),'Set 2'!M2,"")</f>
         <v/>
       </c>
       <c r="L12" s="18" t="str">
-        <f aca="false">IF('Set 2'!N2="","",'Set 2'!N2)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!N2),'Set 2'!N2,"")</f>
         <v/>
       </c>
       <c r="M12" s="19" t="n">
@@ -6653,11 +6663,11 @@
         <v>7.51738999999999</v>
       </c>
       <c r="N12" s="19" t="str">
-        <f aca="false">IF('Set 2'!P2="","",'Set 2'!P2)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!P2),'Set 2'!P2,"")</f>
         <v/>
       </c>
       <c r="O12" s="19" t="str">
-        <f aca="false">IF('Set 2'!Q2="","",'Set 2'!Q2)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!Q2),'Set 2'!Q2,"")</f>
         <v/>
       </c>
       <c r="P12" s="20" t="n">
@@ -6665,23 +6675,23 @@
         <v>194.037396072618</v>
       </c>
       <c r="Q12" s="19" t="str">
-        <f aca="false">IF('Set 2'!S2="","",'Set 2'!S2)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!S2),'Set 2'!S2,"")</f>
         <v/>
       </c>
       <c r="R12" s="20" t="str">
-        <f aca="false">IF('Set 2'!T2="","",'Set 2'!T2)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!T2),'Set 2'!T2,"")</f>
         <v/>
       </c>
       <c r="S12" s="21" t="str">
-        <f aca="false">IF('Set 2'!V2="","",'Set 2'!V2)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!V2),'Set 2'!V2,"")</f>
         <v/>
       </c>
       <c r="T12" s="21" t="str">
-        <f aca="false">IF('Set 2'!W2="","",'Set 2'!W2)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!W2),'Set 2'!W2,"")</f>
         <v/>
       </c>
       <c r="U12" s="22" t="str">
-        <f aca="false">IF('Set 2'!X2="","",'Set 2'!X2)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!X2),'Set 2'!X2,"")</f>
         <v/>
       </c>
     </row>
@@ -6714,11 +6724,11 @@
         <v>252.932975417789</v>
       </c>
       <c r="H13" s="18" t="str">
-        <f aca="false">IF('Set 2'!J3="","",'Set 2'!J3)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!J3),'Set 2'!J3,"")</f>
         <v/>
       </c>
       <c r="I13" s="18" t="str">
-        <f aca="false">IF('Set 2'!K3="","",'Set 2'!K3)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!K3),'Set 2'!K3,"")</f>
         <v/>
       </c>
       <c r="J13" s="18" t="n">
@@ -6726,11 +6736,11 @@
         <v>1271.95778259744</v>
       </c>
       <c r="K13" s="18" t="str">
-        <f aca="false">IF('Set 2'!M3="","",'Set 2'!M3)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!M3),'Set 2'!M3,"")</f>
         <v/>
       </c>
       <c r="L13" s="18" t="str">
-        <f aca="false">IF('Set 2'!N3="","",'Set 2'!N3)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!N3),'Set 2'!N3,"")</f>
         <v/>
       </c>
       <c r="M13" s="19" t="n">
@@ -6738,11 +6748,11 @@
         <v>7.51647999999999</v>
       </c>
       <c r="N13" s="19" t="str">
-        <f aca="false">IF('Set 2'!P3="","",'Set 2'!P3)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!P3),'Set 2'!P3,"")</f>
         <v/>
       </c>
       <c r="O13" s="19" t="str">
-        <f aca="false">IF('Set 2'!Q3="","",'Set 2'!Q3)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!Q3),'Set 2'!Q3,"")</f>
         <v/>
       </c>
       <c r="P13" s="20" t="n">
@@ -6750,23 +6760,23 @@
         <v>194.398322200401</v>
       </c>
       <c r="Q13" s="19" t="str">
-        <f aca="false">IF('Set 2'!S3="","",'Set 2'!S3)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!S3),'Set 2'!S3,"")</f>
         <v/>
       </c>
       <c r="R13" s="20" t="str">
-        <f aca="false">IF('Set 2'!T3="","",'Set 2'!T3)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!T3),'Set 2'!T3,"")</f>
         <v/>
       </c>
       <c r="S13" s="21" t="str">
-        <f aca="false">IF('Set 2'!V3="","",'Set 2'!V3)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!V3),'Set 2'!V3,"")</f>
         <v/>
       </c>
       <c r="T13" s="21" t="str">
-        <f aca="false">IF('Set 2'!W3="","",'Set 2'!W3)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!W3),'Set 2'!W3,"")</f>
         <v/>
       </c>
       <c r="U13" s="22" t="str">
-        <f aca="false">IF('Set 2'!X3="","",'Set 2'!X3)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!X3),'Set 2'!X3,"")</f>
         <v/>
       </c>
     </row>
@@ -6799,11 +6809,11 @@
         <v>252.941476967729</v>
       </c>
       <c r="H14" s="18" t="str">
-        <f aca="false">IF('Set 2'!J4="","",'Set 2'!J4)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!J4),'Set 2'!J4,"")</f>
         <v/>
       </c>
       <c r="I14" s="18" t="str">
-        <f aca="false">IF('Set 2'!K4="","",'Set 2'!K4)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!K4),'Set 2'!K4,"")</f>
         <v/>
       </c>
       <c r="J14" s="18" t="n">
@@ -6811,11 +6821,11 @@
         <v>1274.36021618533</v>
       </c>
       <c r="K14" s="18" t="str">
-        <f aca="false">IF('Set 2'!M4="","",'Set 2'!M4)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!M4),'Set 2'!M4,"")</f>
         <v/>
       </c>
       <c r="L14" s="18" t="str">
-        <f aca="false">IF('Set 2'!N4="","",'Set 2'!N4)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!N4),'Set 2'!N4,"")</f>
         <v/>
       </c>
       <c r="M14" s="19" t="n">
@@ -6823,11 +6833,11 @@
         <v>7.51820299999999</v>
       </c>
       <c r="N14" s="19" t="str">
-        <f aca="false">IF('Set 2'!P4="","",'Set 2'!P4)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!P4),'Set 2'!P4,"")</f>
         <v/>
       </c>
       <c r="O14" s="19" t="str">
-        <f aca="false">IF('Set 2'!Q4="","",'Set 2'!Q4)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!Q4),'Set 2'!Q4,"")</f>
         <v/>
       </c>
       <c r="P14" s="20" t="n">
@@ -6835,23 +6845,23 @@
         <v>195.04844034153</v>
       </c>
       <c r="Q14" s="19" t="str">
-        <f aca="false">IF('Set 2'!S4="","",'Set 2'!S4)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!S4),'Set 2'!S4,"")</f>
         <v/>
       </c>
       <c r="R14" s="20" t="str">
-        <f aca="false">IF('Set 2'!T4="","",'Set 2'!T4)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!T4),'Set 2'!T4,"")</f>
         <v/>
       </c>
       <c r="S14" s="21" t="str">
-        <f aca="false">IF('Set 2'!V4="","",'Set 2'!V4)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!V4),'Set 2'!V4,"")</f>
         <v/>
       </c>
       <c r="T14" s="21" t="str">
-        <f aca="false">IF('Set 2'!W4="","",'Set 2'!W4)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!W4),'Set 2'!W4,"")</f>
         <v/>
       </c>
       <c r="U14" s="22" t="str">
-        <f aca="false">IF('Set 2'!X4="","",'Set 2'!X4)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!X4),'Set 2'!X4,"")</f>
         <v/>
       </c>
     </row>
@@ -6884,11 +6894,11 @@
         <v>244.381588889695</v>
       </c>
       <c r="H15" s="18" t="str">
-        <f aca="false">IF('Set 2'!J5="","",'Set 2'!J5)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!J5),'Set 2'!J5,"")</f>
         <v/>
       </c>
       <c r="I15" s="18" t="str">
-        <f aca="false">IF('Set 2'!K5="","",'Set 2'!K5)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!K5),'Set 2'!K5,"")</f>
         <v/>
       </c>
       <c r="J15" s="18" t="n">
@@ -6896,11 +6906,11 @@
         <v>1240.57518622454</v>
       </c>
       <c r="K15" s="18" t="str">
-        <f aca="false">IF('Set 2'!M5="","",'Set 2'!M5)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!M5),'Set 2'!M5,"")</f>
         <v/>
       </c>
       <c r="L15" s="18" t="str">
-        <f aca="false">IF('Set 2'!N5="","",'Set 2'!N5)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!N5),'Set 2'!N5,"")</f>
         <v/>
       </c>
       <c r="M15" s="19" t="n">
@@ -6908,11 +6918,11 @@
         <v>7.54008299999999</v>
       </c>
       <c r="N15" s="19" t="str">
-        <f aca="false">IF('Set 2'!P5="","",'Set 2'!P5)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!P5),'Set 2'!P5,"")</f>
         <v/>
       </c>
       <c r="O15" s="19" t="str">
-        <f aca="false">IF('Set 2'!Q5="","",'Set 2'!Q5)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!Q5),'Set 2'!Q5,"")</f>
         <v/>
       </c>
       <c r="P15" s="20" t="n">
@@ -6920,23 +6930,23 @@
         <v>265.165023707051</v>
       </c>
       <c r="Q15" s="19" t="str">
-        <f aca="false">IF('Set 2'!S5="","",'Set 2'!S5)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!S5),'Set 2'!S5,"")</f>
         <v/>
       </c>
       <c r="R15" s="20" t="str">
-        <f aca="false">IF('Set 2'!T5="","",'Set 2'!T5)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!T5),'Set 2'!T5,"")</f>
         <v/>
       </c>
       <c r="S15" s="21" t="str">
-        <f aca="false">IF('Set 2'!V5="","",'Set 2'!V5)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!V5),'Set 2'!V5,"")</f>
         <v/>
       </c>
       <c r="T15" s="21" t="str">
-        <f aca="false">IF('Set 2'!W5="","",'Set 2'!W5)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!W5),'Set 2'!W5,"")</f>
         <v/>
       </c>
       <c r="U15" s="22" t="str">
-        <f aca="false">IF('Set 2'!X5="","",'Set 2'!X5)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!X5),'Set 2'!X5,"")</f>
         <v/>
       </c>
     </row>
@@ -6969,11 +6979,11 @@
         <v>244.510942148903</v>
       </c>
       <c r="H16" s="18" t="str">
-        <f aca="false">IF('Set 2'!J6="","",'Set 2'!J6)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!J6),'Set 2'!J6,"")</f>
         <v/>
       </c>
       <c r="I16" s="18" t="str">
-        <f aca="false">IF('Set 2'!K6="","",'Set 2'!K6)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!K6),'Set 2'!K6,"")</f>
         <v/>
       </c>
       <c r="J16" s="18" t="n">
@@ -6981,11 +6991,11 @@
         <v>1241.43819349573</v>
       </c>
       <c r="K16" s="18" t="str">
-        <f aca="false">IF('Set 2'!M6="","",'Set 2'!M6)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!M6),'Set 2'!M6,"")</f>
         <v/>
       </c>
       <c r="L16" s="18" t="str">
-        <f aca="false">IF('Set 2'!N6="","",'Set 2'!N6)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!N6),'Set 2'!N6,"")</f>
         <v/>
       </c>
       <c r="M16" s="19" t="n">
@@ -6993,11 +7003,11 @@
         <v>7.54310199999999</v>
       </c>
       <c r="N16" s="19" t="str">
-        <f aca="false">IF('Set 2'!P6="","",'Set 2'!P6)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!P6),'Set 2'!P6,"")</f>
         <v/>
       </c>
       <c r="O16" s="19" t="str">
-        <f aca="false">IF('Set 2'!Q6="","",'Set 2'!Q6)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!Q6),'Set 2'!Q6,"")</f>
         <v/>
       </c>
       <c r="P16" s="20" t="n">
@@ -7005,23 +7015,23 @@
         <v>265.45253270235</v>
       </c>
       <c r="Q16" s="19" t="str">
-        <f aca="false">IF('Set 2'!S6="","",'Set 2'!S6)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!S6),'Set 2'!S6,"")</f>
         <v/>
       </c>
       <c r="R16" s="20" t="str">
-        <f aca="false">IF('Set 2'!T6="","",'Set 2'!T6)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!T6),'Set 2'!T6,"")</f>
         <v/>
       </c>
       <c r="S16" s="21" t="str">
-        <f aca="false">IF('Set 2'!V6="","",'Set 2'!V6)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!V6),'Set 2'!V6,"")</f>
         <v/>
       </c>
       <c r="T16" s="21" t="str">
-        <f aca="false">IF('Set 2'!W6="","",'Set 2'!W6)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!W6),'Set 2'!W6,"")</f>
         <v/>
       </c>
       <c r="U16" s="22" t="str">
-        <f aca="false">IF('Set 2'!X6="","",'Set 2'!X6)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!X6),'Set 2'!X6,"")</f>
         <v/>
       </c>
     </row>
@@ -7054,11 +7064,11 @@
         <v>244.518491839956</v>
       </c>
       <c r="H17" s="18" t="str">
-        <f aca="false">IF('Set 2'!J7="","",'Set 2'!J7)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!J7),'Set 2'!J7,"")</f>
         <v/>
       </c>
       <c r="I17" s="18" t="str">
-        <f aca="false">IF('Set 2'!K7="","",'Set 2'!K7)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!K7),'Set 2'!K7,"")</f>
         <v/>
       </c>
       <c r="J17" s="18" t="n">
@@ -7066,11 +7076,11 @@
         <v>1244.01182011071</v>
       </c>
       <c r="K17" s="18" t="str">
-        <f aca="false">IF('Set 2'!M7="","",'Set 2'!M7)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!M7),'Set 2'!M7,"")</f>
         <v/>
       </c>
       <c r="L17" s="18" t="str">
-        <f aca="false">IF('Set 2'!N7="","",'Set 2'!N7)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!N7),'Set 2'!N7,"")</f>
         <v/>
       </c>
       <c r="M17" s="19" t="n">
@@ -7078,11 +7088,11 @@
         <v>7.54482499999999</v>
       </c>
       <c r="N17" s="19" t="str">
-        <f aca="false">IF('Set 2'!P7="","",'Set 2'!P7)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!P7),'Set 2'!P7,"")</f>
         <v/>
       </c>
       <c r="O17" s="19" t="str">
-        <f aca="false">IF('Set 2'!Q7="","",'Set 2'!Q7)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!Q7),'Set 2'!Q7,"")</f>
         <v/>
       </c>
       <c r="P17" s="20" t="n">
@@ -7090,23 +7100,23 @@
         <v>266.130053765627</v>
       </c>
       <c r="Q17" s="19" t="str">
-        <f aca="false">IF('Set 2'!S7="","",'Set 2'!S7)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!S7),'Set 2'!S7,"")</f>
         <v/>
       </c>
       <c r="R17" s="20" t="str">
-        <f aca="false">IF('Set 2'!T7="","",'Set 2'!T7)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!T7),'Set 2'!T7,"")</f>
         <v/>
       </c>
       <c r="S17" s="21" t="str">
-        <f aca="false">IF('Set 2'!V7="","",'Set 2'!V7)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!V7),'Set 2'!V7,"")</f>
         <v/>
       </c>
       <c r="T17" s="21" t="str">
-        <f aca="false">IF('Set 2'!W7="","",'Set 2'!W7)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!W7),'Set 2'!W7,"")</f>
         <v/>
       </c>
       <c r="U17" s="22" t="str">
-        <f aca="false">IF('Set 2'!X7="","",'Set 2'!X7)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!X7),'Set 2'!X7,"")</f>
         <v/>
       </c>
     </row>
@@ -7139,11 +7149,11 @@
         <v>312.794696376031</v>
       </c>
       <c r="H18" s="18" t="str">
-        <f aca="false">IF('Set 2'!J8="","",'Set 2'!J8)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!J8),'Set 2'!J8,"")</f>
         <v/>
       </c>
       <c r="I18" s="18" t="str">
-        <f aca="false">IF('Set 2'!K8="","",'Set 2'!K8)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!K8),'Set 2'!K8,"")</f>
         <v/>
       </c>
       <c r="J18" s="18" t="n">
@@ -7151,11 +7161,11 @@
         <v>1161.08798987177</v>
       </c>
       <c r="K18" s="18" t="str">
-        <f aca="false">IF('Set 2'!M8="","",'Set 2'!M8)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!M8),'Set 2'!M8,"")</f>
         <v/>
       </c>
       <c r="L18" s="18" t="str">
-        <f aca="false">IF('Set 2'!N8="","",'Set 2'!N8)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!N8),'Set 2'!N8,"")</f>
         <v/>
       </c>
       <c r="M18" s="19" t="n">
@@ -7163,11 +7173,11 @@
         <v>7.66023</v>
       </c>
       <c r="N18" s="19" t="str">
-        <f aca="false">IF('Set 2'!P8="","",'Set 2'!P8)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!P8),'Set 2'!P8,"")</f>
         <v/>
       </c>
       <c r="O18" s="19" t="str">
-        <f aca="false">IF('Set 2'!Q8="","",'Set 2'!Q8)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!Q8),'Set 2'!Q8,"")</f>
         <v/>
       </c>
       <c r="P18" s="20" t="n">
@@ -7175,23 +7185,23 @@
         <v>612.727627704531</v>
       </c>
       <c r="Q18" s="19" t="str">
-        <f aca="false">IF('Set 2'!S8="","",'Set 2'!S8)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!S8),'Set 2'!S8,"")</f>
         <v/>
       </c>
       <c r="R18" s="20" t="str">
-        <f aca="false">IF('Set 2'!T8="","",'Set 2'!T8)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!T8),'Set 2'!T8,"")</f>
         <v/>
       </c>
       <c r="S18" s="21" t="str">
-        <f aca="false">IF('Set 2'!V8="","",'Set 2'!V8)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!V8),'Set 2'!V8,"")</f>
         <v/>
       </c>
       <c r="T18" s="21" t="str">
-        <f aca="false">IF('Set 2'!W8="","",'Set 2'!W8)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!W8),'Set 2'!W8,"")</f>
         <v/>
       </c>
       <c r="U18" s="22" t="str">
-        <f aca="false">IF('Set 2'!X8="","",'Set 2'!X8)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!X8),'Set 2'!X8,"")</f>
         <v/>
       </c>
     </row>
@@ -7224,11 +7234,11 @@
         <v>312.794696376031</v>
       </c>
       <c r="H19" s="18" t="str">
-        <f aca="false">IF('Set 2'!J9="","",'Set 2'!J9)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!J9),'Set 2'!J9,"")</f>
         <v/>
       </c>
       <c r="I19" s="18" t="str">
-        <f aca="false">IF('Set 2'!K9="","",'Set 2'!K9)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!K9),'Set 2'!K9,"")</f>
         <v/>
       </c>
       <c r="J19" s="18" t="n">
@@ -7236,11 +7246,11 @@
         <v>1161.74939305885</v>
       </c>
       <c r="K19" s="18" t="str">
-        <f aca="false">IF('Set 2'!M9="","",'Set 2'!M9)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!M9),'Set 2'!M9,"")</f>
         <v/>
       </c>
       <c r="L19" s="18" t="str">
-        <f aca="false">IF('Set 2'!N9="","",'Set 2'!N9)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!N9),'Set 2'!N9,"")</f>
         <v/>
       </c>
       <c r="M19" s="19" t="n">
@@ -7248,11 +7258,11 @@
         <v>7.660533</v>
       </c>
       <c r="N19" s="19" t="str">
-        <f aca="false">IF('Set 2'!P9="","",'Set 2'!P9)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!P9),'Set 2'!P9,"")</f>
         <v/>
       </c>
       <c r="O19" s="19" t="str">
-        <f aca="false">IF('Set 2'!Q9="","",'Set 2'!Q9)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!Q9),'Set 2'!Q9,"")</f>
         <v/>
       </c>
       <c r="P19" s="20" t="n">
@@ -7260,23 +7270,23 @@
         <v>613.002453735894</v>
       </c>
       <c r="Q19" s="19" t="str">
-        <f aca="false">IF('Set 2'!S9="","",'Set 2'!S9)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!S9),'Set 2'!S9,"")</f>
         <v/>
       </c>
       <c r="R19" s="20" t="str">
-        <f aca="false">IF('Set 2'!T9="","",'Set 2'!T9)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!T9),'Set 2'!T9,"")</f>
         <v/>
       </c>
       <c r="S19" s="21" t="str">
-        <f aca="false">IF('Set 2'!V9="","",'Set 2'!V9)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!V9),'Set 2'!V9,"")</f>
         <v/>
       </c>
       <c r="T19" s="21" t="str">
-        <f aca="false">IF('Set 2'!W9="","",'Set 2'!W9)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!W9),'Set 2'!W9,"")</f>
         <v/>
       </c>
       <c r="U19" s="22" t="str">
-        <f aca="false">IF('Set 2'!X9="","",'Set 2'!X9)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!X9),'Set 2'!X9,"")</f>
         <v/>
       </c>
     </row>
@@ -7309,11 +7319,11 @@
         <v>365.193909930287</v>
       </c>
       <c r="H20" s="18" t="str">
-        <f aca="false">IF('Set 2'!J10="","",'Set 2'!J10)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!J10),'Set 2'!J10,"")</f>
         <v/>
       </c>
       <c r="I20" s="18" t="str">
-        <f aca="false">IF('Set 2'!K10="","",'Set 2'!K10)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!K10),'Set 2'!K10,"")</f>
         <v/>
       </c>
       <c r="J20" s="18" t="n">
@@ -7321,11 +7331,11 @@
         <v>1153.32150850965</v>
       </c>
       <c r="K20" s="18" t="str">
-        <f aca="false">IF('Set 2'!M10="","",'Set 2'!M10)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!M10),'Set 2'!M10,"")</f>
         <v/>
       </c>
       <c r="L20" s="18" t="str">
-        <f aca="false">IF('Set 2'!N10="","",'Set 2'!N10)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!N10),'Set 2'!N10,"")</f>
         <v/>
       </c>
       <c r="M20" s="19" t="n">
@@ -7333,11 +7343,11 @@
         <v>7.677769</v>
       </c>
       <c r="N20" s="19" t="str">
-        <f aca="false">IF('Set 2'!P10="","",'Set 2'!P10)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!P10),'Set 2'!P10,"")</f>
         <v/>
       </c>
       <c r="O20" s="19" t="str">
-        <f aca="false">IF('Set 2'!Q10="","",'Set 2'!Q10)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!Q10),'Set 2'!Q10,"")</f>
         <v/>
       </c>
       <c r="P20" s="20" t="n">
@@ -7345,23 +7355,23 @@
         <v>646.382176644298</v>
       </c>
       <c r="Q20" s="19" t="str">
-        <f aca="false">IF('Set 2'!S10="","",'Set 2'!S10)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!S10),'Set 2'!S10,"")</f>
         <v/>
       </c>
       <c r="R20" s="20" t="str">
-        <f aca="false">IF('Set 2'!T10="","",'Set 2'!T10)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!T10),'Set 2'!T10,"")</f>
         <v/>
       </c>
       <c r="S20" s="21" t="str">
-        <f aca="false">IF('Set 2'!V10="","",'Set 2'!V10)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!V10),'Set 2'!V10,"")</f>
         <v/>
       </c>
       <c r="T20" s="21" t="str">
-        <f aca="false">IF('Set 2'!W10="","",'Set 2'!W10)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!W10),'Set 2'!W10,"")</f>
         <v/>
       </c>
       <c r="U20" s="22" t="str">
-        <f aca="false">IF('Set 2'!X10="","",'Set 2'!X10)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!X10),'Set 2'!X10,"")</f>
         <v/>
       </c>
     </row>
@@ -7394,11 +7404,11 @@
         <v>365.193909930287</v>
       </c>
       <c r="H21" s="18" t="str">
-        <f aca="false">IF('Set 2'!J11="","",'Set 2'!J11)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!J11),'Set 2'!J11,"")</f>
         <v/>
       </c>
       <c r="I21" s="18" t="str">
-        <f aca="false">IF('Set 2'!K11="","",'Set 2'!K11)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!K11),'Set 2'!K11,"")</f>
         <v/>
       </c>
       <c r="J21" s="18" t="n">
@@ -7406,11 +7416,11 @@
         <v>1147.99922817314</v>
       </c>
       <c r="K21" s="18" t="str">
-        <f aca="false">IF('Set 2'!M11="","",'Set 2'!M11)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!M11),'Set 2'!M11,"")</f>
         <v/>
       </c>
       <c r="L21" s="18" t="str">
-        <f aca="false">IF('Set 2'!N11="","",'Set 2'!N11)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!N11),'Set 2'!N11,"")</f>
         <v/>
       </c>
       <c r="M21" s="19" t="n">
@@ -7418,11 +7428,11 @@
         <v>7.680507</v>
       </c>
       <c r="N21" s="19" t="str">
-        <f aca="false">IF('Set 2'!P11="","",'Set 2'!P11)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!P11),'Set 2'!P11,"")</f>
         <v/>
       </c>
       <c r="O21" s="19" t="str">
-        <f aca="false">IF('Set 2'!Q11="","",'Set 2'!Q11)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!Q11),'Set 2'!Q11,"")</f>
         <v/>
       </c>
       <c r="P21" s="20" t="n">
@@ -7430,23 +7440,23 @@
         <v>655.711579058753</v>
       </c>
       <c r="Q21" s="19" t="str">
-        <f aca="false">IF('Set 2'!S11="","",'Set 2'!S11)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!S11),'Set 2'!S11,"")</f>
         <v/>
       </c>
       <c r="R21" s="20" t="str">
-        <f aca="false">IF('Set 2'!T11="","",'Set 2'!T11)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!T11),'Set 2'!T11,"")</f>
         <v/>
       </c>
       <c r="S21" s="21" t="str">
-        <f aca="false">IF('Set 2'!V11="","",'Set 2'!V11)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!V11),'Set 2'!V11,"")</f>
         <v/>
       </c>
       <c r="T21" s="21" t="str">
-        <f aca="false">IF('Set 2'!W11="","",'Set 2'!W11)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!W11),'Set 2'!W11,"")</f>
         <v/>
       </c>
       <c r="U21" s="22" t="str">
-        <f aca="false">IF('Set 2'!X11="","",'Set 2'!X11)</f>
+        <f aca="false">IF(ISNUMBER('Set 2'!X11),'Set 2'!X11,"")</f>
         <v/>
       </c>
     </row>
@@ -7654,7 +7664,7 @@
     <tabColor rgb="FF7F7F7F"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -7720,7 +7730,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="37" t="s">
         <v>55</v>
       </c>
@@ -7728,45 +7738,45 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="33" t="s">
+    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="38" t="s">
         <v>57</v>
       </c>
       <c r="C11" s="33" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="32" t="s">
+    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="33" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="38" t="s">
+      <c r="C12" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="C14" s="33" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="32" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="38" t="s">
+    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="39" t="s">
         <v>62</v>
       </c>
       <c r="C15" s="33" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="38" t="s">
+    <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="39" t="s">
         <v>64</v>
       </c>
       <c r="C16" s="33" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="38" t="s">
+    <row r="17" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="39" t="s">
         <v>66</v>
       </c>
       <c r="C17" s="33" t="s">
@@ -7774,173 +7784,181 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="38" t="s">
+      <c r="A18" s="39" t="s">
         <v>68</v>
       </c>
       <c r="C18" s="33" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="38" t="s">
+    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="39" t="s">
         <v>70</v>
       </c>
       <c r="C19" s="33" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="38" t="s">
+    <row r="20" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="39" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" s="33" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="33" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="38" t="s">
+      <c r="C21" s="33" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="33" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="38" t="s">
+      <c r="C22" s="33" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="39" t="s">
         <v>24</v>
-      </c>
-      <c r="C22" s="33" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="38" t="s">
-        <v>75</v>
       </c>
       <c r="C23" s="33" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="38" t="s">
+    <row r="24" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="39" t="s">
         <v>77</v>
       </c>
       <c r="C24" s="33" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="38" t="s">
+    <row r="25" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="39" t="s">
+        <v>79</v>
+      </c>
+      <c r="C25" s="33" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C25" s="33" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="32" t="s">
-        <v>80</v>
+      <c r="C26" s="33" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="33" t="s">
-        <v>81</v>
-      </c>
-      <c r="C28" s="33" t="s">
+      <c r="A28" s="32" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="33" t="s">
-        <v>8</v>
-      </c>
-      <c r="B29" s="39" t="n">
-        <v>572</v>
+        <v>83</v>
+      </c>
+      <c r="C29" s="33" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="B30" s="39" t="n">
-        <v>796</v>
+        <v>8</v>
+      </c>
+      <c r="B30" s="40" t="n">
+        <v>572</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="33" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B31" s="40" t="n">
-        <v>4.95</v>
+        <v>796</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="B32" s="40" t="n">
-        <v>5.57</v>
+        <v>14</v>
+      </c>
+      <c r="B32" s="41" t="n">
+        <v>4.95</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="33" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B33" s="41" t="n">
-        <v>0.931</v>
+        <v>5.57</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="B34" s="41" t="n">
-        <v>0.618</v>
+        <v>20</v>
+      </c>
+      <c r="B34" s="42" t="n">
+        <v>0.931</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="B35" s="42" t="n">
+        <v>0.618</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="B35" s="42" t="n">
+      <c r="B36" s="43" t="n">
         <v>0.000178</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="32" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="33" t="s">
-        <v>84</v>
-      </c>
-      <c r="C38" s="33" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="32" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="33" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C39" s="33" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="33" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="33" t="s">
-        <v>84</v>
-      </c>
       <c r="C40" s="33" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="33" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>88</v>
+        <v>89</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="33" t="s">
+        <v>86</v>
+      </c>
+      <c r="C42" s="33" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Match Aum's sweep sheet: c min grid, .vtk paths, dx parameters
Set 1 c min for point 2 now reads 50.558 like his sheet: c min/c max use the last
sample at L - dx, with dx on the Notes sheet (rows 6-7; 5 nm for set 1, an
assumed 0.5 nm for set 2). The CM field column follows his path pattern
(set1_CM/fields/point01_wv400nm_amp0.56pct.vtk), built without locale-dependent
TEXT formats, with column Z widened to hold it. Notes text, header comments and
row heights updated. SIM columns stay blank.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMG2h8P1NWmCTJjSz9snJ3
</commit_message>
<xml_diff>
--- a/CM_Sweep_Sets_1_2.xlsx
+++ b/CM_Sweep_Sets_1_2.xlsx
@@ -85,7 +85,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">avg - amp when the domain holds &gt;= 0.75 waves. With fewer waves, the lowest value reached: avg (at y = 0) or the sine value at the end of the domain, whichever is lower. Closed-form estimate of the sine.m field; see Notes.</t>
+          <t xml:space="preserve">avg - amp once the sampled field holds &gt;= 0.75 waves; with fewer, the lowest value reached: avg (y = 0) or the sine value at the last sample (y = L - dx), whichever is lower. L and dx are on the Notes sheet.</t>
         </r>
       </text>
     </comment>
@@ -97,7 +97,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">avg + amp when the domain holds &gt;= 0.25 waves, otherwise the sine value at the end of the domain (the highest value reached). See Notes.</t>
+          <t xml:space="preserve">avg + amp once the sampled field holds &gt;= 0.25 waves, otherwise the sine value at the last sample (y = L - dx, the highest value reached). L and dx are on the Notes sheet.</t>
         </r>
       </text>
     </comment>
@@ -193,7 +193,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Formula: set&lt;N&gt;_pt&lt;point&gt;.vtk, inferred from sine.m / write_vtk (set2_pt7.vtk). Overwrite with the real file name if yours differ.</t>
+          <t xml:space="preserve">Formula: Aum's path pattern set&lt;N&gt;_CM/fields/point&lt;NN&gt;_wv&lt;lambda&gt;nm_amp&lt;amp&gt;pct.vtk. sine.m writes names like set2_pt7.vtk; overwrite with the real file name if yours differ.</t>
         </r>
       </text>
     </comment>
@@ -263,7 +263,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">avg - amp when the domain holds &gt;= 0.75 waves. With fewer waves, the lowest value reached: avg (at y = 0) or the sine value at the end of the domain, whichever is lower. Closed-form estimate of the sine.m field; see Notes.</t>
+          <t xml:space="preserve">avg - amp once the sampled field holds &gt;= 0.75 waves; with fewer, the lowest value reached: avg (y = 0) or the sine value at the last sample (y = L - dx), whichever is lower. L and dx are on the Notes sheet.</t>
         </r>
       </text>
     </comment>
@@ -275,7 +275,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">avg + amp when the domain holds &gt;= 0.25 waves, otherwise the sine value at the end of the domain (the highest value reached). See Notes.</t>
+          <t xml:space="preserve">avg + amp once the sampled field holds &gt;= 0.25 waves, otherwise the sine value at the last sample (y = L - dx, the highest value reached). L and dx are on the Notes sheet.</t>
         </r>
       </text>
     </comment>
@@ -371,7 +371,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Formula: set&lt;N&gt;_pt&lt;point&gt;.vtk, inferred from sine.m / write_vtk (set2_pt7.vtk). Overwrite with the real file name if yours differ.</t>
+          <t xml:space="preserve">Formula: Aum's path pattern set&lt;N&gt;_CM/fields/point&lt;NN&gt;_wv&lt;lambda&gt;nm_amp&lt;amp&gt;pct.vtk. sine.m writes names like set2_pt7.vtk; overwrite with the real file name if yours differ.</t>
         </r>
       </text>
     </comment>
@@ -380,7 +380,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="95">
   <si>
     <t xml:space="preserve">Point</t>
   </si>
@@ -529,7 +529,7 @@
     <t xml:space="preserve">Set 2 domain length L (nm)</t>
   </si>
   <si>
-    <t xml:space="preserve">Assumption: set to 640 because all 10 Set 2 renders show 640/λ waves (e.g. λ = 640 shows one wave, λ = 80 shows eight). sine.m (Ny = 1280, wv = 1280 for set2_pt7) points to 1280 instead, so the two disagree. Confirm which grid set 2 used; changing this cell updates waves, c min and c max.</t>
+    <t xml:space="preserve">Assumption: set to 640 because all 10 Set 2 renders show 640/λ waves (e.g. λ = 640 shows one wave, λ = 80 shows eight). sine.m (Ny = 1280, wv = 1280 for set2_pt7) points to 1280 instead, so the two disagree. Confirm which grid set 2 used; changing this cell updates waves, c min and c max (check the grid spacing in B7 too).</t>
   </si>
   <si>
     <t xml:space="preserve">Legend</t>
@@ -583,7 +583,7 @@
     <t xml:space="preserve">c min, c max</t>
   </si>
   <si>
-    <t xml:space="preserve">c min = avg − amp once the domain holds 0.75 waves; with fewer, the lowest value reached (avg at y = 0, or the sine value at the end of the domain if that is lower). c max = avg + amp once the domain holds 0.25 waves. Closed-form estimate of the field built in sine.m (c = avg + amp·sin(2πy/λ)). For set 1 point 2 (960 nm in 640 nm, 0.67 waves) this gives c min = 50.550; Aum's sheet lists 50.558, which a coarser 5 nm grid reproduces, so his 2D grid is probably coarser. Every other set 1 point matches.</t>
+    <t xml:space="preserve">c min = avg − amp once the sampled field holds 0.75 waves; with fewer, the lowest value reached (avg at y = 0, or the sine value at the last sample if that is lower). c max = avg + amp once it holds 0.25 waves. The last sample sits at L − dx (dx = grid spacing, rows 6–7 above). Closed-form estimate of the field built in sine.m (c = avg + amp·sin(2πy/λ)); exact when λ is a multiple of 4·dx (true for every current point), otherwise the sampled extremes can sit slightly inside avg ± amp. With dx = 5 nm it reproduces every c min and c max in Aum's sheet, including 50.558 for set 1 point 2 (960 nm in 640 nm, last sample at 635 nm).</t>
   </si>
   <si>
     <t xml:space="preserve">ML V1 / V3 stress, strain range, loop area</t>
@@ -610,7 +610,7 @@
     <t xml:space="preserve">Rank of ML loop area minus rank of SIM loop area, both ascending within the 10 points of the set. Shown only when all 10 SIM loop areas are filled in. Reverse-engineered from Aum's sample, where it reproduces all 10 values.</t>
   </si>
   <si>
-    <t xml:space="preserve">set&lt;N&gt;_pt&lt;point&gt;.vtk, inferred from the write_vtk call in sine.m ('set2_pt7.vtk'). Aum's sheet uses a longer path pattern.</t>
+    <t xml:space="preserve">Aum's path pattern: set&lt;N&gt;_CM/fields/point&lt;NN&gt;_wv&lt;λ&gt;nm_amp&lt;amp&gt;pct.vtk (λ as an integer, amp with 2 decimals). Copied from his sheet for set 1 and extended to set 2 (the set 2 paths are not evidence-based). sine.m itself writes names like 'set2_pt7.vtk'; overwrite the formula if your files use those.</t>
   </si>
   <si>
     <t xml:space="preserve">Combined sheet</t>
@@ -649,10 +649,22 @@
     <t xml:space="preserve">Report 2: set 2 will need its own load steps (its 0.04% amplitude point is close to a uniform composition).</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirm the domain lengths above and the .vtk naming.</t>
+    <t xml:space="preserve">Confirm the set 2 domain length (B5) and grid spacing (B7), and that the .vtk paths match your folders.</t>
   </si>
   <si>
     <t xml:space="preserve">Stress-strain curves and any 2D / pseudo-2D comparison tabs are not built: they need the raw cycle data and 2D results.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set 1 grid spacing dx (nm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inferred from Aum's sheet: only his c min for set 1 point 2 (50.558) depends on dx. It fits a last sample at 635 nm, so 5 nm steps (128 points over 640 nm) is the natural choice (or 2.5 nm if his grid also resets its last slice to avg); any step from about 4.5 to 5.0 nm gives the same displayed value. Used for c min and c max only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set 2 grid spacing dx (nm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption: 0.5 nm = 640 nm over 1280 grid points. sine.m has Ny = 1280 points and writes SPACING 1 1 1 with no unit; read literally that is L = 1280 and dx = 1, so 0.5 nm follows from the L = 640 assumption in B5. dx only matters when the last sample falls before the crest (0.25 wave, c max) or the trough (0.75 wave, c min); at L = 640 that is set 2 point 8, whose c min moves by 0.001. sine.m also resets the last slice to avg, which would move it by a further 0.001. Change this together with B5.</t>
   </si>
 </sst>
 </file>
@@ -843,7 +855,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1017,6 +1029,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4043,7 +4059,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="22" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4146,11 +4162,11 @@
         <v>0.56</v>
       </c>
       <c r="G2" s="6" t="n">
-        <f aca="false">C2+F2*IF(E2&gt;=0.75,-1,MIN(0,SIN(2*PI()*E2)))</f>
+        <f aca="false">C2+F2*IF((Notes!$B$4-Notes!$B$6)/D2&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D2)))</f>
         <v>50.44</v>
       </c>
       <c r="H2" s="6" t="n">
-        <f aca="false">C2+F2*IF(E2&gt;=0.25,1,SIN(2*PI()*E2))</f>
+        <f aca="false">C2+F2*IF((Notes!$B$4-Notes!$B$6)/D2&gt;=0.25,1,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D2))</f>
         <v>51.56</v>
       </c>
       <c r="I2" s="2" t="n">
@@ -4194,8 +4210,8 @@
       <c r="X2" s="14"/>
       <c r="Y2" s="15"/>
       <c r="Z2" s="16" t="str">
-        <f aca="false">"set1_pt"&amp;A2&amp;".vtk"</f>
-        <v>set1_pt1.vtk</v>
+        <f aca="false">"set1_CM/fields/point"&amp;TEXT(A2,"00")&amp;"_wv"&amp;TEXT(D2,"0")&amp;"nm_amp"&amp;INT(ROUND(F2*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F2*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set1_CM/fields/point01_wv400nm_amp0.56pct.vtk</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4217,11 +4233,11 @@
         <v>0.52</v>
       </c>
       <c r="G3" s="6" t="n">
-        <f aca="false">C3+F3*IF(E3&gt;=0.75,-1,MIN(0,SIN(2*PI()*E3)))</f>
-        <v>50.5496667900321</v>
+        <f aca="false">C3+F3*IF((Notes!$B$4-Notes!$B$6)/D3&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D3)))</f>
+        <v>50.558414865606</v>
       </c>
       <c r="H3" s="6" t="n">
-        <f aca="false">C3+F3*IF(E3&gt;=0.25,1,SIN(2*PI()*E3))</f>
+        <f aca="false">C3+F3*IF((Notes!$B$4-Notes!$B$6)/D3&gt;=0.25,1,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D3))</f>
         <v>51.52</v>
       </c>
       <c r="I3" s="2" t="n">
@@ -4265,8 +4281,8 @@
       <c r="X3" s="14"/>
       <c r="Y3" s="15"/>
       <c r="Z3" s="16" t="str">
-        <f aca="false">"set1_pt"&amp;A3&amp;".vtk"</f>
-        <v>set1_pt2.vtk</v>
+        <f aca="false">"set1_CM/fields/point"&amp;TEXT(A3,"00")&amp;"_wv"&amp;TEXT(D3,"0")&amp;"nm_amp"&amp;INT(ROUND(F3*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F3*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set1_CM/fields/point02_wv960nm_amp0.52pct.vtk</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4288,11 +4304,11 @@
         <v>0.52</v>
       </c>
       <c r="G4" s="6" t="n">
-        <f aca="false">C4+F4*IF(E4&gt;=0.75,-1,MIN(0,SIN(2*PI()*E4)))</f>
+        <f aca="false">C4+F4*IF((Notes!$B$4-Notes!$B$6)/D4&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D4)))</f>
         <v>50.48</v>
       </c>
       <c r="H4" s="6" t="n">
-        <f aca="false">C4+F4*IF(E4&gt;=0.25,1,SIN(2*PI()*E4))</f>
+        <f aca="false">C4+F4*IF((Notes!$B$4-Notes!$B$6)/D4&gt;=0.25,1,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D4))</f>
         <v>51.52</v>
       </c>
       <c r="I4" s="2" t="n">
@@ -4336,8 +4352,8 @@
       <c r="X4" s="14"/>
       <c r="Y4" s="15"/>
       <c r="Z4" s="16" t="str">
-        <f aca="false">"set1_pt"&amp;A4&amp;".vtk"</f>
-        <v>set1_pt3.vtk</v>
+        <f aca="false">"set1_CM/fields/point"&amp;TEXT(A4,"00")&amp;"_wv"&amp;TEXT(D4,"0")&amp;"nm_amp"&amp;INT(ROUND(F4*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F4*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set1_CM/fields/point03_wv480nm_amp0.52pct.vtk</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4359,11 +4375,11 @@
         <v>0.52</v>
       </c>
       <c r="G5" s="6" t="n">
-        <f aca="false">C5+F5*IF(E5&gt;=0.75,-1,MIN(0,SIN(2*PI()*E5)))</f>
+        <f aca="false">C5+F5*IF((Notes!$B$4-Notes!$B$6)/D5&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D5)))</f>
         <v>50.48</v>
       </c>
       <c r="H5" s="6" t="n">
-        <f aca="false">C5+F5*IF(E5&gt;=0.25,1,SIN(2*PI()*E5))</f>
+        <f aca="false">C5+F5*IF((Notes!$B$4-Notes!$B$6)/D5&gt;=0.25,1,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D5))</f>
         <v>51.52</v>
       </c>
       <c r="I5" s="2" t="n">
@@ -4407,8 +4423,8 @@
       <c r="X5" s="14"/>
       <c r="Y5" s="15"/>
       <c r="Z5" s="16" t="str">
-        <f aca="false">"set1_pt"&amp;A5&amp;".vtk"</f>
-        <v>set1_pt4.vtk</v>
+        <f aca="false">"set1_CM/fields/point"&amp;TEXT(A5,"00")&amp;"_wv"&amp;TEXT(D5,"0")&amp;"nm_amp"&amp;INT(ROUND(F5*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F5*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set1_CM/fields/point04_wv240nm_amp0.52pct.vtk</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4430,11 +4446,11 @@
         <v>0.52</v>
       </c>
       <c r="G6" s="6" t="n">
-        <f aca="false">C6+F6*IF(E6&gt;=0.75,-1,MIN(0,SIN(2*PI()*E6)))</f>
+        <f aca="false">C6+F6*IF((Notes!$B$4-Notes!$B$6)/D6&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D6)))</f>
         <v>50.43</v>
       </c>
       <c r="H6" s="6" t="n">
-        <f aca="false">C6+F6*IF(E6&gt;=0.25,1,SIN(2*PI()*E6))</f>
+        <f aca="false">C6+F6*IF((Notes!$B$4-Notes!$B$6)/D6&gt;=0.25,1,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D6))</f>
         <v>51.47</v>
       </c>
       <c r="I6" s="2" t="n">
@@ -4478,8 +4494,8 @@
       <c r="X6" s="14"/>
       <c r="Y6" s="15"/>
       <c r="Z6" s="16" t="str">
-        <f aca="false">"set1_pt"&amp;A6&amp;".vtk"</f>
-        <v>set1_pt5.vtk</v>
+        <f aca="false">"set1_CM/fields/point"&amp;TEXT(A6,"00")&amp;"_wv"&amp;TEXT(D6,"0")&amp;"nm_amp"&amp;INT(ROUND(F6*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F6*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set1_CM/fields/point05_wv240nm_amp0.52pct.vtk</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4501,11 +4517,11 @@
         <v>0.52</v>
       </c>
       <c r="G7" s="6" t="n">
-        <f aca="false">C7+F7*IF(E7&gt;=0.75,-1,MIN(0,SIN(2*PI()*E7)))</f>
+        <f aca="false">C7+F7*IF((Notes!$B$4-Notes!$B$6)/D7&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D7)))</f>
         <v>50.43</v>
       </c>
       <c r="H7" s="6" t="n">
-        <f aca="false">C7+F7*IF(E7&gt;=0.25,1,SIN(2*PI()*E7))</f>
+        <f aca="false">C7+F7*IF((Notes!$B$4-Notes!$B$6)/D7&gt;=0.25,1,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D7))</f>
         <v>51.47</v>
       </c>
       <c r="I7" s="2" t="n">
@@ -4549,8 +4565,8 @@
       <c r="X7" s="14"/>
       <c r="Y7" s="15"/>
       <c r="Z7" s="16" t="str">
-        <f aca="false">"set1_pt"&amp;A7&amp;".vtk"</f>
-        <v>set1_pt6.vtk</v>
+        <f aca="false">"set1_CM/fields/point"&amp;TEXT(A7,"00")&amp;"_wv"&amp;TEXT(D7,"0")&amp;"nm_amp"&amp;INT(ROUND(F7*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F7*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set1_CM/fields/point06_wv320nm_amp0.52pct.vtk</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4572,11 +4588,11 @@
         <v>0.4</v>
       </c>
       <c r="G8" s="6" t="n">
-        <f aca="false">C8+F8*IF(E8&gt;=0.75,-1,MIN(0,SIN(2*PI()*E8)))</f>
+        <f aca="false">C8+F8*IF((Notes!$B$4-Notes!$B$6)/D8&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D8)))</f>
         <v>50.6</v>
       </c>
       <c r="H8" s="6" t="n">
-        <f aca="false">C8+F8*IF(E8&gt;=0.25,1,SIN(2*PI()*E8))</f>
+        <f aca="false">C8+F8*IF((Notes!$B$4-Notes!$B$6)/D8&gt;=0.25,1,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D8))</f>
         <v>51.4</v>
       </c>
       <c r="I8" s="2" t="n">
@@ -4620,8 +4636,8 @@
       <c r="X8" s="14"/>
       <c r="Y8" s="15"/>
       <c r="Z8" s="16" t="str">
-        <f aca="false">"set1_pt"&amp;A8&amp;".vtk"</f>
-        <v>set1_pt7.vtk</v>
+        <f aca="false">"set1_CM/fields/point"&amp;TEXT(A8,"00")&amp;"_wv"&amp;TEXT(D8,"0")&amp;"nm_amp"&amp;INT(ROUND(F8*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F8*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set1_CM/fields/point07_wv240nm_amp0.40pct.vtk</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4643,11 +4659,11 @@
         <v>0.48</v>
       </c>
       <c r="G9" s="6" t="n">
-        <f aca="false">C9+F9*IF(E9&gt;=0.75,-1,MIN(0,SIN(2*PI()*E9)))</f>
+        <f aca="false">C9+F9*IF((Notes!$B$4-Notes!$B$6)/D9&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D9)))</f>
         <v>50.47</v>
       </c>
       <c r="H9" s="6" t="n">
-        <f aca="false">C9+F9*IF(E9&gt;=0.25,1,SIN(2*PI()*E9))</f>
+        <f aca="false">C9+F9*IF((Notes!$B$4-Notes!$B$6)/D9&gt;=0.25,1,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D9))</f>
         <v>51.43</v>
       </c>
       <c r="I9" s="2" t="n">
@@ -4691,8 +4707,8 @@
       <c r="X9" s="14"/>
       <c r="Y9" s="15"/>
       <c r="Z9" s="16" t="str">
-        <f aca="false">"set1_pt"&amp;A9&amp;".vtk"</f>
-        <v>set1_pt8.vtk</v>
+        <f aca="false">"set1_CM/fields/point"&amp;TEXT(A9,"00")&amp;"_wv"&amp;TEXT(D9,"0")&amp;"nm_amp"&amp;INT(ROUND(F9*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F9*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set1_CM/fields/point08_wv240nm_amp0.48pct.vtk</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4714,11 +4730,11 @@
         <v>0.48</v>
       </c>
       <c r="G10" s="6" t="n">
-        <f aca="false">C10+F10*IF(E10&gt;=0.75,-1,MIN(0,SIN(2*PI()*E10)))</f>
+        <f aca="false">C10+F10*IF((Notes!$B$4-Notes!$B$6)/D10&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D10)))</f>
         <v>50.52</v>
       </c>
       <c r="H10" s="6" t="n">
-        <f aca="false">C10+F10*IF(E10&gt;=0.25,1,SIN(2*PI()*E10))</f>
+        <f aca="false">C10+F10*IF((Notes!$B$4-Notes!$B$6)/D10&gt;=0.25,1,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D10))</f>
         <v>51.48</v>
       </c>
       <c r="I10" s="2" t="n">
@@ -4762,8 +4778,8 @@
       <c r="X10" s="14"/>
       <c r="Y10" s="15"/>
       <c r="Z10" s="16" t="str">
-        <f aca="false">"set1_pt"&amp;A10&amp;".vtk"</f>
-        <v>set1_pt9.vtk</v>
+        <f aca="false">"set1_CM/fields/point"&amp;TEXT(A10,"00")&amp;"_wv"&amp;TEXT(D10,"0")&amp;"nm_amp"&amp;INT(ROUND(F10*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F10*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set1_CM/fields/point09_wv160nm_amp0.48pct.vtk</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4785,11 +4801,11 @@
         <v>0.44</v>
       </c>
       <c r="G11" s="6" t="n">
-        <f aca="false">C11+F11*IF(E11&gt;=0.75,-1,MIN(0,SIN(2*PI()*E11)))</f>
+        <f aca="false">C11+F11*IF((Notes!$B$4-Notes!$B$6)/D11&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D11)))</f>
         <v>50.56</v>
       </c>
       <c r="H11" s="6" t="n">
-        <f aca="false">C11+F11*IF(E11&gt;=0.25,1,SIN(2*PI()*E11))</f>
+        <f aca="false">C11+F11*IF((Notes!$B$4-Notes!$B$6)/D11&gt;=0.25,1,SIN(2*PI()*(Notes!$B$4-Notes!$B$6)/D11))</f>
         <v>51.44</v>
       </c>
       <c r="I11" s="2" t="n">
@@ -4833,8 +4849,8 @@
       <c r="X11" s="14"/>
       <c r="Y11" s="15"/>
       <c r="Z11" s="16" t="str">
-        <f aca="false">"set1_pt"&amp;A11&amp;".vtk"</f>
-        <v>set1_pt10.vtk</v>
+        <f aca="false">"set1_CM/fields/point"&amp;TEXT(A11,"00")&amp;"_wv"&amp;TEXT(D11,"0")&amp;"nm_amp"&amp;INT(ROUND(F11*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F11*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set1_CM/fields/point10_wv160nm_amp0.44pct.vtk</v>
       </c>
     </row>
   </sheetData>
@@ -4875,7 +4891,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="22" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4978,11 +4994,11 @@
         <v>0.88</v>
       </c>
       <c r="G2" s="6" t="n">
-        <f aca="false">C2+F2*IF(E2&gt;=0.75,-1,MIN(0,SIN(2*PI()*E2)))</f>
+        <f aca="false">C2+F2*IF((Notes!$B$5-Notes!$B$7)/D2&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D2)))</f>
         <v>49.67</v>
       </c>
       <c r="H2" s="6" t="n">
-        <f aca="false">C2+F2*IF(E2&gt;=0.25,1,SIN(2*PI()*E2))</f>
+        <f aca="false">C2+F2*IF((Notes!$B$5-Notes!$B$7)/D2&gt;=0.25,1,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D2))</f>
         <v>51.43</v>
       </c>
       <c r="I2" s="2" t="n">
@@ -5026,8 +5042,8 @@
       <c r="X2" s="14"/>
       <c r="Y2" s="15"/>
       <c r="Z2" s="16" t="str">
-        <f aca="false">"set2_pt"&amp;A2&amp;".vtk"</f>
-        <v>set2_pt1.vtk</v>
+        <f aca="false">"set2_CM/fields/point"&amp;TEXT(A2,"00")&amp;"_wv"&amp;TEXT(D2,"0")&amp;"nm_amp"&amp;INT(ROUND(F2*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F2*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set2_CM/fields/point01_wv80nm_amp0.88pct.vtk</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5049,11 +5065,11 @@
         <v>0.92</v>
       </c>
       <c r="G3" s="6" t="n">
-        <f aca="false">C3+F3*IF(E3&gt;=0.75,-1,MIN(0,SIN(2*PI()*E3)))</f>
+        <f aca="false">C3+F3*IF((Notes!$B$5-Notes!$B$7)/D3&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D3)))</f>
         <v>49.63</v>
       </c>
       <c r="H3" s="6" t="n">
-        <f aca="false">C3+F3*IF(E3&gt;=0.25,1,SIN(2*PI()*E3))</f>
+        <f aca="false">C3+F3*IF((Notes!$B$5-Notes!$B$7)/D3&gt;=0.25,1,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D3))</f>
         <v>51.47</v>
       </c>
       <c r="I3" s="2" t="n">
@@ -5097,8 +5113,8 @@
       <c r="X3" s="14"/>
       <c r="Y3" s="15"/>
       <c r="Z3" s="16" t="str">
-        <f aca="false">"set2_pt"&amp;A3&amp;".vtk"</f>
-        <v>set2_pt2.vtk</v>
+        <f aca="false">"set2_CM/fields/point"&amp;TEXT(A3,"00")&amp;"_wv"&amp;TEXT(D3,"0")&amp;"nm_amp"&amp;INT(ROUND(F3*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F3*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set2_CM/fields/point02_wv320nm_amp0.92pct.vtk</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5120,11 +5136,11 @@
         <v>0.8</v>
       </c>
       <c r="G4" s="6" t="n">
-        <f aca="false">C4+F4*IF(E4&gt;=0.75,-1,MIN(0,SIN(2*PI()*E4)))</f>
+        <f aca="false">C4+F4*IF((Notes!$B$5-Notes!$B$7)/D4&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D4)))</f>
         <v>49.75</v>
       </c>
       <c r="H4" s="6" t="n">
-        <f aca="false">C4+F4*IF(E4&gt;=0.25,1,SIN(2*PI()*E4))</f>
+        <f aca="false">C4+F4*IF((Notes!$B$5-Notes!$B$7)/D4&gt;=0.25,1,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D4))</f>
         <v>51.35</v>
       </c>
       <c r="I4" s="2" t="n">
@@ -5168,8 +5184,8 @@
       <c r="X4" s="14"/>
       <c r="Y4" s="15"/>
       <c r="Z4" s="16" t="str">
-        <f aca="false">"set2_pt"&amp;A4&amp;".vtk"</f>
-        <v>set2_pt3.vtk</v>
+        <f aca="false">"set2_CM/fields/point"&amp;TEXT(A4,"00")&amp;"_wv"&amp;TEXT(D4,"0")&amp;"nm_amp"&amp;INT(ROUND(F4*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F4*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set2_CM/fields/point03_wv240nm_amp0.80pct.vtk</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5191,11 +5207,11 @@
         <v>1</v>
       </c>
       <c r="G5" s="6" t="n">
-        <f aca="false">C5+F5*IF(E5&gt;=0.75,-1,MIN(0,SIN(2*PI()*E5)))</f>
+        <f aca="false">C5+F5*IF((Notes!$B$5-Notes!$B$7)/D5&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D5)))</f>
         <v>49.55</v>
       </c>
       <c r="H5" s="6" t="n">
-        <f aca="false">C5+F5*IF(E5&gt;=0.25,1,SIN(2*PI()*E5))</f>
+        <f aca="false">C5+F5*IF((Notes!$B$5-Notes!$B$7)/D5&gt;=0.25,1,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D5))</f>
         <v>51.55</v>
       </c>
       <c r="I5" s="2" t="n">
@@ -5239,8 +5255,8 @@
       <c r="X5" s="14"/>
       <c r="Y5" s="15"/>
       <c r="Z5" s="16" t="str">
-        <f aca="false">"set2_pt"&amp;A5&amp;".vtk"</f>
-        <v>set2_pt4.vtk</v>
+        <f aca="false">"set2_CM/fields/point"&amp;TEXT(A5,"00")&amp;"_wv"&amp;TEXT(D5,"0")&amp;"nm_amp"&amp;INT(ROUND(F5*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F5*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set2_CM/fields/point04_wv640nm_amp1.00pct.vtk</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5262,11 +5278,11 @@
         <v>0.92</v>
       </c>
       <c r="G6" s="6" t="n">
-        <f aca="false">C6+F6*IF(E6&gt;=0.75,-1,MIN(0,SIN(2*PI()*E6)))</f>
+        <f aca="false">C6+F6*IF((Notes!$B$5-Notes!$B$7)/D6&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D6)))</f>
         <v>49.63</v>
       </c>
       <c r="H6" s="6" t="n">
-        <f aca="false">C6+F6*IF(E6&gt;=0.25,1,SIN(2*PI()*E6))</f>
+        <f aca="false">C6+F6*IF((Notes!$B$5-Notes!$B$7)/D6&gt;=0.25,1,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D6))</f>
         <v>51.47</v>
       </c>
       <c r="I6" s="2" t="n">
@@ -5310,8 +5326,8 @@
       <c r="X6" s="14"/>
       <c r="Y6" s="15"/>
       <c r="Z6" s="16" t="str">
-        <f aca="false">"set2_pt"&amp;A6&amp;".vtk"</f>
-        <v>set2_pt5.vtk</v>
+        <f aca="false">"set2_CM/fields/point"&amp;TEXT(A6,"00")&amp;"_wv"&amp;TEXT(D6,"0")&amp;"nm_amp"&amp;INT(ROUND(F6*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F6*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set2_CM/fields/point05_wv480nm_amp0.92pct.vtk</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5333,11 +5349,11 @@
         <v>0.8</v>
       </c>
       <c r="G7" s="6" t="n">
-        <f aca="false">C7+F7*IF(E7&gt;=0.75,-1,MIN(0,SIN(2*PI()*E7)))</f>
+        <f aca="false">C7+F7*IF((Notes!$B$5-Notes!$B$7)/D7&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D7)))</f>
         <v>49.75</v>
       </c>
       <c r="H7" s="6" t="n">
-        <f aca="false">C7+F7*IF(E7&gt;=0.25,1,SIN(2*PI()*E7))</f>
+        <f aca="false">C7+F7*IF((Notes!$B$5-Notes!$B$7)/D7&gt;=0.25,1,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D7))</f>
         <v>51.35</v>
       </c>
       <c r="I7" s="2" t="n">
@@ -5381,8 +5397,8 @@
       <c r="X7" s="14"/>
       <c r="Y7" s="15"/>
       <c r="Z7" s="16" t="str">
-        <f aca="false">"set2_pt"&amp;A7&amp;".vtk"</f>
-        <v>set2_pt6.vtk</v>
+        <f aca="false">"set2_CM/fields/point"&amp;TEXT(A7,"00")&amp;"_wv"&amp;TEXT(D7,"0")&amp;"nm_amp"&amp;INT(ROUND(F7*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F7*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set2_CM/fields/point06_wv640nm_amp0.80pct.vtk</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5404,11 +5420,11 @@
         <v>0.68</v>
       </c>
       <c r="G8" s="6" t="n">
-        <f aca="false">C8+F8*IF(E8&gt;=0.75,-1,MIN(0,SIN(2*PI()*E8)))</f>
+        <f aca="false">C8+F8*IF((Notes!$B$5-Notes!$B$7)/D8&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D8)))</f>
         <v>50.55</v>
       </c>
       <c r="H8" s="6" t="n">
-        <f aca="false">C8+F8*IF(E8&gt;=0.25,1,SIN(2*PI()*E8))</f>
+        <f aca="false">C8+F8*IF((Notes!$B$5-Notes!$B$7)/D8&gt;=0.25,1,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D8))</f>
         <v>51.23</v>
       </c>
       <c r="I8" s="2" t="n">
@@ -5452,8 +5468,8 @@
       <c r="X8" s="14"/>
       <c r="Y8" s="15"/>
       <c r="Z8" s="16" t="str">
-        <f aca="false">"set2_pt"&amp;A8&amp;".vtk"</f>
-        <v>set2_pt7.vtk</v>
+        <f aca="false">"set2_CM/fields/point"&amp;TEXT(A8,"00")&amp;"_wv"&amp;TEXT(D8,"0")&amp;"nm_amp"&amp;INT(ROUND(F8*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F8*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set2_CM/fields/point07_wv1280nm_amp0.68pct.vtk</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5475,11 +5491,11 @@
         <v>0.56</v>
       </c>
       <c r="G9" s="6" t="n">
-        <f aca="false">C9+F9*IF(E9&gt;=0.75,-1,MIN(0,SIN(2*PI()*E9)))</f>
-        <v>50.1786513113852</v>
+        <f aca="false">C9+F9*IF((Notes!$B$5-Notes!$B$7)/D9&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D9)))</f>
+        <v>50.179919204589</v>
       </c>
       <c r="H9" s="6" t="n">
-        <f aca="false">C9+F9*IF(E9&gt;=0.25,1,SIN(2*PI()*E9))</f>
+        <f aca="false">C9+F9*IF((Notes!$B$5-Notes!$B$7)/D9&gt;=0.25,1,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D9))</f>
         <v>51.11</v>
       </c>
       <c r="I9" s="2" t="n">
@@ -5523,8 +5539,8 @@
       <c r="X9" s="14"/>
       <c r="Y9" s="15"/>
       <c r="Z9" s="16" t="str">
-        <f aca="false">"set2_pt"&amp;A9&amp;".vtk"</f>
-        <v>set2_pt8.vtk</v>
+        <f aca="false">"set2_CM/fields/point"&amp;TEXT(A9,"00")&amp;"_wv"&amp;TEXT(D9,"0")&amp;"nm_amp"&amp;INT(ROUND(F9*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F9*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set2_CM/fields/point08_wv1040nm_amp0.56pct.vtk</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5546,11 +5562,11 @@
         <v>0.6</v>
       </c>
       <c r="G10" s="6" t="n">
-        <f aca="false">C10+F10*IF(E10&gt;=0.75,-1,MIN(0,SIN(2*PI()*E10)))</f>
+        <f aca="false">C10+F10*IF((Notes!$B$5-Notes!$B$7)/D10&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D10)))</f>
         <v>49.95</v>
       </c>
       <c r="H10" s="6" t="n">
-        <f aca="false">C10+F10*IF(E10&gt;=0.25,1,SIN(2*PI()*E10))</f>
+        <f aca="false">C10+F10*IF((Notes!$B$5-Notes!$B$7)/D10&gt;=0.25,1,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D10))</f>
         <v>51.15</v>
       </c>
       <c r="I10" s="2" t="n">
@@ -5594,8 +5610,8 @@
       <c r="X10" s="14"/>
       <c r="Y10" s="15"/>
       <c r="Z10" s="16" t="str">
-        <f aca="false">"set2_pt"&amp;A10&amp;".vtk"</f>
-        <v>set2_pt9.vtk</v>
+        <f aca="false">"set2_CM/fields/point"&amp;TEXT(A10,"00")&amp;"_wv"&amp;TEXT(D10,"0")&amp;"nm_amp"&amp;INT(ROUND(F10*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F10*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set2_CM/fields/point09_wv720nm_amp0.60pct.vtk</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5617,11 +5633,11 @@
         <v>0.04</v>
       </c>
       <c r="G11" s="6" t="n">
-        <f aca="false">C11+F11*IF(E11&gt;=0.75,-1,MIN(0,SIN(2*PI()*E11)))</f>
+        <f aca="false">C11+F11*IF((Notes!$B$5-Notes!$B$7)/D11&gt;=0.75,-1,MIN(0,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D11)))</f>
         <v>50.51</v>
       </c>
       <c r="H11" s="6" t="n">
-        <f aca="false">C11+F11*IF(E11&gt;=0.25,1,SIN(2*PI()*E11))</f>
+        <f aca="false">C11+F11*IF((Notes!$B$5-Notes!$B$7)/D11&gt;=0.25,1,SIN(2*PI()*(Notes!$B$5-Notes!$B$7)/D11))</f>
         <v>50.59</v>
       </c>
       <c r="I11" s="2" t="n">
@@ -5665,8 +5681,8 @@
       <c r="X11" s="14"/>
       <c r="Y11" s="15"/>
       <c r="Z11" s="16" t="str">
-        <f aca="false">"set2_pt"&amp;A11&amp;".vtk"</f>
-        <v>set2_pt10.vtk</v>
+        <f aca="false">"set2_CM/fields/point"&amp;TEXT(A11,"00")&amp;"_wv"&amp;TEXT(D11,"0")&amp;"nm_amp"&amp;INT(ROUND(F11*100,0)/100)&amp;"."&amp;TEXT(MOD(ROUND(F11*100,0),100),"00")&amp;"pct.vtk"</f>
+        <v>set2_CM/fields/point10_wv720nm_amp0.04pct.vtk</v>
       </c>
     </row>
   </sheetData>
@@ -7664,7 +7680,7 @@
     <tabColor rgb="FF7F7F7F"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -7698,7 +7714,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="33" t="s">
         <v>48</v>
       </c>
@@ -7709,248 +7725,254 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="32" t="s">
+    <row r="6" customFormat="false" ht="57.0" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="33" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="44" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="33" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7" s="44" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C7" s="33" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="32" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="35" t="s">
+    <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="33" t="s">
+      <c r="C10" s="33" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="36" t="s">
+    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C11" s="33" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="37" t="s">
+    <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="37" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C12" s="33" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="38" t="s">
+    <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="C11" s="33" t="s">
+      <c r="C13" s="33" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="33" t="s">
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="33" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="33" t="s">
+      <c r="C14" s="33" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="32" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="32" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="39" t="s">
+    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="C15" s="33" t="s">
+      <c r="C17" s="33" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="39" t="s">
+    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="39" t="s">
         <v>64</v>
       </c>
-      <c r="C16" s="33" t="s">
+      <c r="C18" s="33" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="39" t="s">
+    <row r="19" customFormat="false" ht="97.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="39" t="s">
         <v>66</v>
       </c>
-      <c r="C17" s="33" t="s">
+      <c r="C19" s="33" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="39" t="s">
+    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="C18" s="33" t="s">
+      <c r="C20" s="33" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="39" t="s">
+    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="C19" s="33" t="s">
+      <c r="C21" s="33" t="s">
         <v>71</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="39" t="s">
-        <v>72</v>
-      </c>
-      <c r="C20" s="33" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="39" t="s">
-        <v>18</v>
-      </c>
-      <c r="C21" s="33" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="39" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" s="33" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="33" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="33" t="s">
+      <c r="C24" s="33" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="39" t="s">
+    <row r="25" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="33" t="s">
+      <c r="C25" s="33" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="39" t="s">
+    <row r="26" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="39" t="s">
         <v>77</v>
       </c>
-      <c r="C24" s="33" t="s">
+      <c r="C26" s="33" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="39" t="s">
+    <row r="27" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="39" t="s">
         <v>79</v>
       </c>
-      <c r="C25" s="33" t="s">
+      <c r="C27" s="33" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="39" t="s">
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C26" s="33" t="s">
+      <c r="C28" s="33" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="32" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="32" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="33" t="s">
+    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="33" t="s">
         <v>83</v>
       </c>
-      <c r="C29" s="33" t="s">
+      <c r="C31" s="33" t="s">
         <v>84</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="33" t="s">
-        <v>8</v>
-      </c>
-      <c r="B30" s="40" t="n">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="B31" s="40" t="n">
-        <v>796</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="33" t="s">
-        <v>14</v>
-      </c>
-      <c r="B32" s="41" t="n">
-        <v>4.95</v>
+        <v>8</v>
+      </c>
+      <c r="B32" s="40" t="n">
+        <v>572</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="B33" s="41" t="n">
-        <v>5.57</v>
+        <v>11</v>
+      </c>
+      <c r="B33" s="40" t="n">
+        <v>796</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="33" t="s">
-        <v>20</v>
-      </c>
-      <c r="B34" s="42" t="n">
-        <v>0.931</v>
+        <v>14</v>
+      </c>
+      <c r="B34" s="41" t="n">
+        <v>4.95</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="B35" s="42" t="n">
-        <v>0.618</v>
+        <v>17</v>
+      </c>
+      <c r="B35" s="41" t="n">
+        <v>5.57</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" s="42" t="n">
+        <v>0.931</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="B37" s="42" t="n">
+        <v>0.618</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="B36" s="43" t="n">
+      <c r="B38" s="43" t="n">
         <v>0.000178</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="32" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="32" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="33" t="s">
-        <v>86</v>
-      </c>
-      <c r="C39" s="33" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="33" t="s">
-        <v>86</v>
-      </c>
-      <c r="C40" s="33" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="33" t="s">
         <v>86</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7958,6 +7980,22 @@
         <v>86</v>
       </c>
       <c r="C42" s="33" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="33" t="s">
+        <v>86</v>
+      </c>
+      <c r="C43" s="33" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="33" t="s">
+        <v>86</v>
+      </c>
+      <c r="C44" s="33" t="s">
         <v>90</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Set 1 pseudo-2D and Set 1 2D vs 3D tabs with one-period check
Pseudo-2D tab: run plan (cell length along the CM, 10-unit thin axis, periods in
cell with a >=1 check, survey-sweep window and fine-sweep step count) plus blank
2D result columns. 2D vs 3D tab: ML / 3D / 2D / delta blocks and Pearson r for
2D vs 3D, ML vs 2D and ML vs 3D, all linked. Charts gains four 2D vs 3D plots.
The waves columns on the Set sheets turn red below one period.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011WnE18kmcTTQHQwwBdKitt
</commit_message>
<xml_diff>
--- a/CM_Sweep_Sets_1_2.xlsx
+++ b/CM_Sweep_Sets_1_2.xlsx
@@ -11,8 +11,10 @@
     <sheet name="Set 1" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Set 2" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Combined" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Charts" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Notes" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Set 1 2D vs 3D" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Set 1 pseudo-2D" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Charts" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Notes" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -61,7 +63,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">= L / lambda, where L is the domain length set on the Notes sheet (cell B4 for Set 1, B5 for Set 2).</t>
+          <t xml:space="preserve">= L / lambda, where L is the domain length set on the Notes sheet (cell B4 for Set 1, B5 for Set 2). Turns red below 1: the cell then holds less than one full period of the CM.</t>
         </r>
       </text>
     </comment>
@@ -239,7 +241,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">= L / lambda, where L is the domain length set on the Notes sheet (cell B4 for Set 1, B5 for Set 2).</t>
+          <t xml:space="preserve">= L / lambda, where L is the domain length set on the Notes sheet (cell B4 for Set 1, B5 for Set 2). Turns red below 1: the cell then holds less than one full period of the CM.</t>
         </r>
       </text>
     </comment>
@@ -379,8 +381,184 @@
 </comments>
 </file>
 
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">2D = pseudo-2D sweep (Set 1 pseudo-2D tab). 3D = the regular 3D sweep (SIM columns of the Set 1 tab). Δ = 2D − 3D.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">2D = pseudo-2D sweep (Set 1 pseudo-2D tab). 3D = the regular 3D sweep (SIM columns of the Set 1 tab). Δ = 2D − 3D.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">2D = pseudo-2D sweep (Set 1 pseudo-2D tab). 3D = the regular 3D sweep (SIM columns of the Set 1 tab). Δ = 2D − 3D.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">2D = pseudo-2D sweep (Set 1 pseudo-2D tab). 3D = the regular 3D sweep (SIM columns of the Set 1 tab). Δ = 2D − 3D.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="E1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Input: simulation-cell length along the CM direction. Default is 640 (the Set 1 cell), raised to λ where λ &gt; 640 so that at least one full period fits. Overwrite with the real cell length.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">From Notes!B6: the pseudo-2D cell is 10 units thick in the thin direction. Confirm which axis that is: sine.m modulates along y.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">= cell length ÷ λ. Red below 1.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">OK when the cell holds at least one full period of the CM wavelength.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Information only. With periodic boundaries a non-integer number of periods leaves a seam where the sine does not meet itself.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Survey sweep: coarse stress steps to find where the transformation happens. Enter where the transformation window starts.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Where the transformation window ends, from the survey sweep.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Stress step for the fine sweep inside the window. 10 MPa is the value Report 2 used; edit as needed.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">= ROUNDUP((end − start) ÷ step) + 1. Blank until the window is entered.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="143">
   <si>
     <t xml:space="preserve">Point</t>
   </si>
@@ -505,12 +683,135 @@
     <t xml:space="preserve">Loop area</t>
   </si>
   <si>
+    <t xml:space="preserve">3D V1 stress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2D V1 stress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ V1 stress (2D−3D)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3D V3 stress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2D V3 stress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ V3 stress (2D−3D)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ML Strain range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3D Strain range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2D Strain range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ Strain range (2D−3D)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ML Loop area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3D Loop area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2D Loop area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ Loop area (2D−3D)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3D max vf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2D max vf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ max vf (2D−3D)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pearson r (blank until at least 3 paired points)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n 2D–3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">r 2D vs 3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n ML–2D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">r ML vs 2D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n ML–3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">r ML vs 3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cell length along CM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thin axis length (units)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Periods in cell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-period check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integer periods?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Survey window start (MPa)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Survey window end (MPa)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fine step (MPa)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fine sweep steps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sweep status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2D strain range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2D loop area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2D cliff Δvf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2D residual strain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2D notes</t>
+  </si>
+  <si>
     <t xml:space="preserve">ML vs SIM scatter plots</t>
   </si>
   <si>
     <t xml:space="preserve">Points appear as SIM values are filled in on the Set sheets. Stress-strain curves will be added once the raw cycle data is available.</t>
   </si>
   <si>
+    <t xml:space="preserve">Pseudo-2D vs 3D (Set 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3D = the regular 3D sweep (SIM columns on the Set 1 tab); 2D = the pseudo-2D sweep. Points appear as both are filled in.</t>
+  </si>
+  <si>
     <t xml:space="preserve">CM sweep, Sets 1 and 2: notes, assumptions and legend</t>
   </si>
   <si>
@@ -523,13 +824,19 @@
     <t xml:space="preserve">Set 1 domain length L (nm)</t>
   </si>
   <si>
-    <t xml:space="preserve">Assumption: taken from the 'waves / 640 nm' header in Aum's 2D sweep sheet; the Set 1 renders agree (stripe count = 640/λ).</t>
+    <t xml:space="preserve">Assumption: taken from the 'waves / 640 nm' header in Aum's 2D sweep sheet; the Set 1 renders agree (stripe count = 640/λ). Point 2 (λ = 960) holds only 0.67 periods at 640, so it breaks the one-period rule: it needs a cell of at least 960.</t>
   </si>
   <si>
     <t xml:space="preserve">Set 2 domain length L (nm)</t>
   </si>
   <si>
-    <t xml:space="preserve">Assumption: set to 640 because all 10 Set 2 renders show 640/λ waves (e.g. λ = 640 shows one wave, λ = 80 shows eight). sine.m (Ny = 1280, wv = 1280 for set2_pt7) points to 1280 instead, so the two disagree. Confirm which grid set 2 used; changing this cell updates waves, c min and c max.</t>
+    <t xml:space="preserve">Assumption: set to 640 because all 10 Set 2 renders show 640/λ waves. At 640, points 7–10 hold fewer than one period (0.50, 0.62, 0.89, 0.89), which breaks the one-period rule; a 1280 cell fits all ten. sine.m also uses 1280 (Ny = 1280, wv = 1280 for set2_pt7), so the renders and the code disagree. Confirm which cell the Set 2 runs used; changing this cell updates waves, c min and c max.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pseudo-2D thin axis (units)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From your note: the pseudo-2D cell is 10 units thick. Confirm which axis is thinned: sine.m modulates along y, so if y is the thin axis the CM has to run along x or z.</t>
   </si>
   <si>
     <t xml:space="preserve">Legend</t>
@@ -595,7 +902,7 @@
     <t xml:space="preserve">SIM columns</t>
   </si>
   <si>
-    <t xml:space="preserve">Blank. To be filled from the 3D phase-field cycles. Exact definitions (V1/V3 transformation stress, loop area, max vf, cliff Δvf, residual strain) to be confirmed against the post-processing scripts.</t>
+    <t xml:space="preserve">Blank. To be filled from the 3D phase-field cycles (the regular 3D sweep, which the 2D vs 3D sheet reads). Exact definitions (V1/V3 transformation stress, loop area, max vf, cliff Δvf, residual strain) to be confirmed against the post-processing scripts.</t>
   </si>
   <si>
     <t xml:space="preserve">Δ V1, Δ V3, Δ strain (pp)</t>
@@ -625,6 +932,24 @@
     <t xml:space="preserve">Scatter plots of ML (x) against SIM (y) for V1, V3, strain range and loop area, one series per set. They read the Set sheets directly, so points appear as SIM values are filled in. Stress-strain curves are not here yet; they need the raw cycle data.</t>
   </si>
   <si>
+    <t xml:space="preserve">One-period rule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The simulation cell must hold at least one full period of the CM wavelength along the modulation direction (cell length ≥ λ). The waves column on the Set sheets, and Periods in cell on the pseudo-2D sheet, turn red below 1. A non-integer number of periods also leaves a seam under periodic boundaries (the PBC line in sine.m forces the last plane to avg); the pseudo-2D sheet shows this as information only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set 1 pseudo-2D sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run plan and results for the pseudo-2D sweep of the 10 Set 1 points. Procedure: (1) make the thin axis 10 units and the cell at least one period long; (2) run a coarse survey sweep and enter the transformation window; (3) run the fine sweep inside that window at the step shown (10 MPa, as in Report 2); (4) enter the results in the yellow 2D columns. Default cell length is 640 (the Set 1 cell), raised to 960 for point 2 so that one period fits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set 1 2D vs 3D sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compares the pseudo-2D results (2D) with the regular 3D sweep (the SIM columns on the Set 1 tab) and with the Shanghai ML values. Every cell is a link. Δ = 2D − 3D. The table under it gives Pearson r for 2D vs 3D, ML vs 2D and ML vs 3D; it needs at least 3 paired points. The Charts tab plots 2D against 3D.</t>
+  </si>
+  <si>
     <t xml:space="preserve">ParaView renders from VTK_Field_Report.xlsx, one per point. They appear to be auto-scaled to each field's own range, so amplitude differences between points are not visible.</t>
   </si>
   <si>
@@ -652,7 +977,16 @@
     <t xml:space="preserve">Confirm the domain lengths above and the .vtk naming.</t>
   </si>
   <si>
-    <t xml:space="preserve">Stress-strain curves and any 2D / pseudo-2D comparison tabs are not built: they need the raw cycle data and 2D results.</t>
+    <t xml:space="preserve">Confirm which axis is the thin (10-unit) one. sine.m modulates along y, so in the pseudo-2D cell the CM must run along a different axis.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-period rule: Set 1 point 2 (960 nm) needs a cell of at least 960, but its existing 3D run used 640 (0.67 periods). A like-for-like 2D vs 3D comparison for that point needs a 3D run in a cell of at least 960.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-period rule: Set 2 points 7–10 break it in a 640 cell. Confirm the cell the Set 2 runs used.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stress-strain curves and the Raw data tabs are not built: they need the raw cycle data.</t>
   </si>
 </sst>
 </file>
@@ -1029,6 +1363,22 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <color rgb="FF9C0006"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -1039,10 +1389,10 @@
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF9C0006"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF548235"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFBFBFBF"/>
@@ -1070,7 +1420,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFFC7CE"/>
       <rgbColor rgb="FF2E75B6"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -1348,11 +1698,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="78884795"/>
-        <c:axId val="7905892"/>
+        <c:axId val="38986248"/>
+        <c:axId val="64274837"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="78884795"/>
+        <c:axId val="38986248"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1428,12 +1778,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7905892"/>
+        <c:crossAx val="64274837"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="7905892"/>
+        <c:axId val="64274837"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1509,7 +1859,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78884795"/>
+        <c:crossAx val="38986248"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1817,11 +2167,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="37380373"/>
-        <c:axId val="47674793"/>
+        <c:axId val="72562490"/>
+        <c:axId val="23694930"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="37380373"/>
+        <c:axId val="72562490"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1897,12 +2247,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47674793"/>
+        <c:crossAx val="23694930"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="47674793"/>
+        <c:axId val="23694930"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1978,7 +2328,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37380373"/>
+        <c:crossAx val="72562490"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2286,11 +2636,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="51108273"/>
-        <c:axId val="66932665"/>
+        <c:axId val="8290263"/>
+        <c:axId val="87717462"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="51108273"/>
+        <c:axId val="8290263"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2366,12 +2716,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66932665"/>
+        <c:crossAx val="87717462"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="66932665"/>
+        <c:axId val="87717462"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2447,7 +2797,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51108273"/>
+        <c:crossAx val="8290263"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2755,11 +3105,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="52103404"/>
-        <c:axId val="47569270"/>
+        <c:axId val="69833587"/>
+        <c:axId val="42185557"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="52103404"/>
+        <c:axId val="69833587"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2835,12 +3185,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47569270"/>
+        <c:crossAx val="42185557"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="47569270"/>
+        <c:axId val="42185557"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2916,7 +3266,1339 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52103404"/>
+        <c:crossAx val="69833587"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>V1 stress: 2D vs 3D</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Set 1"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Set 1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="1f3864"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1f3864"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Set 1'!$J$2:$J$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Set 1 pseudo-2D'!$O$2:$O$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:axId val="50465810"/>
+        <c:axId val="50372058"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="50465810"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>3D V1 stress</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50372058"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="50372058"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>2D V1 stress</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50465810"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>V3 stress: 2D vs 3D</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Set 1"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Set 1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="1f3864"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1f3864"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Set 1'!$M$2:$M$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Set 1 pseudo-2D'!$P$2:$P$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:axId val="66534308"/>
+        <c:axId val="28674830"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="66534308"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>3D V3 stress</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="28674830"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="28674830"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>2D V3 stress</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="66534308"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Strain range: 2D vs 3D</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Set 1"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Set 1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="1f3864"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1f3864"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Set 1'!$P$2:$P$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Set 1 pseudo-2D'!$Q$2:$Q$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:axId val="74024720"/>
+        <c:axId val="76240116"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="74024720"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>3D strain range</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="76240116"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="76240116"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>2D strain range</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="74024720"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Loop area: 2D vs 3D</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Set 1"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Set 1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="1f3864"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1f3864"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Set 1'!$S$2:$S$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Set 1 pseudo-2D'!$R$2:$R$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:axId val="6394594"/>
+        <c:axId val="93832438"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="6394594"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>3D loop area</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="93832438"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="93832438"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>2D loop area</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="6394594"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3840,6 +5522,126 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>4680</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>170640</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="24" name="Chart 5"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="9334440"/>
+        <a:ext cx="6119640" cy="3599640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>4320</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>170640</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="25" name="Chart 6"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="6114960" y="9334440"/>
+        <a:ext cx="6119640" cy="3599640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>4680</xdr:colOff>
+      <xdr:row>89</xdr:row>
+      <xdr:rowOff>170640</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="26" name="Chart 7"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="13525560"/>
+        <a:ext cx="6119640" cy="3599640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>4320</xdr:colOff>
+      <xdr:row>89</xdr:row>
+      <xdr:rowOff>170640</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="27" name="Chart 8"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="6114960" y="13525560"/>
+        <a:ext cx="6119640" cy="3599640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -4838,6 +6640,11 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="E2:E11">
+    <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -5670,6 +7477,11 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="E2:E11">
+    <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -7630,26 +9442,1853 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
+    <tabColor rgb="FF548235"/>
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:V19"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="4" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="18" t="n">
+        <f aca="false">'Set 1'!A2</f>
+        <v>1</v>
+      </c>
+      <c r="B2" s="18" t="n">
+        <f aca="false">'Set 1'!D2</f>
+        <v>400</v>
+      </c>
+      <c r="C2" s="19" t="n">
+        <f aca="false">'Set 1'!F2</f>
+        <v>0.56</v>
+      </c>
+      <c r="D2" s="18" t="n">
+        <f aca="false">'Set 1'!I2</f>
+        <v>1421.15811288509</v>
+      </c>
+      <c r="E2" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!J2),'Set 1'!J2,"")</f>
+        <v/>
+      </c>
+      <c r="F2" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!O2),'Set 1 pseudo-2D'!O2,"")</f>
+        <v/>
+      </c>
+      <c r="G2" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E2),ISNUMBER(F2)),F2-E2,"")</f>
+        <v/>
+      </c>
+      <c r="H2" s="18" t="n">
+        <f aca="false">'Set 1'!L2</f>
+        <v>1746.44105539347</v>
+      </c>
+      <c r="I2" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!M2),'Set 1'!M2,"")</f>
+        <v/>
+      </c>
+      <c r="J2" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!P2),'Set 1 pseudo-2D'!P2,"")</f>
+        <v/>
+      </c>
+      <c r="K2" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(I2),ISNUMBER(J2)),J2-I2,"")</f>
+        <v/>
+      </c>
+      <c r="L2" s="19" t="n">
+        <f aca="false">'Set 1'!O2</f>
+        <v>7.550116</v>
+      </c>
+      <c r="M2" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!P2),'Set 1'!P2,"")</f>
+        <v/>
+      </c>
+      <c r="N2" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!Q2),'Set 1 pseudo-2D'!Q2,"")</f>
+        <v/>
+      </c>
+      <c r="O2" s="5" t="str">
+        <f aca="false">IF(AND(ISNUMBER(M2),ISNUMBER(N2)),N2-M2,"")</f>
+        <v/>
+      </c>
+      <c r="P2" s="20" t="n">
+        <f aca="false">'Set 1'!R2</f>
+        <v>263.959090135506</v>
+      </c>
+      <c r="Q2" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!S2),'Set 1'!S2,"")</f>
+        <v/>
+      </c>
+      <c r="R2" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R2),'Set 1 pseudo-2D'!R2,"")</f>
+        <v/>
+      </c>
+      <c r="S2" s="11" t="str">
+        <f aca="false">IF(AND(ISNUMBER(Q2),ISNUMBER(R2)),R2-Q2,"")</f>
+        <v/>
+      </c>
+      <c r="T2" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!V2),'Set 1'!V2,"")</f>
+        <v/>
+      </c>
+      <c r="U2" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!S2),'Set 1 pseudo-2D'!S2,"")</f>
+        <v/>
+      </c>
+      <c r="V2" s="6" t="str">
+        <f aca="false">IF(AND(ISNUMBER(T2),ISNUMBER(U2)),U2-T2,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="18" t="n">
+        <f aca="false">'Set 1'!A3</f>
+        <v>2</v>
+      </c>
+      <c r="B3" s="18" t="n">
+        <f aca="false">'Set 1'!D3</f>
+        <v>960</v>
+      </c>
+      <c r="C3" s="19" t="n">
+        <f aca="false">'Set 1'!F3</f>
+        <v>0.52</v>
+      </c>
+      <c r="D3" s="18" t="n">
+        <f aca="false">'Set 1'!I3</f>
+        <v>1380.32366821806</v>
+      </c>
+      <c r="E3" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!J3),'Set 1'!J3,"")</f>
+        <v/>
+      </c>
+      <c r="F3" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!O3),'Set 1 pseudo-2D'!O3,"")</f>
+        <v/>
+      </c>
+      <c r="G3" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E3),ISNUMBER(F3)),F3-E3,"")</f>
+        <v/>
+      </c>
+      <c r="H3" s="18" t="n">
+        <f aca="false">'Set 1'!L3</f>
+        <v>1744.46534440925</v>
+      </c>
+      <c r="I3" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!M3),'Set 1'!M3,"")</f>
+        <v/>
+      </c>
+      <c r="J3" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!P3),'Set 1 pseudo-2D'!P3,"")</f>
+        <v/>
+      </c>
+      <c r="K3" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(I3),ISNUMBER(J3)),J3-I3,"")</f>
+        <v/>
+      </c>
+      <c r="L3" s="19" t="n">
+        <f aca="false">'Set 1'!O3</f>
+        <v>7.61353533333333</v>
+      </c>
+      <c r="M3" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!P3),'Set 1'!P3,"")</f>
+        <v/>
+      </c>
+      <c r="N3" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!Q3),'Set 1 pseudo-2D'!Q3,"")</f>
+        <v/>
+      </c>
+      <c r="O3" s="5" t="str">
+        <f aca="false">IF(AND(ISNUMBER(M3),ISNUMBER(N3)),N3-M3,"")</f>
+        <v/>
+      </c>
+      <c r="P3" s="20" t="n">
+        <f aca="false">'Set 1'!R3</f>
+        <v>543.22722833229</v>
+      </c>
+      <c r="Q3" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!S3),'Set 1'!S3,"")</f>
+        <v/>
+      </c>
+      <c r="R3" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R3),'Set 1 pseudo-2D'!R3,"")</f>
+        <v/>
+      </c>
+      <c r="S3" s="11" t="str">
+        <f aca="false">IF(AND(ISNUMBER(Q3),ISNUMBER(R3)),R3-Q3,"")</f>
+        <v/>
+      </c>
+      <c r="T3" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!V3),'Set 1'!V3,"")</f>
+        <v/>
+      </c>
+      <c r="U3" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!S3),'Set 1 pseudo-2D'!S3,"")</f>
+        <v/>
+      </c>
+      <c r="V3" s="6" t="str">
+        <f aca="false">IF(AND(ISNUMBER(T3),ISNUMBER(U3)),U3-T3,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="18" t="n">
+        <f aca="false">'Set 1'!A4</f>
+        <v>3</v>
+      </c>
+      <c r="B4" s="18" t="n">
+        <f aca="false">'Set 1'!D4</f>
+        <v>480</v>
+      </c>
+      <c r="C4" s="19" t="n">
+        <f aca="false">'Set 1'!F4</f>
+        <v>0.52</v>
+      </c>
+      <c r="D4" s="18" t="n">
+        <f aca="false">'Set 1'!I4</f>
+        <v>1408.29891867377</v>
+      </c>
+      <c r="E4" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!J4),'Set 1'!J4,"")</f>
+        <v/>
+      </c>
+      <c r="F4" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!O4),'Set 1 pseudo-2D'!O4,"")</f>
+        <v/>
+      </c>
+      <c r="G4" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E4),ISNUMBER(F4)),F4-E4,"")</f>
+        <v/>
+      </c>
+      <c r="H4" s="18" t="n">
+        <f aca="false">'Set 1'!L4</f>
+        <v>1745.71301367738</v>
+      </c>
+      <c r="I4" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!M4),'Set 1'!M4,"")</f>
+        <v/>
+      </c>
+      <c r="J4" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!P4),'Set 1 pseudo-2D'!P4,"")</f>
+        <v/>
+      </c>
+      <c r="K4" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(I4),ISNUMBER(J4)),J4-I4,"")</f>
+        <v/>
+      </c>
+      <c r="L4" s="19" t="n">
+        <f aca="false">'Set 1'!O4</f>
+        <v>7.63308399999999</v>
+      </c>
+      <c r="M4" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!P4),'Set 1'!P4,"")</f>
+        <v/>
+      </c>
+      <c r="N4" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!Q4),'Set 1 pseudo-2D'!Q4,"")</f>
+        <v/>
+      </c>
+      <c r="O4" s="5" t="str">
+        <f aca="false">IF(AND(ISNUMBER(M4),ISNUMBER(N4)),N4-M4,"")</f>
+        <v/>
+      </c>
+      <c r="P4" s="20" t="n">
+        <f aca="false">'Set 1'!R4</f>
+        <v>632.07201334017</v>
+      </c>
+      <c r="Q4" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!S4),'Set 1'!S4,"")</f>
+        <v/>
+      </c>
+      <c r="R4" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R4),'Set 1 pseudo-2D'!R4,"")</f>
+        <v/>
+      </c>
+      <c r="S4" s="11" t="str">
+        <f aca="false">IF(AND(ISNUMBER(Q4),ISNUMBER(R4)),R4-Q4,"")</f>
+        <v/>
+      </c>
+      <c r="T4" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!V4),'Set 1'!V4,"")</f>
+        <v/>
+      </c>
+      <c r="U4" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!S4),'Set 1 pseudo-2D'!S4,"")</f>
+        <v/>
+      </c>
+      <c r="V4" s="6" t="str">
+        <f aca="false">IF(AND(ISNUMBER(T4),ISNUMBER(U4)),U4-T4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="n">
+        <f aca="false">'Set 1'!A5</f>
+        <v>4</v>
+      </c>
+      <c r="B5" s="18" t="n">
+        <f aca="false">'Set 1'!D5</f>
+        <v>240</v>
+      </c>
+      <c r="C5" s="19" t="n">
+        <f aca="false">'Set 1'!F5</f>
+        <v>0.52</v>
+      </c>
+      <c r="D5" s="18" t="n">
+        <f aca="false">'Set 1'!I5</f>
+        <v>1409.06706888271</v>
+      </c>
+      <c r="E5" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!J5),'Set 1'!J5,"")</f>
+        <v/>
+      </c>
+      <c r="F5" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!O5),'Set 1 pseudo-2D'!O5,"")</f>
+        <v/>
+      </c>
+      <c r="G5" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E5),ISNUMBER(F5)),F5-E5,"")</f>
+        <v/>
+      </c>
+      <c r="H5" s="18" t="n">
+        <f aca="false">'Set 1'!L5</f>
+        <v>1746.41676186042</v>
+      </c>
+      <c r="I5" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!M5),'Set 1'!M5,"")</f>
+        <v/>
+      </c>
+      <c r="J5" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!P5),'Set 1 pseudo-2D'!P5,"")</f>
+        <v/>
+      </c>
+      <c r="K5" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(I5),ISNUMBER(J5)),J5-I5,"")</f>
+        <v/>
+      </c>
+      <c r="L5" s="19" t="n">
+        <f aca="false">'Set 1'!O5</f>
+        <v>7.62935699999999</v>
+      </c>
+      <c r="M5" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!P5),'Set 1'!P5,"")</f>
+        <v/>
+      </c>
+      <c r="N5" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!Q5),'Set 1 pseudo-2D'!Q5,"")</f>
+        <v/>
+      </c>
+      <c r="O5" s="5" t="str">
+        <f aca="false">IF(AND(ISNUMBER(M5),ISNUMBER(N5)),N5-M5,"")</f>
+        <v/>
+      </c>
+      <c r="P5" s="20" t="n">
+        <f aca="false">'Set 1'!R5</f>
+        <v>650.201104432882</v>
+      </c>
+      <c r="Q5" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!S5),'Set 1'!S5,"")</f>
+        <v/>
+      </c>
+      <c r="R5" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R5),'Set 1 pseudo-2D'!R5,"")</f>
+        <v/>
+      </c>
+      <c r="S5" s="11" t="str">
+        <f aca="false">IF(AND(ISNUMBER(Q5),ISNUMBER(R5)),R5-Q5,"")</f>
+        <v/>
+      </c>
+      <c r="T5" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!V5),'Set 1'!V5,"")</f>
+        <v/>
+      </c>
+      <c r="U5" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!S5),'Set 1 pseudo-2D'!S5,"")</f>
+        <v/>
+      </c>
+      <c r="V5" s="6" t="str">
+        <f aca="false">IF(AND(ISNUMBER(T5),ISNUMBER(U5)),U5-T5,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="18" t="n">
+        <f aca="false">'Set 1'!A6</f>
+        <v>5</v>
+      </c>
+      <c r="B6" s="18" t="n">
+        <f aca="false">'Set 1'!D6</f>
+        <v>240</v>
+      </c>
+      <c r="C6" s="19" t="n">
+        <f aca="false">'Set 1'!F6</f>
+        <v>0.52</v>
+      </c>
+      <c r="D6" s="18" t="n">
+        <f aca="false">'Set 1'!I6</f>
+        <v>1407.499351274</v>
+      </c>
+      <c r="E6" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!J6),'Set 1'!J6,"")</f>
+        <v/>
+      </c>
+      <c r="F6" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!O6),'Set 1 pseudo-2D'!O6,"")</f>
+        <v/>
+      </c>
+      <c r="G6" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E6),ISNUMBER(F6)),F6-E6,"")</f>
+        <v/>
+      </c>
+      <c r="H6" s="18" t="n">
+        <f aca="false">'Set 1'!L6</f>
+        <v>1746.37860154084</v>
+      </c>
+      <c r="I6" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!M6),'Set 1'!M6,"")</f>
+        <v/>
+      </c>
+      <c r="J6" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!P6),'Set 1 pseudo-2D'!P6,"")</f>
+        <v/>
+      </c>
+      <c r="K6" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(I6),ISNUMBER(J6)),J6-I6,"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="19" t="n">
+        <f aca="false">'Set 1'!O6</f>
+        <v>7.63384199999999</v>
+      </c>
+      <c r="M6" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!P6),'Set 1'!P6,"")</f>
+        <v/>
+      </c>
+      <c r="N6" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!Q6),'Set 1 pseudo-2D'!Q6,"")</f>
+        <v/>
+      </c>
+      <c r="O6" s="5" t="str">
+        <f aca="false">IF(AND(ISNUMBER(M6),ISNUMBER(N6)),N6-M6,"")</f>
+        <v/>
+      </c>
+      <c r="P6" s="20" t="n">
+        <f aca="false">'Set 1'!R6</f>
+        <v>656.430712583907</v>
+      </c>
+      <c r="Q6" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!S6),'Set 1'!S6,"")</f>
+        <v/>
+      </c>
+      <c r="R6" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R6),'Set 1 pseudo-2D'!R6,"")</f>
+        <v/>
+      </c>
+      <c r="S6" s="11" t="str">
+        <f aca="false">IF(AND(ISNUMBER(Q6),ISNUMBER(R6)),R6-Q6,"")</f>
+        <v/>
+      </c>
+      <c r="T6" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!V6),'Set 1'!V6,"")</f>
+        <v/>
+      </c>
+      <c r="U6" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!S6),'Set 1 pseudo-2D'!S6,"")</f>
+        <v/>
+      </c>
+      <c r="V6" s="6" t="str">
+        <f aca="false">IF(AND(ISNUMBER(T6),ISNUMBER(U6)),U6-T6,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="n">
+        <f aca="false">'Set 1'!A7</f>
+        <v>6</v>
+      </c>
+      <c r="B7" s="18" t="n">
+        <f aca="false">'Set 1'!D7</f>
+        <v>320</v>
+      </c>
+      <c r="C7" s="19" t="n">
+        <f aca="false">'Set 1'!F7</f>
+        <v>0.52</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <f aca="false">'Set 1'!I7</f>
+        <v>1407.29955396803</v>
+      </c>
+      <c r="E7" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!J7),'Set 1'!J7,"")</f>
+        <v/>
+      </c>
+      <c r="F7" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!O7),'Set 1 pseudo-2D'!O7,"")</f>
+        <v/>
+      </c>
+      <c r="G7" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E7),ISNUMBER(F7)),F7-E7,"")</f>
+        <v/>
+      </c>
+      <c r="H7" s="18" t="n">
+        <f aca="false">'Set 1'!L7</f>
+        <v>1745.65194202208</v>
+      </c>
+      <c r="I7" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!M7),'Set 1'!M7,"")</f>
+        <v/>
+      </c>
+      <c r="J7" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!P7),'Set 1 pseudo-2D'!P7,"")</f>
+        <v/>
+      </c>
+      <c r="K7" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(I7),ISNUMBER(J7)),J7-I7,"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="19" t="n">
+        <f aca="false">'Set 1'!O7</f>
+        <v>7.64592499999999</v>
+      </c>
+      <c r="M7" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!P7),'Set 1'!P7,"")</f>
+        <v/>
+      </c>
+      <c r="N7" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!Q7),'Set 1 pseudo-2D'!Q7,"")</f>
+        <v/>
+      </c>
+      <c r="O7" s="5" t="str">
+        <f aca="false">IF(AND(ISNUMBER(M7),ISNUMBER(N7)),N7-M7,"")</f>
+        <v/>
+      </c>
+      <c r="P7" s="20" t="n">
+        <f aca="false">'Set 1'!R7</f>
+        <v>661.922490247295</v>
+      </c>
+      <c r="Q7" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!S7),'Set 1'!S7,"")</f>
+        <v/>
+      </c>
+      <c r="R7" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R7),'Set 1 pseudo-2D'!R7,"")</f>
+        <v/>
+      </c>
+      <c r="S7" s="11" t="str">
+        <f aca="false">IF(AND(ISNUMBER(Q7),ISNUMBER(R7)),R7-Q7,"")</f>
+        <v/>
+      </c>
+      <c r="T7" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!V7),'Set 1'!V7,"")</f>
+        <v/>
+      </c>
+      <c r="U7" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!S7),'Set 1 pseudo-2D'!S7,"")</f>
+        <v/>
+      </c>
+      <c r="V7" s="6" t="str">
+        <f aca="false">IF(AND(ISNUMBER(T7),ISNUMBER(U7)),U7-T7,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="n">
+        <f aca="false">'Set 1'!A8</f>
+        <v>7</v>
+      </c>
+      <c r="B8" s="18" t="n">
+        <f aca="false">'Set 1'!D8</f>
+        <v>240</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <f aca="false">'Set 1'!F8</f>
+        <v>0.4</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <f aca="false">'Set 1'!I8</f>
+        <v>1409.21728292278</v>
+      </c>
+      <c r="E8" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!J8),'Set 1'!J8,"")</f>
+        <v/>
+      </c>
+      <c r="F8" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!O8),'Set 1 pseudo-2D'!O8,"")</f>
+        <v/>
+      </c>
+      <c r="G8" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E8),ISNUMBER(F8)),F8-E8,"")</f>
+        <v/>
+      </c>
+      <c r="H8" s="18" t="n">
+        <f aca="false">'Set 1'!L8</f>
+        <v>1746.53707486242</v>
+      </c>
+      <c r="I8" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!M8),'Set 1'!M8,"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!P8),'Set 1 pseudo-2D'!P8,"")</f>
+        <v/>
+      </c>
+      <c r="K8" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(I8),ISNUMBER(J8)),J8-I8,"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="19" t="n">
+        <f aca="false">'Set 1'!O8</f>
+        <v>7.64266299999999</v>
+      </c>
+      <c r="M8" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!P8),'Set 1'!P8,"")</f>
+        <v/>
+      </c>
+      <c r="N8" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!Q8),'Set 1 pseudo-2D'!Q8,"")</f>
+        <v/>
+      </c>
+      <c r="O8" s="5" t="str">
+        <f aca="false">IF(AND(ISNUMBER(M8),ISNUMBER(N8)),N8-M8,"")</f>
+        <v/>
+      </c>
+      <c r="P8" s="20" t="n">
+        <f aca="false">'Set 1'!R8</f>
+        <v>722.735643650416</v>
+      </c>
+      <c r="Q8" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!S8),'Set 1'!S8,"")</f>
+        <v/>
+      </c>
+      <c r="R8" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R8),'Set 1 pseudo-2D'!R8,"")</f>
+        <v/>
+      </c>
+      <c r="S8" s="11" t="str">
+        <f aca="false">IF(AND(ISNUMBER(Q8),ISNUMBER(R8)),R8-Q8,"")</f>
+        <v/>
+      </c>
+      <c r="T8" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!V8),'Set 1'!V8,"")</f>
+        <v/>
+      </c>
+      <c r="U8" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!S8),'Set 1 pseudo-2D'!S8,"")</f>
+        <v/>
+      </c>
+      <c r="V8" s="6" t="str">
+        <f aca="false">IF(AND(ISNUMBER(T8),ISNUMBER(U8)),U8-T8,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18" t="n">
+        <f aca="false">'Set 1'!A9</f>
+        <v>8</v>
+      </c>
+      <c r="B9" s="18" t="n">
+        <f aca="false">'Set 1'!D9</f>
+        <v>240</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <f aca="false">'Set 1'!F9</f>
+        <v>0.48</v>
+      </c>
+      <c r="D9" s="18" t="n">
+        <f aca="false">'Set 1'!I9</f>
+        <v>1402.53857129639</v>
+      </c>
+      <c r="E9" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!J9),'Set 1'!J9,"")</f>
+        <v/>
+      </c>
+      <c r="F9" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!O9),'Set 1 pseudo-2D'!O9,"")</f>
+        <v/>
+      </c>
+      <c r="G9" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E9),ISNUMBER(F9)),F9-E9,"")</f>
+        <v/>
+      </c>
+      <c r="H9" s="18" t="n">
+        <f aca="false">'Set 1'!L9</f>
+        <v>1746.17439480164</v>
+      </c>
+      <c r="I9" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!M9),'Set 1'!M9,"")</f>
+        <v/>
+      </c>
+      <c r="J9" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!P9),'Set 1 pseudo-2D'!P9,"")</f>
+        <v/>
+      </c>
+      <c r="K9" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(I9),ISNUMBER(J9)),J9-I9,"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="19" t="n">
+        <f aca="false">'Set 1'!O9</f>
+        <v>7.64895899999999</v>
+      </c>
+      <c r="M9" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!P9),'Set 1'!P9,"")</f>
+        <v/>
+      </c>
+      <c r="N9" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!Q9),'Set 1 pseudo-2D'!Q9,"")</f>
+        <v/>
+      </c>
+      <c r="O9" s="5" t="str">
+        <f aca="false">IF(AND(ISNUMBER(M9),ISNUMBER(N9)),N9-M9,"")</f>
+        <v/>
+      </c>
+      <c r="P9" s="20" t="n">
+        <f aca="false">'Set 1'!R9</f>
+        <v>731.734711525745</v>
+      </c>
+      <c r="Q9" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!S9),'Set 1'!S9,"")</f>
+        <v/>
+      </c>
+      <c r="R9" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R9),'Set 1 pseudo-2D'!R9,"")</f>
+        <v/>
+      </c>
+      <c r="S9" s="11" t="str">
+        <f aca="false">IF(AND(ISNUMBER(Q9),ISNUMBER(R9)),R9-Q9,"")</f>
+        <v/>
+      </c>
+      <c r="T9" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!V9),'Set 1'!V9,"")</f>
+        <v/>
+      </c>
+      <c r="U9" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!S9),'Set 1 pseudo-2D'!S9,"")</f>
+        <v/>
+      </c>
+      <c r="V9" s="6" t="str">
+        <f aca="false">IF(AND(ISNUMBER(T9),ISNUMBER(U9)),U9-T9,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="n">
+        <f aca="false">'Set 1'!A10</f>
+        <v>9</v>
+      </c>
+      <c r="B10" s="18" t="n">
+        <f aca="false">'Set 1'!D10</f>
+        <v>160</v>
+      </c>
+      <c r="C10" s="19" t="n">
+        <f aca="false">'Set 1'!F10</f>
+        <v>0.48</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <f aca="false">'Set 1'!I10</f>
+        <v>1403.69923690996</v>
+      </c>
+      <c r="E10" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!J10),'Set 1'!J10,"")</f>
+        <v/>
+      </c>
+      <c r="F10" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!O10),'Set 1 pseudo-2D'!O10,"")</f>
+        <v/>
+      </c>
+      <c r="G10" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E10),ISNUMBER(F10)),F10-E10,"")</f>
+        <v/>
+      </c>
+      <c r="H10" s="18" t="n">
+        <f aca="false">'Set 1'!L10</f>
+        <v>1749.6312767733</v>
+      </c>
+      <c r="I10" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!M10),'Set 1'!M10,"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!P10),'Set 1 pseudo-2D'!P10,"")</f>
+        <v/>
+      </c>
+      <c r="K10" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(I10),ISNUMBER(J10)),J10-I10,"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="19" t="n">
+        <f aca="false">'Set 1'!O10</f>
+        <v>7.64311299999999</v>
+      </c>
+      <c r="M10" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!P10),'Set 1'!P10,"")</f>
+        <v/>
+      </c>
+      <c r="N10" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!Q10),'Set 1 pseudo-2D'!Q10,"")</f>
+        <v/>
+      </c>
+      <c r="O10" s="5" t="str">
+        <f aca="false">IF(AND(ISNUMBER(M10),ISNUMBER(N10)),N10-M10,"")</f>
+        <v/>
+      </c>
+      <c r="P10" s="20" t="n">
+        <f aca="false">'Set 1'!R10</f>
+        <v>741.859239328738</v>
+      </c>
+      <c r="Q10" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!S10),'Set 1'!S10,"")</f>
+        <v/>
+      </c>
+      <c r="R10" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R10),'Set 1 pseudo-2D'!R10,"")</f>
+        <v/>
+      </c>
+      <c r="S10" s="11" t="str">
+        <f aca="false">IF(AND(ISNUMBER(Q10),ISNUMBER(R10)),R10-Q10,"")</f>
+        <v/>
+      </c>
+      <c r="T10" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!V10),'Set 1'!V10,"")</f>
+        <v/>
+      </c>
+      <c r="U10" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!S10),'Set 1 pseudo-2D'!S10,"")</f>
+        <v/>
+      </c>
+      <c r="V10" s="6" t="str">
+        <f aca="false">IF(AND(ISNUMBER(T10),ISNUMBER(U10)),U10-T10,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="n">
+        <f aca="false">'Set 1'!A11</f>
+        <v>10</v>
+      </c>
+      <c r="B11" s="18" t="n">
+        <f aca="false">'Set 1'!D11</f>
+        <v>160</v>
+      </c>
+      <c r="C11" s="19" t="n">
+        <f aca="false">'Set 1'!F11</f>
+        <v>0.44</v>
+      </c>
+      <c r="D11" s="18" t="n">
+        <f aca="false">'Set 1'!I11</f>
+        <v>1404.60593589585</v>
+      </c>
+      <c r="E11" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!J11),'Set 1'!J11,"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!O11),'Set 1 pseudo-2D'!O11,"")</f>
+        <v/>
+      </c>
+      <c r="G11" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E11),ISNUMBER(F11)),F11-E11,"")</f>
+        <v/>
+      </c>
+      <c r="H11" s="18" t="n">
+        <f aca="false">'Set 1'!L11</f>
+        <v>1749.65293005789</v>
+      </c>
+      <c r="I11" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!M11),'Set 1'!M11,"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="18" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!P11),'Set 1 pseudo-2D'!P11,"")</f>
+        <v/>
+      </c>
+      <c r="K11" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(I11),ISNUMBER(J11)),J11-I11,"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="19" t="n">
+        <f aca="false">'Set 1'!O11</f>
+        <v>7.64497699999999</v>
+      </c>
+      <c r="M11" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!P11),'Set 1'!P11,"")</f>
+        <v/>
+      </c>
+      <c r="N11" s="19" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!Q11),'Set 1 pseudo-2D'!Q11,"")</f>
+        <v/>
+      </c>
+      <c r="O11" s="5" t="str">
+        <f aca="false">IF(AND(ISNUMBER(M11),ISNUMBER(N11)),N11-M11,"")</f>
+        <v/>
+      </c>
+      <c r="P11" s="20" t="n">
+        <f aca="false">'Set 1'!R11</f>
+        <v>749.678589646605</v>
+      </c>
+      <c r="Q11" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!S11),'Set 1'!S11,"")</f>
+        <v/>
+      </c>
+      <c r="R11" s="20" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R11),'Set 1 pseudo-2D'!R11,"")</f>
+        <v/>
+      </c>
+      <c r="S11" s="11" t="str">
+        <f aca="false">IF(AND(ISNUMBER(Q11),ISNUMBER(R11)),R11-Q11,"")</f>
+        <v/>
+      </c>
+      <c r="T11" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1'!V11),'Set 1'!V11,"")</f>
+        <v/>
+      </c>
+      <c r="U11" s="21" t="str">
+        <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!S11),'Set 1 pseudo-2D'!S11,"")</f>
+        <v/>
+      </c>
+      <c r="V11" s="6" t="str">
+        <f aca="false">IF(AND(ISNUMBER(T11),ISNUMBER(U11)),U11-T11,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="23" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(E$2:E$11)*ISNUMBER(F$2:F$11))</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="27" t="str">
+        <f aca="false">IF(D16&gt;=3,IFERROR(CORREL(E$2:E$11,F$2:F$11),""),"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(D$2:D$11)*ISNUMBER(F$2:F$11))</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="27" t="str">
+        <f aca="false">IF(F16&gt;=3,IFERROR(CORREL(D$2:D$11,F$2:F$11),""),"")</f>
+        <v/>
+      </c>
+      <c r="H16" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(D$2:D$11)*ISNUMBER(E$2:E$11))</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="27" t="str">
+        <f aca="false">IF(H16&gt;=3,IFERROR(CORREL(D$2:D$11,E$2:E$11),""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="25"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(I$2:I$11)*ISNUMBER(J$2:J$11))</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="27" t="str">
+        <f aca="false">IF(D17&gt;=3,IFERROR(CORREL(I$2:I$11,J$2:J$11),""),"")</f>
+        <v/>
+      </c>
+      <c r="F17" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(H$2:H$11)*ISNUMBER(J$2:J$11))</f>
+        <v>0</v>
+      </c>
+      <c r="G17" s="27" t="str">
+        <f aca="false">IF(F17&gt;=3,IFERROR(CORREL(H$2:H$11,J$2:J$11),""),"")</f>
+        <v/>
+      </c>
+      <c r="H17" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(H$2:H$11)*ISNUMBER(I$2:I$11))</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="27" t="str">
+        <f aca="false">IF(H17&gt;=3,IFERROR(CORREL(H$2:H$11,I$2:I$11),""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" s="25"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(M$2:M$11)*ISNUMBER(N$2:N$11))</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="27" t="str">
+        <f aca="false">IF(D18&gt;=3,IFERROR(CORREL(M$2:M$11,N$2:N$11),""),"")</f>
+        <v/>
+      </c>
+      <c r="F18" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(L$2:L$11)*ISNUMBER(N$2:N$11))</f>
+        <v>0</v>
+      </c>
+      <c r="G18" s="27" t="str">
+        <f aca="false">IF(F18&gt;=3,IFERROR(CORREL(L$2:L$11,N$2:N$11),""),"")</f>
+        <v/>
+      </c>
+      <c r="H18" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(L$2:L$11)*ISNUMBER(M$2:M$11))</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="27" t="str">
+        <f aca="false">IF(H18&gt;=3,IFERROR(CORREL(L$2:L$11,M$2:M$11),""),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(Q$2:Q$11)*ISNUMBER(R$2:R$11))</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="27" t="str">
+        <f aca="false">IF(D19&gt;=3,IFERROR(CORREL(Q$2:Q$11,R$2:R$11),""),"")</f>
+        <v/>
+      </c>
+      <c r="F19" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(P$2:P$11)*ISNUMBER(R$2:R$11))</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="27" t="str">
+        <f aca="false">IF(F19&gt;=3,IFERROR(CORREL(P$2:P$11,R$2:R$11),""),"")</f>
+        <v/>
+      </c>
+      <c r="H19" s="26" t="n">
+        <f aca="false">SUMPRODUCT(ISNUMBER(P$2:P$11)*ISNUMBER(Q$2:Q$11))</f>
+        <v>0</v>
+      </c>
+      <c r="I19" s="27" t="str">
+        <f aca="false">IF(H19&gt;=3,IFERROR(CORREL(P$2:P$11,Q$2:Q$11),""),"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A19:C19"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FF548235"/>
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:V11"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="15" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="19" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="28"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="18" t="n">
+        <f aca="false">'Set 1'!A2</f>
+        <v>1</v>
+      </c>
+      <c r="B2" s="19" t="n">
+        <f aca="false">'Set 1'!C2</f>
+        <v>51</v>
+      </c>
+      <c r="C2" s="18" t="n">
+        <f aca="false">'Set 1'!D2</f>
+        <v>400</v>
+      </c>
+      <c r="D2" s="19" t="n">
+        <f aca="false">'Set 1'!F2</f>
+        <v>0.56</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="F2" s="18" t="n">
+        <f aca="false">Notes!$B$6</f>
+        <v>10</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <f aca="false">E2/C2</f>
+        <v>1.6</v>
+      </c>
+      <c r="H2" s="16" t="str">
+        <f aca="false">IF(G2&gt;=1,"OK","&lt;1 period")</f>
+        <v>OK</v>
+      </c>
+      <c r="I2" s="16" t="str">
+        <f aca="false">IF(ABS(G2-ROUND(G2,0))&lt;0.001,"yes","no")</f>
+        <v>no</v>
+      </c>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M2" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(J2),ISNUMBER(K2),ISNUMBER(L2)),IF(AND(L2&gt;0,K2&gt;=J2),ROUNDUP((K2-J2)/L2,0)+1,""),"")</f>
+        <v/>
+      </c>
+      <c r="N2" s="15"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="9"/>
+      <c r="R2" s="9"/>
+      <c r="S2" s="13"/>
+      <c r="T2" s="13"/>
+      <c r="U2" s="14"/>
+      <c r="V2" s="15"/>
+    </row>
+    <row r="3" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="18" t="n">
+        <f aca="false">'Set 1'!A3</f>
+        <v>2</v>
+      </c>
+      <c r="B3" s="19" t="n">
+        <f aca="false">'Set 1'!C3</f>
+        <v>51</v>
+      </c>
+      <c r="C3" s="18" t="n">
+        <f aca="false">'Set 1'!D3</f>
+        <v>960</v>
+      </c>
+      <c r="D3" s="19" t="n">
+        <f aca="false">'Set 1'!F3</f>
+        <v>0.52</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>960</v>
+      </c>
+      <c r="F3" s="18" t="n">
+        <f aca="false">Notes!$B$6</f>
+        <v>10</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <f aca="false">E3/C3</f>
+        <v>1</v>
+      </c>
+      <c r="H3" s="16" t="str">
+        <f aca="false">IF(G3&gt;=1,"OK","&lt;1 period")</f>
+        <v>OK</v>
+      </c>
+      <c r="I3" s="16" t="str">
+        <f aca="false">IF(ABS(G3-ROUND(G3,0))&lt;0.001,"yes","no")</f>
+        <v>yes</v>
+      </c>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M3" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(J3),ISNUMBER(K3),ISNUMBER(L3)),IF(AND(L3&gt;0,K3&gt;=J3),ROUNDUP((K3-J3)/L3,0)+1,""),"")</f>
+        <v/>
+      </c>
+      <c r="N3" s="15"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
+      <c r="S3" s="13"/>
+      <c r="T3" s="13"/>
+      <c r="U3" s="14"/>
+      <c r="V3" s="15"/>
+    </row>
+    <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="18" t="n">
+        <f aca="false">'Set 1'!A4</f>
+        <v>3</v>
+      </c>
+      <c r="B4" s="19" t="n">
+        <f aca="false">'Set 1'!C4</f>
+        <v>51</v>
+      </c>
+      <c r="C4" s="18" t="n">
+        <f aca="false">'Set 1'!D4</f>
+        <v>480</v>
+      </c>
+      <c r="D4" s="19" t="n">
+        <f aca="false">'Set 1'!F4</f>
+        <v>0.52</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="F4" s="18" t="n">
+        <f aca="false">Notes!$B$6</f>
+        <v>10</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <f aca="false">E4/C4</f>
+        <v>1.33333333333333</v>
+      </c>
+      <c r="H4" s="16" t="str">
+        <f aca="false">IF(G4&gt;=1,"OK","&lt;1 period")</f>
+        <v>OK</v>
+      </c>
+      <c r="I4" s="16" t="str">
+        <f aca="false">IF(ABS(G4-ROUND(G4,0))&lt;0.001,"yes","no")</f>
+        <v>no</v>
+      </c>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M4" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(J4),ISNUMBER(K4),ISNUMBER(L4)),IF(AND(L4&gt;0,K4&gt;=J4),ROUNDUP((K4-J4)/L4,0)+1,""),"")</f>
+        <v/>
+      </c>
+      <c r="N4" s="15"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9"/>
+      <c r="S4" s="13"/>
+      <c r="T4" s="13"/>
+      <c r="U4" s="14"/>
+      <c r="V4" s="15"/>
+    </row>
+    <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="n">
+        <f aca="false">'Set 1'!A5</f>
+        <v>4</v>
+      </c>
+      <c r="B5" s="19" t="n">
+        <f aca="false">'Set 1'!C5</f>
+        <v>51</v>
+      </c>
+      <c r="C5" s="18" t="n">
+        <f aca="false">'Set 1'!D5</f>
+        <v>240</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <f aca="false">'Set 1'!F5</f>
+        <v>0.52</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="F5" s="18" t="n">
+        <f aca="false">Notes!$B$6</f>
+        <v>10</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <f aca="false">E5/C5</f>
+        <v>2.66666666666667</v>
+      </c>
+      <c r="H5" s="16" t="str">
+        <f aca="false">IF(G5&gt;=1,"OK","&lt;1 period")</f>
+        <v>OK</v>
+      </c>
+      <c r="I5" s="16" t="str">
+        <f aca="false">IF(ABS(G5-ROUND(G5,0))&lt;0.001,"yes","no")</f>
+        <v>no</v>
+      </c>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M5" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(J5),ISNUMBER(K5),ISNUMBER(L5)),IF(AND(L5&gt;0,K5&gt;=J5),ROUNDUP((K5-J5)/L5,0)+1,""),"")</f>
+        <v/>
+      </c>
+      <c r="N5" s="15"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="9"/>
+      <c r="R5" s="9"/>
+      <c r="S5" s="13"/>
+      <c r="T5" s="13"/>
+      <c r="U5" s="14"/>
+      <c r="V5" s="15"/>
+    </row>
+    <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="18" t="n">
+        <f aca="false">'Set 1'!A6</f>
+        <v>5</v>
+      </c>
+      <c r="B6" s="19" t="n">
+        <f aca="false">'Set 1'!C6</f>
+        <v>50.95</v>
+      </c>
+      <c r="C6" s="18" t="n">
+        <f aca="false">'Set 1'!D6</f>
+        <v>240</v>
+      </c>
+      <c r="D6" s="19" t="n">
+        <f aca="false">'Set 1'!F6</f>
+        <v>0.52</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <f aca="false">Notes!$B$6</f>
+        <v>10</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <f aca="false">E6/C6</f>
+        <v>2.66666666666667</v>
+      </c>
+      <c r="H6" s="16" t="str">
+        <f aca="false">IF(G6&gt;=1,"OK","&lt;1 period")</f>
+        <v>OK</v>
+      </c>
+      <c r="I6" s="16" t="str">
+        <f aca="false">IF(ABS(G6-ROUND(G6,0))&lt;0.001,"yes","no")</f>
+        <v>no</v>
+      </c>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M6" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(J6),ISNUMBER(K6),ISNUMBER(L6)),IF(AND(L6&gt;0,K6&gt;=J6),ROUNDUP((K6-J6)/L6,0)+1,""),"")</f>
+        <v/>
+      </c>
+      <c r="N6" s="15"/>
+      <c r="O6" s="7"/>
+      <c r="P6" s="7"/>
+      <c r="Q6" s="9"/>
+      <c r="R6" s="9"/>
+      <c r="S6" s="13"/>
+      <c r="T6" s="13"/>
+      <c r="U6" s="14"/>
+      <c r="V6" s="15"/>
+    </row>
+    <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="n">
+        <f aca="false">'Set 1'!A7</f>
+        <v>6</v>
+      </c>
+      <c r="B7" s="19" t="n">
+        <f aca="false">'Set 1'!C7</f>
+        <v>50.95</v>
+      </c>
+      <c r="C7" s="18" t="n">
+        <f aca="false">'Set 1'!D7</f>
+        <v>320</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <f aca="false">'Set 1'!F7</f>
+        <v>0.52</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="F7" s="18" t="n">
+        <f aca="false">Notes!$B$6</f>
+        <v>10</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <f aca="false">E7/C7</f>
+        <v>2</v>
+      </c>
+      <c r="H7" s="16" t="str">
+        <f aca="false">IF(G7&gt;=1,"OK","&lt;1 period")</f>
+        <v>OK</v>
+      </c>
+      <c r="I7" s="16" t="str">
+        <f aca="false">IF(ABS(G7-ROUND(G7,0))&lt;0.001,"yes","no")</f>
+        <v>yes</v>
+      </c>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M7" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(J7),ISNUMBER(K7),ISNUMBER(L7)),IF(AND(L7&gt;0,K7&gt;=J7),ROUNDUP((K7-J7)/L7,0)+1,""),"")</f>
+        <v/>
+      </c>
+      <c r="N7" s="15"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="9"/>
+      <c r="R7" s="9"/>
+      <c r="S7" s="13"/>
+      <c r="T7" s="13"/>
+      <c r="U7" s="14"/>
+      <c r="V7" s="15"/>
+    </row>
+    <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="n">
+        <f aca="false">'Set 1'!A8</f>
+        <v>7</v>
+      </c>
+      <c r="B8" s="19" t="n">
+        <f aca="false">'Set 1'!C8</f>
+        <v>51</v>
+      </c>
+      <c r="C8" s="18" t="n">
+        <f aca="false">'Set 1'!D8</f>
+        <v>240</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <f aca="false">'Set 1'!F8</f>
+        <v>0.4</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <f aca="false">Notes!$B$6</f>
+        <v>10</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <f aca="false">E8/C8</f>
+        <v>2.66666666666667</v>
+      </c>
+      <c r="H8" s="16" t="str">
+        <f aca="false">IF(G8&gt;=1,"OK","&lt;1 period")</f>
+        <v>OK</v>
+      </c>
+      <c r="I8" s="16" t="str">
+        <f aca="false">IF(ABS(G8-ROUND(G8,0))&lt;0.001,"yes","no")</f>
+        <v>no</v>
+      </c>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M8" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(J8),ISNUMBER(K8),ISNUMBER(L8)),IF(AND(L8&gt;0,K8&gt;=J8),ROUNDUP((K8-J8)/L8,0)+1,""),"")</f>
+        <v/>
+      </c>
+      <c r="N8" s="15"/>
+      <c r="O8" s="7"/>
+      <c r="P8" s="7"/>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="9"/>
+      <c r="S8" s="13"/>
+      <c r="T8" s="13"/>
+      <c r="U8" s="14"/>
+      <c r="V8" s="15"/>
+    </row>
+    <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18" t="n">
+        <f aca="false">'Set 1'!A9</f>
+        <v>8</v>
+      </c>
+      <c r="B9" s="19" t="n">
+        <f aca="false">'Set 1'!C9</f>
+        <v>50.95</v>
+      </c>
+      <c r="C9" s="18" t="n">
+        <f aca="false">'Set 1'!D9</f>
+        <v>240</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <f aca="false">'Set 1'!F9</f>
+        <v>0.48</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <f aca="false">Notes!$B$6</f>
+        <v>10</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <f aca="false">E9/C9</f>
+        <v>2.66666666666667</v>
+      </c>
+      <c r="H9" s="16" t="str">
+        <f aca="false">IF(G9&gt;=1,"OK","&lt;1 period")</f>
+        <v>OK</v>
+      </c>
+      <c r="I9" s="16" t="str">
+        <f aca="false">IF(ABS(G9-ROUND(G9,0))&lt;0.001,"yes","no")</f>
+        <v>no</v>
+      </c>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M9" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(J9),ISNUMBER(K9),ISNUMBER(L9)),IF(AND(L9&gt;0,K9&gt;=J9),ROUNDUP((K9-J9)/L9,0)+1,""),"")</f>
+        <v/>
+      </c>
+      <c r="N9" s="15"/>
+      <c r="O9" s="7"/>
+      <c r="P9" s="7"/>
+      <c r="Q9" s="9"/>
+      <c r="R9" s="9"/>
+      <c r="S9" s="13"/>
+      <c r="T9" s="13"/>
+      <c r="U9" s="14"/>
+      <c r="V9" s="15"/>
+    </row>
+    <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="n">
+        <f aca="false">'Set 1'!A10</f>
+        <v>9</v>
+      </c>
+      <c r="B10" s="19" t="n">
+        <f aca="false">'Set 1'!C10</f>
+        <v>51</v>
+      </c>
+      <c r="C10" s="18" t="n">
+        <f aca="false">'Set 1'!D10</f>
+        <v>160</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <f aca="false">'Set 1'!F10</f>
+        <v>0.48</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <f aca="false">Notes!$B$6</f>
+        <v>10</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <f aca="false">E10/C10</f>
+        <v>4</v>
+      </c>
+      <c r="H10" s="16" t="str">
+        <f aca="false">IF(G10&gt;=1,"OK","&lt;1 period")</f>
+        <v>OK</v>
+      </c>
+      <c r="I10" s="16" t="str">
+        <f aca="false">IF(ABS(G10-ROUND(G10,0))&lt;0.001,"yes","no")</f>
+        <v>yes</v>
+      </c>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M10" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(J10),ISNUMBER(K10),ISNUMBER(L10)),IF(AND(L10&gt;0,K10&gt;=J10),ROUNDUP((K10-J10)/L10,0)+1,""),"")</f>
+        <v/>
+      </c>
+      <c r="N10" s="15"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
+      <c r="Q10" s="9"/>
+      <c r="R10" s="9"/>
+      <c r="S10" s="13"/>
+      <c r="T10" s="13"/>
+      <c r="U10" s="14"/>
+      <c r="V10" s="15"/>
+    </row>
+    <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="n">
+        <f aca="false">'Set 1'!A11</f>
+        <v>10</v>
+      </c>
+      <c r="B11" s="19" t="n">
+        <f aca="false">'Set 1'!C11</f>
+        <v>51</v>
+      </c>
+      <c r="C11" s="18" t="n">
+        <f aca="false">'Set 1'!D11</f>
+        <v>160</v>
+      </c>
+      <c r="D11" s="19" t="n">
+        <f aca="false">'Set 1'!F11</f>
+        <v>0.44</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="F11" s="18" t="n">
+        <f aca="false">Notes!$B$6</f>
+        <v>10</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <f aca="false">E11/C11</f>
+        <v>4</v>
+      </c>
+      <c r="H11" s="16" t="str">
+        <f aca="false">IF(G11&gt;=1,"OK","&lt;1 period")</f>
+        <v>OK</v>
+      </c>
+      <c r="I11" s="16" t="str">
+        <f aca="false">IF(ABS(G11-ROUND(G11,0))&lt;0.001,"yes","no")</f>
+        <v>yes</v>
+      </c>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M11" s="8" t="str">
+        <f aca="false">IF(AND(ISNUMBER(J11),ISNUMBER(K11),ISNUMBER(L11)),IF(AND(L11&gt;0,K11&gt;=J11),ROUNDUP((K11-J11)/L11,0)+1,""),"")</f>
+        <v/>
+      </c>
+      <c r="N11" s="15"/>
+      <c r="O11" s="7"/>
+      <c r="P11" s="7"/>
+      <c r="Q11" s="9"/>
+      <c r="R11" s="9"/>
+      <c r="S11" s="13"/>
+      <c r="T11" s="13"/>
+      <c r="U11" s="14"/>
+      <c r="V11" s="15"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="G2:G11">
+    <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
     <tabColor rgb="FF2E75B6"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="28" t="s">
-        <v>41</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>42</v>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="28" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="29" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -7658,13 +11297,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF7F7F7F"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -7674,137 +11313,148 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="30" t="s">
-        <v>43</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="31" t="s">
-        <v>44</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="32" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="33" t="s">
-        <v>46</v>
+        <v>87</v>
       </c>
       <c r="B4" s="34" t="n">
         <v>640</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="33" t="s">
-        <v>48</v>
+        <v>89</v>
       </c>
       <c r="B5" s="34" t="n">
         <v>640</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>49</v>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="33" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="34" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" s="33" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>50</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="35" t="s">
-        <v>51</v>
+        <v>94</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>52</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="36" t="s">
-        <v>53</v>
+        <v>96</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>54</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="37" t="s">
-        <v>55</v>
+        <v>98</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>56</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="38" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="33" t="s">
-        <v>59</v>
+        <v>102</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>60</v>
+        <v>103</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>61</v>
+        <v>104</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="39" t="s">
-        <v>62</v>
+        <v>105</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>63</v>
+        <v>106</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="39" t="s">
-        <v>64</v>
+        <v>107</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="39" t="s">
-        <v>66</v>
+        <v>109</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>67</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="39" t="s">
-        <v>68</v>
+        <v>111</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="39" t="s">
-        <v>70</v>
+        <v>113</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>71</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="39" t="s">
-        <v>72</v>
+        <v>115</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>73</v>
+        <v>116</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7812,7 +11462,7 @@
         <v>18</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>74</v>
+        <v>117</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7820,7 +11470,7 @@
         <v>19</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>75</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7828,137 +11478,185 @@
         <v>24</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>76</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="39" t="s">
-        <v>77</v>
+        <v>120</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>78</v>
+        <v>121</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="39" t="s">
-        <v>79</v>
+        <v>122</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="C26" s="33" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="39" t="s">
+        <v>126</v>
+      </c>
+      <c r="C27" s="33" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="C28" s="33" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C26" s="33" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="32" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="33" t="s">
-        <v>83</v>
-      </c>
       <c r="C29" s="33" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="33" t="s">
-        <v>8</v>
-      </c>
-      <c r="B30" s="40" t="n">
-        <v>572</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="B31" s="40" t="n">
-        <v>796</v>
+      <c r="A31" s="32" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="33" t="s">
-        <v>14</v>
-      </c>
-      <c r="B32" s="41" t="n">
-        <v>4.95</v>
+        <v>132</v>
+      </c>
+      <c r="C32" s="33" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="B33" s="41" t="n">
-        <v>5.57</v>
+        <v>8</v>
+      </c>
+      <c r="B33" s="40" t="n">
+        <v>572</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="33" t="s">
-        <v>20</v>
-      </c>
-      <c r="B34" s="42" t="n">
-        <v>0.931</v>
+        <v>11</v>
+      </c>
+      <c r="B34" s="40" t="n">
+        <v>796</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="B35" s="42" t="n">
-        <v>0.618</v>
+        <v>14</v>
+      </c>
+      <c r="B35" s="41" t="n">
+        <v>4.95</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="B36" s="41" t="n">
+        <v>5.57</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="B37" s="42" t="n">
+        <v>0.931</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="B38" s="42" t="n">
+        <v>0.618</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="B36" s="43" t="n">
+      <c r="B39" s="43" t="n">
         <v>0.000178</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="32" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="33" t="s">
-        <v>86</v>
-      </c>
-      <c r="C39" s="33" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="33" t="s">
-        <v>86</v>
-      </c>
-      <c r="C40" s="33" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="33" t="s">
-        <v>86</v>
-      </c>
-      <c r="C41" s="33" t="s">
-        <v>89</v>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="32" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="33" t="s">
-        <v>86</v>
+        <v>135</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>90</v>
+        <v>136</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="33" t="s">
+        <v>135</v>
+      </c>
+      <c r="C43" s="33" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="33" t="s">
+        <v>135</v>
+      </c>
+      <c r="C44" s="33" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="33" t="s">
+        <v>135</v>
+      </c>
+      <c r="C45" s="33" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="33" t="s">
+        <v>135</v>
+      </c>
+      <c r="C46" s="33" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="33" t="s">
+        <v>135</v>
+      </c>
+      <c r="C47" s="33" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="33" t="s">
+        <v>135</v>
+      </c>
+      <c r="C48" s="33" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Harden pseudo-2D and 2D vs 3D tabs after audit
Guard the periods/check formulas against blank or text cell lengths, show
'check window' for an invalid sweep window, add a 2D vs 3D cell-length
comparison with a mismatch flag, and blank Pearson r for constant series.
Validate the Notes parameter cells, relabel the survey-window columns, and
tighten the Notes wording (legend, 2D vs 3D description, PBC seam, naming).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011WnE18kmcTTQHQwwBdKitt
</commit_message>
<xml_diff>
--- a/CM_Sweep_Sets_1_2.xlsx
+++ b/CM_Sweep_Sets_1_2.xlsx
@@ -183,7 +183,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Rank of ML loop area minus rank of SIM loop area, both ascending within the 10 points of the set. Shown only once all 10 SIM loop areas are filled in. Reverse-engineered from Aum's 2D sweep sample (matches all 10 rows).</t>
+          <t xml:space="preserve">Rank of ML loop area minus rank of SIM loop area, both ascending within the 10 points of the set. Shown only once all 10 SIM loop areas are filled in. Reverse-engineered from Aum's CM sweep sample (matches all 10 rows).</t>
         </r>
       </text>
     </comment>
@@ -361,7 +361,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Rank of ML loop area minus rank of SIM loop area, both ascending within the 10 points of the set. Shown only once all 10 SIM loop areas are filled in. Reverse-engineered from Aum's 2D sweep sample (matches all 10 rows).</t>
+          <t xml:space="preserve">Rank of ML loop area minus rank of SIM loop area, both ascending within the 10 points of the set. Shown only once all 10 SIM loop areas are filled in. Reverse-engineered from Aum's CM sweep sample (matches all 10 rows).</t>
         </r>
       </text>
     </comment>
@@ -435,6 +435,18 @@
         </r>
       </text>
     </comment>
+    <comment ref="X1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">3D cell length is the Set 1 assumption on Notes!B4; 2D cell length comes from the pseudo-2D tab.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -453,7 +465,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Input: simulation-cell length along the CM direction. Default is 640 (the Set 1 cell), raised to λ where λ &gt; 640 so that at least one full period fits. Overwrite with the real cell length.</t>
+          <t xml:space="preserve">Input: simulation-cell length along the CM direction, in the same units as λ (nm). Default is 640 (the Set 1 cell), raised to λ where λ &gt; 640 so that at least one full period fits. Overwrite with the real cell length.</t>
         </r>
       </text>
     </comment>
@@ -465,7 +477,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">From Notes!B6: the pseudo-2D cell is 10 units thick in the thin direction. Confirm which axis that is: sine.m modulates along y.</t>
+          <t xml:space="preserve">From Notes!B6: the pseudo-2D cell is 10 units thick in the thin direction (1 unit = 1 grid point; write_vtk uses SPACING 1, assumed 1 nm like λ). Confirm which axis that is: sine.m modulates along y.</t>
         </r>
       </text>
     </comment>
@@ -513,7 +525,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Survey sweep: coarse stress steps to find where the transformation happens. Enter where the transformation window starts.</t>
+          <t xml:space="preserve">From the survey sweep (coarse stress steps): the lowest stress where the transformation starts. If the reverse transformation sits at a clearly different stress, use the outer limits that cover both.</t>
         </r>
       </text>
     </comment>
@@ -525,7 +537,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Where the transformation window ends, from the survey sweep.</t>
+          <t xml:space="preserve">From the survey sweep: the highest stress where the transformation ends (outer limit, as for the start).</t>
         </r>
       </text>
     </comment>
@@ -549,7 +561,19 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">= ROUNDUP((end − start) ÷ step) + 1. Blank until the window is entered.</t>
+          <t xml:space="preserve">= ROUNDUP((end − start) ÷ step) + 1. Blank until the window and step are entered; shows "check window" if the end is below the start or the step is 0 or less.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Free text, e.g. survey done, fine sweep running, done.</t>
         </r>
       </text>
     </comment>
@@ -558,7 +582,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="147">
   <si>
     <t xml:space="preserve">Point</t>
   </si>
@@ -734,6 +758,15 @@
     <t xml:space="preserve">Δ max vf (2D−3D)</t>
   </si>
   <si>
+    <t xml:space="preserve">2D cell length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3D cell length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same cell?</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pearson r (blank until at least 3 paired points)</t>
   </si>
   <si>
@@ -755,10 +788,10 @@
     <t xml:space="preserve">r ML vs 3D</t>
   </si>
   <si>
-    <t xml:space="preserve">Cell length along CM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thin axis length (units)</t>
+    <t xml:space="preserve">Cell length along CM (nm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thin axis length (grid units)</t>
   </si>
   <si>
     <t xml:space="preserve">Periods in cell</t>
@@ -770,10 +803,10 @@
     <t xml:space="preserve">Integer periods?</t>
   </si>
   <si>
-    <t xml:space="preserve">Survey window start (MPa)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Survey window end (MPa)</t>
+    <t xml:space="preserve">Transformation window start (MPa)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transformation window end (MPa)</t>
   </si>
   <si>
     <t xml:space="preserve">Fine step (MPa)</t>
@@ -815,7 +848,7 @@
     <t xml:space="preserve">CM sweep, Sets 1 and 2: notes, assumptions and legend</t>
   </si>
   <si>
-    <t xml:space="preserve">Layout follows Aum's 2D sweep sheet. ML columns, avg/λ/amp and renders are filled in; SIM columns are blank until the 3D results are added.</t>
+    <t xml:space="preserve">Layout follows Aum's CM sweep sheet. ML columns, avg/λ/amp and renders are filled in; SIM columns are blank until the 3D results are added.</t>
   </si>
   <si>
     <t xml:space="preserve">Parameters (edit here)</t>
@@ -824,7 +857,7 @@
     <t xml:space="preserve">Set 1 domain length L (nm)</t>
   </si>
   <si>
-    <t xml:space="preserve">Assumption: taken from the 'waves / 640 nm' header in Aum's 2D sweep sheet; the Set 1 renders agree (stripe count = 640/λ). Point 2 (λ = 960) holds only 0.67 periods at 640, so it breaks the one-period rule: it needs a cell of at least 960.</t>
+    <t xml:space="preserve">Assumption: taken from the 'waves / 640 nm' header in Aum's CM sweep sheet; the Set 1 renders agree (stripe count = 640/λ). Point 2 (λ = 960) holds only 0.67 periods at 640, so it breaks the one-period rule: it needs a cell of at least 960.</t>
   </si>
   <si>
     <t xml:space="preserve">Set 2 domain length L (nm)</t>
@@ -836,7 +869,7 @@
     <t xml:space="preserve">Pseudo-2D thin axis (units)</t>
   </si>
   <si>
-    <t xml:space="preserve">From your note: the pseudo-2D cell is 10 units thick. Confirm which axis is thinned: sine.m modulates along y, so if y is the thin axis the CM has to run along x or z.</t>
+    <t xml:space="preserve">From your note: the pseudo-2D cell is 10 units thick (1 unit = 1 grid point; write_vtk uses SPACING 1, assumed 1 nm like λ). Confirm which axis is thinned: sine.m modulates along y, so if y is the thin axis the CM has to run along x or z.</t>
   </si>
   <si>
     <t xml:space="preserve">Legend</t>
@@ -857,13 +890,13 @@
     <t xml:space="preserve">Blue text, yellow fill</t>
   </si>
   <si>
-    <t xml:space="preserve">Cell to fill in: the SIM columns. Everything that depends on them (Δ columns, loop ratio, loop rank Δ, Combined, Charts) fills itself in. Leave a cell empty if there is no value: text such as n/a can plot as 0 in Excel charts, and Combined only passes numbers through.</t>
+    <t xml:space="preserve">Cell to fill in: the SIM columns, plus the transformation-window and 2D result cells on the pseudo-2D tab. Everything that depends on them (Δ columns, loop ratio, loop rank Δ, Combined, Charts, 2D vs 3D) fills itself in. Leave a cell empty if there is no value: text such as n/a can plot as 0 in Excel charts, and the Combined and 2D vs 3D tabs only pass numbers through.</t>
   </si>
   <si>
     <t xml:space="preserve">Green text</t>
   </si>
   <si>
-    <t xml:space="preserve">Link to another sheet (the Combined tab). Do not overwrite.</t>
+    <t xml:space="preserve">Link to another sheet (Combined, 2D vs 3D and pseudo-2D tabs). Do not overwrite.</t>
   </si>
   <si>
     <t xml:space="preserve">Do not sort or filter</t>
@@ -935,7 +968,7 @@
     <t xml:space="preserve">One-period rule</t>
   </si>
   <si>
-    <t xml:space="preserve">The simulation cell must hold at least one full period of the CM wavelength along the modulation direction (cell length ≥ λ). The waves column on the Set sheets, and Periods in cell on the pseudo-2D sheet, turn red below 1. A non-integer number of periods also leaves a seam under periodic boundaries (the PBC line in sine.m forces the last plane to avg); the pseudo-2D sheet shows this as information only.</t>
+    <t xml:space="preserve">The simulation cell must hold at least one full period of the CM wavelength along the modulation direction (cell length ≥ λ). The waves column on the Set sheets, and Periods in cell on the pseudo-2D sheet, turn red below 1. Separately, a non-integer number of periods leaves a seam under periodic boundaries; the PBC line in sine.m only sets the last plane to avg, which does not remove it. The pseudo-2D sheet shows this as information only (at 640, 6 of the 10 Set 1 points have a non-integer number of periods).</t>
   </si>
   <si>
     <t xml:space="preserve">Set 1 pseudo-2D sheet</t>
@@ -947,7 +980,7 @@
     <t xml:space="preserve">Set 1 2D vs 3D sheet</t>
   </si>
   <si>
-    <t xml:space="preserve">Compares the pseudo-2D results (2D) with the regular 3D sweep (the SIM columns on the Set 1 tab) and with the Shanghai ML values. Every cell is a link. Δ = 2D − 3D. The table under it gives Pearson r for 2D vs 3D, ML vs 2D and ML vs 3D; it needs at least 3 paired points. The Charts tab plots 2D against 3D.</t>
+    <t xml:space="preserve">Compares the pseudo-2D results (2D) with the regular 3D sweep (the SIM columns on the Set 1 tab) and with the Shanghai ML values. Values are linked from the Set 1 and pseudo-2D tabs; Δ (2D − 3D) and the Pearson table are calculated. Columns W–Y compare the 2D cell length with the 3D cell length assumed in B4 (red where they differ); the r table includes every point, so check them before reading it. r needs at least 3 paired points. The Charts tab plots 2D against 3D.</t>
   </si>
   <si>
     <t xml:space="preserve">ParaView renders from VTK_Field_Report.xlsx, one per point. They appear to be auto-scaled to each field's own range, so amplitude differences between points are not visible.</t>
@@ -959,7 +992,7 @@
     <t xml:space="preserve">Source of the example values</t>
   </si>
   <si>
-    <t xml:space="preserve">Aum's 2D sweep sheet, set 1 point 1. Shown only so you can see the expected number format; it is not entered in the Set 1 sheet.</t>
+    <t xml:space="preserve">Aum's CM sweep sheet, set 1 point 1. Shown only so you can see the expected number format; it is not entered in the Set 1 sheet.</t>
   </si>
   <si>
     <t xml:space="preserve">Open items</t>
@@ -980,7 +1013,10 @@
     <t xml:space="preserve">Confirm which axis is the thin (10-unit) one. sine.m modulates along y, so in the pseudo-2D cell the CM must run along a different axis.</t>
   </si>
   <si>
-    <t xml:space="preserve">One-period rule: Set 1 point 2 (960 nm) needs a cell of at least 960, but its existing 3D run used 640 (0.67 periods). A like-for-like 2D vs 3D comparison for that point needs a 3D run in a cell of at least 960.</t>
+    <t xml:space="preserve">The third (lateral) dimension of the pseudo-2D cell is not recorded on the pseudo-2D tab.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-period rule: if the Set 1 point 2 3D run used a 640 cell (assumed, B4) it holds 0.67 periods and breaks the rule. Decide whether it should be re-run in a cell of at least 960; the 2D vs 3D tab flags the mismatch (Same cell? = no).</t>
   </si>
   <si>
     <t xml:space="preserve">One-period rule: Set 2 points 7–10 break it in a 640 cell. Confirm the cell the Set 2 runs used.</t>
@@ -1698,11 +1734,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="38986248"/>
-        <c:axId val="64274837"/>
+        <c:axId val="75842010"/>
+        <c:axId val="74849449"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="38986248"/>
+        <c:axId val="75842010"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1778,12 +1814,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64274837"/>
+        <c:crossAx val="74849449"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="64274837"/>
+        <c:axId val="74849449"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1859,7 +1895,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38986248"/>
+        <c:crossAx val="75842010"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2167,11 +2203,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="72562490"/>
-        <c:axId val="23694930"/>
+        <c:axId val="9354521"/>
+        <c:axId val="54065120"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="72562490"/>
+        <c:axId val="9354521"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2247,12 +2283,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23694930"/>
+        <c:crossAx val="54065120"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="23694930"/>
+        <c:axId val="54065120"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2328,7 +2364,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72562490"/>
+        <c:crossAx val="9354521"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2636,11 +2672,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="8290263"/>
-        <c:axId val="87717462"/>
+        <c:axId val="56821607"/>
+        <c:axId val="391956"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="8290263"/>
+        <c:axId val="56821607"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2716,12 +2752,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87717462"/>
+        <c:crossAx val="391956"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="87717462"/>
+        <c:axId val="391956"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2797,7 +2833,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8290263"/>
+        <c:crossAx val="56821607"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3105,11 +3141,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="69833587"/>
-        <c:axId val="42185557"/>
+        <c:axId val="32790036"/>
+        <c:axId val="99147768"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="69833587"/>
+        <c:axId val="32790036"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3185,12 +3221,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42185557"/>
+        <c:crossAx val="99147768"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="42185557"/>
+        <c:axId val="99147768"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3266,7 +3302,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69833587"/>
+        <c:crossAx val="32790036"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3438,11 +3474,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="50465810"/>
-        <c:axId val="50372058"/>
+        <c:axId val="44922478"/>
+        <c:axId val="68456179"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="50465810"/>
+        <c:axId val="44922478"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3518,12 +3554,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50372058"/>
+        <c:crossAx val="68456179"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="50372058"/>
+        <c:axId val="68456179"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3599,7 +3635,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50465810"/>
+        <c:crossAx val="44922478"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3771,11 +3807,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="66534308"/>
-        <c:axId val="28674830"/>
+        <c:axId val="57946275"/>
+        <c:axId val="50354332"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="66534308"/>
+        <c:axId val="57946275"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3851,12 +3887,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="28674830"/>
+        <c:crossAx val="50354332"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="28674830"/>
+        <c:axId val="50354332"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3932,7 +3968,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66534308"/>
+        <c:crossAx val="57946275"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4104,11 +4140,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="74024720"/>
-        <c:axId val="76240116"/>
+        <c:axId val="71070335"/>
+        <c:axId val="30852454"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="74024720"/>
+        <c:axId val="71070335"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4184,12 +4220,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="76240116"/>
+        <c:crossAx val="30852454"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="76240116"/>
+        <c:axId val="30852454"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4265,7 +4301,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74024720"/>
+        <c:crossAx val="71070335"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4437,11 +4473,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="6394594"/>
-        <c:axId val="93832438"/>
+        <c:axId val="81176402"/>
+        <c:axId val="36498013"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="6394594"/>
+        <c:axId val="81176402"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4517,12 +4553,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93832438"/>
+        <c:crossAx val="36498013"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="93832438"/>
+        <c:axId val="36498013"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4598,7 +4634,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6394594"/>
+        <c:crossAx val="81176402"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -9311,7 +9347,7 @@
         <v>0</v>
       </c>
       <c r="D26" s="27" t="str">
-        <f aca="false">IF(C26&gt;=3,IFERROR(CORREL(G$2:G$11,H$2:H$11),""),"")</f>
+        <f aca="false">IF(AND(C26&gt;=3,MAX(G$2:G$11)-MIN(G$2:G$11)&gt;0.000000001*(ABS(MAX(G$2:G$11))+ABS(MIN(G$2:G$11))),MAX(H$2:H$11)-MIN(H$2:H$11)&gt;0.000000001*(ABS(MAX(H$2:H$11))+ABS(MIN(H$2:H$11)))),IFERROR(CORREL(G$2:G$11,H$2:H$11),""),"")</f>
         <v/>
       </c>
       <c r="E26" s="26" t="n">
@@ -9319,7 +9355,7 @@
         <v>0</v>
       </c>
       <c r="F26" s="27" t="str">
-        <f aca="false">IF(E26&gt;=3,IFERROR(CORREL(G$12:G$21,H$12:H$21),""),"")</f>
+        <f aca="false">IF(AND(E26&gt;=3,MAX(G$12:G$21)-MIN(G$12:G$21)&gt;0.000000001*(ABS(MAX(G$12:G$21))+ABS(MIN(G$12:G$21))),MAX(H$12:H$21)-MIN(H$12:H$21)&gt;0.000000001*(ABS(MAX(H$12:H$21))+ABS(MIN(H$12:H$21)))),IFERROR(CORREL(G$12:G$21,H$12:H$21),""),"")</f>
         <v/>
       </c>
       <c r="G26" s="26" t="n">
@@ -9327,7 +9363,7 @@
         <v>0</v>
       </c>
       <c r="H26" s="27" t="str">
-        <f aca="false">IF(G26&gt;=3,IFERROR(CORREL(G$2:G$21,H$2:H$21),""),"")</f>
+        <f aca="false">IF(AND(G26&gt;=3,MAX(G$2:G$21)-MIN(G$2:G$21)&gt;0.000000001*(ABS(MAX(G$2:G$21))+ABS(MIN(G$2:G$21))),MAX(H$2:H$21)-MIN(H$2:H$21)&gt;0.000000001*(ABS(MAX(H$2:H$21))+ABS(MIN(H$2:H$21)))),IFERROR(CORREL(G$2:G$21,H$2:H$21),""),"")</f>
         <v/>
       </c>
     </row>
@@ -9341,7 +9377,7 @@
         <v>0</v>
       </c>
       <c r="D27" s="27" t="str">
-        <f aca="false">IF(C27&gt;=3,IFERROR(CORREL(J$2:J$11,K$2:K$11),""),"")</f>
+        <f aca="false">IF(AND(C27&gt;=3,MAX(J$2:J$11)-MIN(J$2:J$11)&gt;0.000000001*(ABS(MAX(J$2:J$11))+ABS(MIN(J$2:J$11))),MAX(K$2:K$11)-MIN(K$2:K$11)&gt;0.000000001*(ABS(MAX(K$2:K$11))+ABS(MIN(K$2:K$11)))),IFERROR(CORREL(J$2:J$11,K$2:K$11),""),"")</f>
         <v/>
       </c>
       <c r="E27" s="26" t="n">
@@ -9349,7 +9385,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="27" t="str">
-        <f aca="false">IF(E27&gt;=3,IFERROR(CORREL(J$12:J$21,K$12:K$21),""),"")</f>
+        <f aca="false">IF(AND(E27&gt;=3,MAX(J$12:J$21)-MIN(J$12:J$21)&gt;0.000000001*(ABS(MAX(J$12:J$21))+ABS(MIN(J$12:J$21))),MAX(K$12:K$21)-MIN(K$12:K$21)&gt;0.000000001*(ABS(MAX(K$12:K$21))+ABS(MIN(K$12:K$21)))),IFERROR(CORREL(J$12:J$21,K$12:K$21),""),"")</f>
         <v/>
       </c>
       <c r="G27" s="26" t="n">
@@ -9357,7 +9393,7 @@
         <v>0</v>
       </c>
       <c r="H27" s="27" t="str">
-        <f aca="false">IF(G27&gt;=3,IFERROR(CORREL(J$2:J$21,K$2:K$21),""),"")</f>
+        <f aca="false">IF(AND(G27&gt;=3,MAX(J$2:J$21)-MIN(J$2:J$21)&gt;0.000000001*(ABS(MAX(J$2:J$21))+ABS(MIN(J$2:J$21))),MAX(K$2:K$21)-MIN(K$2:K$21)&gt;0.000000001*(ABS(MAX(K$2:K$21))+ABS(MIN(K$2:K$21)))),IFERROR(CORREL(J$2:J$21,K$2:K$21),""),"")</f>
         <v/>
       </c>
     </row>
@@ -9371,7 +9407,7 @@
         <v>0</v>
       </c>
       <c r="D28" s="27" t="str">
-        <f aca="false">IF(C28&gt;=3,IFERROR(CORREL(M$2:M$11,N$2:N$11),""),"")</f>
+        <f aca="false">IF(AND(C28&gt;=3,MAX(M$2:M$11)-MIN(M$2:M$11)&gt;0.000000001*(ABS(MAX(M$2:M$11))+ABS(MIN(M$2:M$11))),MAX(N$2:N$11)-MIN(N$2:N$11)&gt;0.000000001*(ABS(MAX(N$2:N$11))+ABS(MIN(N$2:N$11)))),IFERROR(CORREL(M$2:M$11,N$2:N$11),""),"")</f>
         <v/>
       </c>
       <c r="E28" s="26" t="n">
@@ -9379,7 +9415,7 @@
         <v>0</v>
       </c>
       <c r="F28" s="27" t="str">
-        <f aca="false">IF(E28&gt;=3,IFERROR(CORREL(M$12:M$21,N$12:N$21),""),"")</f>
+        <f aca="false">IF(AND(E28&gt;=3,MAX(M$12:M$21)-MIN(M$12:M$21)&gt;0.000000001*(ABS(MAX(M$12:M$21))+ABS(MIN(M$12:M$21))),MAX(N$12:N$21)-MIN(N$12:N$21)&gt;0.000000001*(ABS(MAX(N$12:N$21))+ABS(MIN(N$12:N$21)))),IFERROR(CORREL(M$12:M$21,N$12:N$21),""),"")</f>
         <v/>
       </c>
       <c r="G28" s="26" t="n">
@@ -9387,7 +9423,7 @@
         <v>0</v>
       </c>
       <c r="H28" s="27" t="str">
-        <f aca="false">IF(G28&gt;=3,IFERROR(CORREL(M$2:M$21,N$2:N$21),""),"")</f>
+        <f aca="false">IF(AND(G28&gt;=3,MAX(M$2:M$21)-MIN(M$2:M$21)&gt;0.000000001*(ABS(MAX(M$2:M$21))+ABS(MIN(M$2:M$21))),MAX(N$2:N$21)-MIN(N$2:N$21)&gt;0.000000001*(ABS(MAX(N$2:N$21))+ABS(MIN(N$2:N$21)))),IFERROR(CORREL(M$2:M$21,N$2:N$21),""),"")</f>
         <v/>
       </c>
     </row>
@@ -9401,7 +9437,7 @@
         <v>0</v>
       </c>
       <c r="D29" s="27" t="str">
-        <f aca="false">IF(C29&gt;=3,IFERROR(CORREL(P$2:P$11,Q$2:Q$11),""),"")</f>
+        <f aca="false">IF(AND(C29&gt;=3,MAX(P$2:P$11)-MIN(P$2:P$11)&gt;0.000000001*(ABS(MAX(P$2:P$11))+ABS(MIN(P$2:P$11))),MAX(Q$2:Q$11)-MIN(Q$2:Q$11)&gt;0.000000001*(ABS(MAX(Q$2:Q$11))+ABS(MIN(Q$2:Q$11)))),IFERROR(CORREL(P$2:P$11,Q$2:Q$11),""),"")</f>
         <v/>
       </c>
       <c r="E29" s="26" t="n">
@@ -9409,7 +9445,7 @@
         <v>0</v>
       </c>
       <c r="F29" s="27" t="str">
-        <f aca="false">IF(E29&gt;=3,IFERROR(CORREL(P$12:P$21,Q$12:Q$21),""),"")</f>
+        <f aca="false">IF(AND(E29&gt;=3,MAX(P$12:P$21)-MIN(P$12:P$21)&gt;0.000000001*(ABS(MAX(P$12:P$21))+ABS(MIN(P$12:P$21))),MAX(Q$12:Q$21)-MIN(Q$12:Q$21)&gt;0.000000001*(ABS(MAX(Q$12:Q$21))+ABS(MIN(Q$12:Q$21)))),IFERROR(CORREL(P$12:P$21,Q$12:Q$21),""),"")</f>
         <v/>
       </c>
       <c r="G29" s="26" t="n">
@@ -9417,7 +9453,7 @@
         <v>0</v>
       </c>
       <c r="H29" s="27" t="str">
-        <f aca="false">IF(G29&gt;=3,IFERROR(CORREL(P$2:P$21,Q$2:Q$21),""),"")</f>
+        <f aca="false">IF(AND(G29&gt;=3,MAX(P$2:P$21)-MIN(P$2:P$21)&gt;0.000000001*(ABS(MAX(P$2:P$21))+ABS(MIN(P$2:P$21))),MAX(Q$2:Q$21)-MIN(Q$2:Q$21)&gt;0.000000001*(ABS(MAX(Q$2:Q$21))+ABS(MIN(Q$2:Q$21)))),IFERROR(CORREL(P$2:P$21,Q$2:Q$21),""),"")</f>
         <v/>
       </c>
     </row>
@@ -9445,12 +9481,12 @@
     <tabColor rgb="FF548235"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:V19"/>
+  <dimension ref="A1:Y19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="4" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9520,6 +9556,15 @@
       <c r="V1" s="1" t="s">
         <v>57</v>
       </c>
+      <c r="W1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="18" t="n">
@@ -9582,19 +9627,19 @@
         <f aca="false">IF(AND(ISNUMBER(M2),ISNUMBER(N2)),N2-M2,"")</f>
         <v/>
       </c>
-      <c r="P2" s="20" t="n">
+      <c r="P2" s="19" t="n">
         <f aca="false">'Set 1'!R2</f>
         <v>263.959090135506</v>
       </c>
-      <c r="Q2" s="20" t="str">
+      <c r="Q2" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1'!S2),'Set 1'!S2,"")</f>
         <v/>
       </c>
-      <c r="R2" s="20" t="str">
+      <c r="R2" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R2),'Set 1 pseudo-2D'!R2,"")</f>
         <v/>
       </c>
-      <c r="S2" s="11" t="str">
+      <c r="S2" s="5" t="str">
         <f aca="false">IF(AND(ISNUMBER(Q2),ISNUMBER(R2)),R2-Q2,"")</f>
         <v/>
       </c>
@@ -9609,6 +9654,18 @@
       <c r="V2" s="6" t="str">
         <f aca="false">IF(AND(ISNUMBER(T2),ISNUMBER(U2)),U2-T2,"")</f>
         <v/>
+      </c>
+      <c r="W2" s="18" t="n">
+        <f aca="false">'Set 1 pseudo-2D'!E2</f>
+        <v>640</v>
+      </c>
+      <c r="X2" s="18" t="n">
+        <f aca="false">Notes!$B$4</f>
+        <v>640</v>
+      </c>
+      <c r="Y2" s="16" t="str">
+        <f aca="false">IF(AND(ISNUMBER(W2),ISNUMBER(X2)),IF(W2=X2,"yes","no"),"")</f>
+        <v>yes</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9672,19 +9729,19 @@
         <f aca="false">IF(AND(ISNUMBER(M3),ISNUMBER(N3)),N3-M3,"")</f>
         <v/>
       </c>
-      <c r="P3" s="20" t="n">
+      <c r="P3" s="19" t="n">
         <f aca="false">'Set 1'!R3</f>
         <v>543.22722833229</v>
       </c>
-      <c r="Q3" s="20" t="str">
+      <c r="Q3" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1'!S3),'Set 1'!S3,"")</f>
         <v/>
       </c>
-      <c r="R3" s="20" t="str">
+      <c r="R3" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R3),'Set 1 pseudo-2D'!R3,"")</f>
         <v/>
       </c>
-      <c r="S3" s="11" t="str">
+      <c r="S3" s="5" t="str">
         <f aca="false">IF(AND(ISNUMBER(Q3),ISNUMBER(R3)),R3-Q3,"")</f>
         <v/>
       </c>
@@ -9699,6 +9756,18 @@
       <c r="V3" s="6" t="str">
         <f aca="false">IF(AND(ISNUMBER(T3),ISNUMBER(U3)),U3-T3,"")</f>
         <v/>
+      </c>
+      <c r="W3" s="18" t="n">
+        <f aca="false">'Set 1 pseudo-2D'!E3</f>
+        <v>960</v>
+      </c>
+      <c r="X3" s="18" t="n">
+        <f aca="false">Notes!$B$4</f>
+        <v>640</v>
+      </c>
+      <c r="Y3" s="16" t="str">
+        <f aca="false">IF(AND(ISNUMBER(W3),ISNUMBER(X3)),IF(W3=X3,"yes","no"),"")</f>
+        <v>no</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9762,19 +9831,19 @@
         <f aca="false">IF(AND(ISNUMBER(M4),ISNUMBER(N4)),N4-M4,"")</f>
         <v/>
       </c>
-      <c r="P4" s="20" t="n">
+      <c r="P4" s="19" t="n">
         <f aca="false">'Set 1'!R4</f>
         <v>632.07201334017</v>
       </c>
-      <c r="Q4" s="20" t="str">
+      <c r="Q4" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1'!S4),'Set 1'!S4,"")</f>
         <v/>
       </c>
-      <c r="R4" s="20" t="str">
+      <c r="R4" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R4),'Set 1 pseudo-2D'!R4,"")</f>
         <v/>
       </c>
-      <c r="S4" s="11" t="str">
+      <c r="S4" s="5" t="str">
         <f aca="false">IF(AND(ISNUMBER(Q4),ISNUMBER(R4)),R4-Q4,"")</f>
         <v/>
       </c>
@@ -9789,6 +9858,18 @@
       <c r="V4" s="6" t="str">
         <f aca="false">IF(AND(ISNUMBER(T4),ISNUMBER(U4)),U4-T4,"")</f>
         <v/>
+      </c>
+      <c r="W4" s="18" t="n">
+        <f aca="false">'Set 1 pseudo-2D'!E4</f>
+        <v>640</v>
+      </c>
+      <c r="X4" s="18" t="n">
+        <f aca="false">Notes!$B$4</f>
+        <v>640</v>
+      </c>
+      <c r="Y4" s="16" t="str">
+        <f aca="false">IF(AND(ISNUMBER(W4),ISNUMBER(X4)),IF(W4=X4,"yes","no"),"")</f>
+        <v>yes</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9852,19 +9933,19 @@
         <f aca="false">IF(AND(ISNUMBER(M5),ISNUMBER(N5)),N5-M5,"")</f>
         <v/>
       </c>
-      <c r="P5" s="20" t="n">
+      <c r="P5" s="19" t="n">
         <f aca="false">'Set 1'!R5</f>
         <v>650.201104432882</v>
       </c>
-      <c r="Q5" s="20" t="str">
+      <c r="Q5" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1'!S5),'Set 1'!S5,"")</f>
         <v/>
       </c>
-      <c r="R5" s="20" t="str">
+      <c r="R5" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R5),'Set 1 pseudo-2D'!R5,"")</f>
         <v/>
       </c>
-      <c r="S5" s="11" t="str">
+      <c r="S5" s="5" t="str">
         <f aca="false">IF(AND(ISNUMBER(Q5),ISNUMBER(R5)),R5-Q5,"")</f>
         <v/>
       </c>
@@ -9879,6 +9960,18 @@
       <c r="V5" s="6" t="str">
         <f aca="false">IF(AND(ISNUMBER(T5),ISNUMBER(U5)),U5-T5,"")</f>
         <v/>
+      </c>
+      <c r="W5" s="18" t="n">
+        <f aca="false">'Set 1 pseudo-2D'!E5</f>
+        <v>640</v>
+      </c>
+      <c r="X5" s="18" t="n">
+        <f aca="false">Notes!$B$4</f>
+        <v>640</v>
+      </c>
+      <c r="Y5" s="16" t="str">
+        <f aca="false">IF(AND(ISNUMBER(W5),ISNUMBER(X5)),IF(W5=X5,"yes","no"),"")</f>
+        <v>yes</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9942,19 +10035,19 @@
         <f aca="false">IF(AND(ISNUMBER(M6),ISNUMBER(N6)),N6-M6,"")</f>
         <v/>
       </c>
-      <c r="P6" s="20" t="n">
+      <c r="P6" s="19" t="n">
         <f aca="false">'Set 1'!R6</f>
         <v>656.430712583907</v>
       </c>
-      <c r="Q6" s="20" t="str">
+      <c r="Q6" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1'!S6),'Set 1'!S6,"")</f>
         <v/>
       </c>
-      <c r="R6" s="20" t="str">
+      <c r="R6" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R6),'Set 1 pseudo-2D'!R6,"")</f>
         <v/>
       </c>
-      <c r="S6" s="11" t="str">
+      <c r="S6" s="5" t="str">
         <f aca="false">IF(AND(ISNUMBER(Q6),ISNUMBER(R6)),R6-Q6,"")</f>
         <v/>
       </c>
@@ -9969,6 +10062,18 @@
       <c r="V6" s="6" t="str">
         <f aca="false">IF(AND(ISNUMBER(T6),ISNUMBER(U6)),U6-T6,"")</f>
         <v/>
+      </c>
+      <c r="W6" s="18" t="n">
+        <f aca="false">'Set 1 pseudo-2D'!E6</f>
+        <v>640</v>
+      </c>
+      <c r="X6" s="18" t="n">
+        <f aca="false">Notes!$B$4</f>
+        <v>640</v>
+      </c>
+      <c r="Y6" s="16" t="str">
+        <f aca="false">IF(AND(ISNUMBER(W6),ISNUMBER(X6)),IF(W6=X6,"yes","no"),"")</f>
+        <v>yes</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10032,19 +10137,19 @@
         <f aca="false">IF(AND(ISNUMBER(M7),ISNUMBER(N7)),N7-M7,"")</f>
         <v/>
       </c>
-      <c r="P7" s="20" t="n">
+      <c r="P7" s="19" t="n">
         <f aca="false">'Set 1'!R7</f>
         <v>661.922490247295</v>
       </c>
-      <c r="Q7" s="20" t="str">
+      <c r="Q7" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1'!S7),'Set 1'!S7,"")</f>
         <v/>
       </c>
-      <c r="R7" s="20" t="str">
+      <c r="R7" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R7),'Set 1 pseudo-2D'!R7,"")</f>
         <v/>
       </c>
-      <c r="S7" s="11" t="str">
+      <c r="S7" s="5" t="str">
         <f aca="false">IF(AND(ISNUMBER(Q7),ISNUMBER(R7)),R7-Q7,"")</f>
         <v/>
       </c>
@@ -10059,6 +10164,18 @@
       <c r="V7" s="6" t="str">
         <f aca="false">IF(AND(ISNUMBER(T7),ISNUMBER(U7)),U7-T7,"")</f>
         <v/>
+      </c>
+      <c r="W7" s="18" t="n">
+        <f aca="false">'Set 1 pseudo-2D'!E7</f>
+        <v>640</v>
+      </c>
+      <c r="X7" s="18" t="n">
+        <f aca="false">Notes!$B$4</f>
+        <v>640</v>
+      </c>
+      <c r="Y7" s="16" t="str">
+        <f aca="false">IF(AND(ISNUMBER(W7),ISNUMBER(X7)),IF(W7=X7,"yes","no"),"")</f>
+        <v>yes</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10122,19 +10239,19 @@
         <f aca="false">IF(AND(ISNUMBER(M8),ISNUMBER(N8)),N8-M8,"")</f>
         <v/>
       </c>
-      <c r="P8" s="20" t="n">
+      <c r="P8" s="19" t="n">
         <f aca="false">'Set 1'!R8</f>
         <v>722.735643650416</v>
       </c>
-      <c r="Q8" s="20" t="str">
+      <c r="Q8" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1'!S8),'Set 1'!S8,"")</f>
         <v/>
       </c>
-      <c r="R8" s="20" t="str">
+      <c r="R8" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R8),'Set 1 pseudo-2D'!R8,"")</f>
         <v/>
       </c>
-      <c r="S8" s="11" t="str">
+      <c r="S8" s="5" t="str">
         <f aca="false">IF(AND(ISNUMBER(Q8),ISNUMBER(R8)),R8-Q8,"")</f>
         <v/>
       </c>
@@ -10149,6 +10266,18 @@
       <c r="V8" s="6" t="str">
         <f aca="false">IF(AND(ISNUMBER(T8),ISNUMBER(U8)),U8-T8,"")</f>
         <v/>
+      </c>
+      <c r="W8" s="18" t="n">
+        <f aca="false">'Set 1 pseudo-2D'!E8</f>
+        <v>640</v>
+      </c>
+      <c r="X8" s="18" t="n">
+        <f aca="false">Notes!$B$4</f>
+        <v>640</v>
+      </c>
+      <c r="Y8" s="16" t="str">
+        <f aca="false">IF(AND(ISNUMBER(W8),ISNUMBER(X8)),IF(W8=X8,"yes","no"),"")</f>
+        <v>yes</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10212,19 +10341,19 @@
         <f aca="false">IF(AND(ISNUMBER(M9),ISNUMBER(N9)),N9-M9,"")</f>
         <v/>
       </c>
-      <c r="P9" s="20" t="n">
+      <c r="P9" s="19" t="n">
         <f aca="false">'Set 1'!R9</f>
         <v>731.734711525745</v>
       </c>
-      <c r="Q9" s="20" t="str">
+      <c r="Q9" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1'!S9),'Set 1'!S9,"")</f>
         <v/>
       </c>
-      <c r="R9" s="20" t="str">
+      <c r="R9" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R9),'Set 1 pseudo-2D'!R9,"")</f>
         <v/>
       </c>
-      <c r="S9" s="11" t="str">
+      <c r="S9" s="5" t="str">
         <f aca="false">IF(AND(ISNUMBER(Q9),ISNUMBER(R9)),R9-Q9,"")</f>
         <v/>
       </c>
@@ -10239,6 +10368,18 @@
       <c r="V9" s="6" t="str">
         <f aca="false">IF(AND(ISNUMBER(T9),ISNUMBER(U9)),U9-T9,"")</f>
         <v/>
+      </c>
+      <c r="W9" s="18" t="n">
+        <f aca="false">'Set 1 pseudo-2D'!E9</f>
+        <v>640</v>
+      </c>
+      <c r="X9" s="18" t="n">
+        <f aca="false">Notes!$B$4</f>
+        <v>640</v>
+      </c>
+      <c r="Y9" s="16" t="str">
+        <f aca="false">IF(AND(ISNUMBER(W9),ISNUMBER(X9)),IF(W9=X9,"yes","no"),"")</f>
+        <v>yes</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10302,19 +10443,19 @@
         <f aca="false">IF(AND(ISNUMBER(M10),ISNUMBER(N10)),N10-M10,"")</f>
         <v/>
       </c>
-      <c r="P10" s="20" t="n">
+      <c r="P10" s="19" t="n">
         <f aca="false">'Set 1'!R10</f>
         <v>741.859239328738</v>
       </c>
-      <c r="Q10" s="20" t="str">
+      <c r="Q10" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1'!S10),'Set 1'!S10,"")</f>
         <v/>
       </c>
-      <c r="R10" s="20" t="str">
+      <c r="R10" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R10),'Set 1 pseudo-2D'!R10,"")</f>
         <v/>
       </c>
-      <c r="S10" s="11" t="str">
+      <c r="S10" s="5" t="str">
         <f aca="false">IF(AND(ISNUMBER(Q10),ISNUMBER(R10)),R10-Q10,"")</f>
         <v/>
       </c>
@@ -10329,6 +10470,18 @@
       <c r="V10" s="6" t="str">
         <f aca="false">IF(AND(ISNUMBER(T10),ISNUMBER(U10)),U10-T10,"")</f>
         <v/>
+      </c>
+      <c r="W10" s="18" t="n">
+        <f aca="false">'Set 1 pseudo-2D'!E10</f>
+        <v>640</v>
+      </c>
+      <c r="X10" s="18" t="n">
+        <f aca="false">Notes!$B$4</f>
+        <v>640</v>
+      </c>
+      <c r="Y10" s="16" t="str">
+        <f aca="false">IF(AND(ISNUMBER(W10),ISNUMBER(X10)),IF(W10=X10,"yes","no"),"")</f>
+        <v>yes</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10392,19 +10545,19 @@
         <f aca="false">IF(AND(ISNUMBER(M11),ISNUMBER(N11)),N11-M11,"")</f>
         <v/>
       </c>
-      <c r="P11" s="20" t="n">
+      <c r="P11" s="19" t="n">
         <f aca="false">'Set 1'!R11</f>
         <v>749.678589646605</v>
       </c>
-      <c r="Q11" s="20" t="str">
+      <c r="Q11" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1'!S11),'Set 1'!S11,"")</f>
         <v/>
       </c>
-      <c r="R11" s="20" t="str">
+      <c r="R11" s="19" t="str">
         <f aca="false">IF(ISNUMBER('Set 1 pseudo-2D'!R11),'Set 1 pseudo-2D'!R11,"")</f>
         <v/>
       </c>
-      <c r="S11" s="11" t="str">
+      <c r="S11" s="5" t="str">
         <f aca="false">IF(AND(ISNUMBER(Q11),ISNUMBER(R11)),R11-Q11,"")</f>
         <v/>
       </c>
@@ -10420,10 +10573,22 @@
         <f aca="false">IF(AND(ISNUMBER(T11),ISNUMBER(U11)),U11-T11,"")</f>
         <v/>
       </c>
+      <c r="W11" s="18" t="n">
+        <f aca="false">'Set 1 pseudo-2D'!E11</f>
+        <v>640</v>
+      </c>
+      <c r="X11" s="18" t="n">
+        <f aca="false">Notes!$B$4</f>
+        <v>640</v>
+      </c>
+      <c r="Y11" s="16" t="str">
+        <f aca="false">IF(AND(ISNUMBER(W11),ISNUMBER(X11)),IF(W11=X11,"yes","no"),"")</f>
+        <v>yes</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="23" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10433,22 +10598,22 @@
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10462,7 +10627,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="27" t="str">
-        <f aca="false">IF(D16&gt;=3,IFERROR(CORREL(E$2:E$11,F$2:F$11),""),"")</f>
+        <f aca="false">IF(AND(D16&gt;=3,MAX(E$2:E$11)-MIN(E$2:E$11)&gt;0.000000001*(ABS(MAX(E$2:E$11))+ABS(MIN(E$2:E$11))),MAX(F$2:F$11)-MIN(F$2:F$11)&gt;0.000000001*(ABS(MAX(F$2:F$11))+ABS(MIN(F$2:F$11)))),IFERROR(CORREL(E$2:E$11,F$2:F$11),""),"")</f>
         <v/>
       </c>
       <c r="F16" s="26" t="n">
@@ -10470,7 +10635,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="27" t="str">
-        <f aca="false">IF(F16&gt;=3,IFERROR(CORREL(D$2:D$11,F$2:F$11),""),"")</f>
+        <f aca="false">IF(AND(F16&gt;=3,MAX(D$2:D$11)-MIN(D$2:D$11)&gt;0.000000001*(ABS(MAX(D$2:D$11))+ABS(MIN(D$2:D$11))),MAX(F$2:F$11)-MIN(F$2:F$11)&gt;0.000000001*(ABS(MAX(F$2:F$11))+ABS(MIN(F$2:F$11)))),IFERROR(CORREL(D$2:D$11,F$2:F$11),""),"")</f>
         <v/>
       </c>
       <c r="H16" s="26" t="n">
@@ -10478,7 +10643,7 @@
         <v>0</v>
       </c>
       <c r="I16" s="27" t="str">
-        <f aca="false">IF(H16&gt;=3,IFERROR(CORREL(D$2:D$11,E$2:E$11),""),"")</f>
+        <f aca="false">IF(AND(H16&gt;=3,MAX(D$2:D$11)-MIN(D$2:D$11)&gt;0.000000001*(ABS(MAX(D$2:D$11))+ABS(MIN(D$2:D$11))),MAX(E$2:E$11)-MIN(E$2:E$11)&gt;0.000000001*(ABS(MAX(E$2:E$11))+ABS(MIN(E$2:E$11)))),IFERROR(CORREL(D$2:D$11,E$2:E$11),""),"")</f>
         <v/>
       </c>
     </row>
@@ -10493,7 +10658,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="27" t="str">
-        <f aca="false">IF(D17&gt;=3,IFERROR(CORREL(I$2:I$11,J$2:J$11),""),"")</f>
+        <f aca="false">IF(AND(D17&gt;=3,MAX(I$2:I$11)-MIN(I$2:I$11)&gt;0.000000001*(ABS(MAX(I$2:I$11))+ABS(MIN(I$2:I$11))),MAX(J$2:J$11)-MIN(J$2:J$11)&gt;0.000000001*(ABS(MAX(J$2:J$11))+ABS(MIN(J$2:J$11)))),IFERROR(CORREL(I$2:I$11,J$2:J$11),""),"")</f>
         <v/>
       </c>
       <c r="F17" s="26" t="n">
@@ -10501,7 +10666,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="27" t="str">
-        <f aca="false">IF(F17&gt;=3,IFERROR(CORREL(H$2:H$11,J$2:J$11),""),"")</f>
+        <f aca="false">IF(AND(F17&gt;=3,MAX(H$2:H$11)-MIN(H$2:H$11)&gt;0.000000001*(ABS(MAX(H$2:H$11))+ABS(MIN(H$2:H$11))),MAX(J$2:J$11)-MIN(J$2:J$11)&gt;0.000000001*(ABS(MAX(J$2:J$11))+ABS(MIN(J$2:J$11)))),IFERROR(CORREL(H$2:H$11,J$2:J$11),""),"")</f>
         <v/>
       </c>
       <c r="H17" s="26" t="n">
@@ -10509,7 +10674,7 @@
         <v>0</v>
       </c>
       <c r="I17" s="27" t="str">
-        <f aca="false">IF(H17&gt;=3,IFERROR(CORREL(H$2:H$11,I$2:I$11),""),"")</f>
+        <f aca="false">IF(AND(H17&gt;=3,MAX(H$2:H$11)-MIN(H$2:H$11)&gt;0.000000001*(ABS(MAX(H$2:H$11))+ABS(MIN(H$2:H$11))),MAX(I$2:I$11)-MIN(I$2:I$11)&gt;0.000000001*(ABS(MAX(I$2:I$11))+ABS(MIN(I$2:I$11)))),IFERROR(CORREL(H$2:H$11,I$2:I$11),""),"")</f>
         <v/>
       </c>
     </row>
@@ -10524,7 +10689,7 @@
         <v>0</v>
       </c>
       <c r="E18" s="27" t="str">
-        <f aca="false">IF(D18&gt;=3,IFERROR(CORREL(M$2:M$11,N$2:N$11),""),"")</f>
+        <f aca="false">IF(AND(D18&gt;=3,MAX(M$2:M$11)-MIN(M$2:M$11)&gt;0.000000001*(ABS(MAX(M$2:M$11))+ABS(MIN(M$2:M$11))),MAX(N$2:N$11)-MIN(N$2:N$11)&gt;0.000000001*(ABS(MAX(N$2:N$11))+ABS(MIN(N$2:N$11)))),IFERROR(CORREL(M$2:M$11,N$2:N$11),""),"")</f>
         <v/>
       </c>
       <c r="F18" s="26" t="n">
@@ -10532,7 +10697,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="27" t="str">
-        <f aca="false">IF(F18&gt;=3,IFERROR(CORREL(L$2:L$11,N$2:N$11),""),"")</f>
+        <f aca="false">IF(AND(F18&gt;=3,MAX(L$2:L$11)-MIN(L$2:L$11)&gt;0.000000001*(ABS(MAX(L$2:L$11))+ABS(MIN(L$2:L$11))),MAX(N$2:N$11)-MIN(N$2:N$11)&gt;0.000000001*(ABS(MAX(N$2:N$11))+ABS(MIN(N$2:N$11)))),IFERROR(CORREL(L$2:L$11,N$2:N$11),""),"")</f>
         <v/>
       </c>
       <c r="H18" s="26" t="n">
@@ -10540,7 +10705,7 @@
         <v>0</v>
       </c>
       <c r="I18" s="27" t="str">
-        <f aca="false">IF(H18&gt;=3,IFERROR(CORREL(L$2:L$11,M$2:M$11),""),"")</f>
+        <f aca="false">IF(AND(H18&gt;=3,MAX(L$2:L$11)-MIN(L$2:L$11)&gt;0.000000001*(ABS(MAX(L$2:L$11))+ABS(MIN(L$2:L$11))),MAX(M$2:M$11)-MIN(M$2:M$11)&gt;0.000000001*(ABS(MAX(M$2:M$11))+ABS(MIN(M$2:M$11)))),IFERROR(CORREL(L$2:L$11,M$2:M$11),""),"")</f>
         <v/>
       </c>
     </row>
@@ -10555,7 +10720,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="27" t="str">
-        <f aca="false">IF(D19&gt;=3,IFERROR(CORREL(Q$2:Q$11,R$2:R$11),""),"")</f>
+        <f aca="false">IF(AND(D19&gt;=3,MAX(Q$2:Q$11)-MIN(Q$2:Q$11)&gt;0.000000001*(ABS(MAX(Q$2:Q$11))+ABS(MIN(Q$2:Q$11))),MAX(R$2:R$11)-MIN(R$2:R$11)&gt;0.000000001*(ABS(MAX(R$2:R$11))+ABS(MIN(R$2:R$11)))),IFERROR(CORREL(Q$2:Q$11,R$2:R$11),""),"")</f>
         <v/>
       </c>
       <c r="F19" s="26" t="n">
@@ -10563,7 +10728,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="27" t="str">
-        <f aca="false">IF(F19&gt;=3,IFERROR(CORREL(P$2:P$11,R$2:R$11),""),"")</f>
+        <f aca="false">IF(AND(F19&gt;=3,MAX(P$2:P$11)-MIN(P$2:P$11)&gt;0.000000001*(ABS(MAX(P$2:P$11))+ABS(MIN(P$2:P$11))),MAX(R$2:R$11)-MIN(R$2:R$11)&gt;0.000000001*(ABS(MAX(R$2:R$11))+ABS(MIN(R$2:R$11)))),IFERROR(CORREL(P$2:P$11,R$2:R$11),""),"")</f>
         <v/>
       </c>
       <c r="H19" s="26" t="n">
@@ -10571,7 +10736,7 @@
         <v>0</v>
       </c>
       <c r="I19" s="27" t="str">
-        <f aca="false">IF(H19&gt;=3,IFERROR(CORREL(P$2:P$11,Q$2:Q$11),""),"")</f>
+        <f aca="false">IF(AND(H19&gt;=3,MAX(P$2:P$11)-MIN(P$2:P$11)&gt;0.000000001*(ABS(MAX(P$2:P$11))+ABS(MIN(P$2:P$11))),MAX(Q$2:Q$11)-MIN(Q$2:Q$11)&gt;0.000000001*(ABS(MAX(Q$2:Q$11))+ABS(MIN(Q$2:Q$11)))),IFERROR(CORREL(P$2:P$11,Q$2:Q$11),""),"")</f>
         <v/>
       </c>
     </row>
@@ -10583,6 +10748,11 @@
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A19:C19"/>
   </mergeCells>
+  <conditionalFormatting sqref="Y2:Y11">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"no"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -10635,34 +10805,34 @@
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>42</v>
@@ -10671,22 +10841,22 @@
         <v>45</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>56</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10713,16 +10883,16 @@
         <f aca="false">Notes!$B$6</f>
         <v>10</v>
       </c>
-      <c r="G2" s="5" t="n">
-        <f aca="false">E2/C2</f>
+      <c r="G2" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(E2),E2/C2,"")</f>
         <v>1.6</v>
       </c>
       <c r="H2" s="16" t="str">
-        <f aca="false">IF(G2&gt;=1,"OK","&lt;1 period")</f>
+        <f aca="false">IF(ISNUMBER(G2),IF(G2&gt;=1,"OK","&lt;1 period"),"")</f>
         <v>OK</v>
       </c>
       <c r="I2" s="16" t="str">
-        <f aca="false">IF(ABS(G2-ROUND(G2,0))&lt;0.001,"yes","no")</f>
+        <f aca="false">IF(AND(ISNUMBER(G2),G2&gt;0),IF(ABS(G2-ROUND(G2,0))&lt;0.001,"yes","no"),"")</f>
         <v>no</v>
       </c>
       <c r="J2" s="7"/>
@@ -10731,7 +10901,7 @@
         <v>10</v>
       </c>
       <c r="M2" s="8" t="str">
-        <f aca="false">IF(AND(ISNUMBER(J2),ISNUMBER(K2),ISNUMBER(L2)),IF(AND(L2&gt;0,K2&gt;=J2),ROUNDUP((K2-J2)/L2,0)+1,""),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(J2),ISNUMBER(K2),ISNUMBER(L2)),IF(AND(L2&gt;0,K2&gt;=J2),ROUNDUP((K2-J2)/L2,0)+1,"check window"),"")</f>
         <v/>
       </c>
       <c r="N2" s="15"/>
@@ -10768,16 +10938,16 @@
         <f aca="false">Notes!$B$6</f>
         <v>10</v>
       </c>
-      <c r="G3" s="5" t="n">
-        <f aca="false">E3/C3</f>
+      <c r="G3" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(E3),E3/C3,"")</f>
         <v>1</v>
       </c>
       <c r="H3" s="16" t="str">
-        <f aca="false">IF(G3&gt;=1,"OK","&lt;1 period")</f>
+        <f aca="false">IF(ISNUMBER(G3),IF(G3&gt;=1,"OK","&lt;1 period"),"")</f>
         <v>OK</v>
       </c>
       <c r="I3" s="16" t="str">
-        <f aca="false">IF(ABS(G3-ROUND(G3,0))&lt;0.001,"yes","no")</f>
+        <f aca="false">IF(AND(ISNUMBER(G3),G3&gt;0),IF(ABS(G3-ROUND(G3,0))&lt;0.001,"yes","no"),"")</f>
         <v>yes</v>
       </c>
       <c r="J3" s="7"/>
@@ -10786,7 +10956,7 @@
         <v>10</v>
       </c>
       <c r="M3" s="8" t="str">
-        <f aca="false">IF(AND(ISNUMBER(J3),ISNUMBER(K3),ISNUMBER(L3)),IF(AND(L3&gt;0,K3&gt;=J3),ROUNDUP((K3-J3)/L3,0)+1,""),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(J3),ISNUMBER(K3),ISNUMBER(L3)),IF(AND(L3&gt;0,K3&gt;=J3),ROUNDUP((K3-J3)/L3,0)+1,"check window"),"")</f>
         <v/>
       </c>
       <c r="N3" s="15"/>
@@ -10823,16 +10993,16 @@
         <f aca="false">Notes!$B$6</f>
         <v>10</v>
       </c>
-      <c r="G4" s="5" t="n">
-        <f aca="false">E4/C4</f>
+      <c r="G4" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(E4),E4/C4,"")</f>
         <v>1.33333333333333</v>
       </c>
       <c r="H4" s="16" t="str">
-        <f aca="false">IF(G4&gt;=1,"OK","&lt;1 period")</f>
+        <f aca="false">IF(ISNUMBER(G4),IF(G4&gt;=1,"OK","&lt;1 period"),"")</f>
         <v>OK</v>
       </c>
       <c r="I4" s="16" t="str">
-        <f aca="false">IF(ABS(G4-ROUND(G4,0))&lt;0.001,"yes","no")</f>
+        <f aca="false">IF(AND(ISNUMBER(G4),G4&gt;0),IF(ABS(G4-ROUND(G4,0))&lt;0.001,"yes","no"),"")</f>
         <v>no</v>
       </c>
       <c r="J4" s="7"/>
@@ -10841,7 +11011,7 @@
         <v>10</v>
       </c>
       <c r="M4" s="8" t="str">
-        <f aca="false">IF(AND(ISNUMBER(J4),ISNUMBER(K4),ISNUMBER(L4)),IF(AND(L4&gt;0,K4&gt;=J4),ROUNDUP((K4-J4)/L4,0)+1,""),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(J4),ISNUMBER(K4),ISNUMBER(L4)),IF(AND(L4&gt;0,K4&gt;=J4),ROUNDUP((K4-J4)/L4,0)+1,"check window"),"")</f>
         <v/>
       </c>
       <c r="N4" s="15"/>
@@ -10878,16 +11048,16 @@
         <f aca="false">Notes!$B$6</f>
         <v>10</v>
       </c>
-      <c r="G5" s="5" t="n">
-        <f aca="false">E5/C5</f>
+      <c r="G5" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(E5),E5/C5,"")</f>
         <v>2.66666666666667</v>
       </c>
       <c r="H5" s="16" t="str">
-        <f aca="false">IF(G5&gt;=1,"OK","&lt;1 period")</f>
+        <f aca="false">IF(ISNUMBER(G5),IF(G5&gt;=1,"OK","&lt;1 period"),"")</f>
         <v>OK</v>
       </c>
       <c r="I5" s="16" t="str">
-        <f aca="false">IF(ABS(G5-ROUND(G5,0))&lt;0.001,"yes","no")</f>
+        <f aca="false">IF(AND(ISNUMBER(G5),G5&gt;0),IF(ABS(G5-ROUND(G5,0))&lt;0.001,"yes","no"),"")</f>
         <v>no</v>
       </c>
       <c r="J5" s="7"/>
@@ -10896,7 +11066,7 @@
         <v>10</v>
       </c>
       <c r="M5" s="8" t="str">
-        <f aca="false">IF(AND(ISNUMBER(J5),ISNUMBER(K5),ISNUMBER(L5)),IF(AND(L5&gt;0,K5&gt;=J5),ROUNDUP((K5-J5)/L5,0)+1,""),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(J5),ISNUMBER(K5),ISNUMBER(L5)),IF(AND(L5&gt;0,K5&gt;=J5),ROUNDUP((K5-J5)/L5,0)+1,"check window"),"")</f>
         <v/>
       </c>
       <c r="N5" s="15"/>
@@ -10933,16 +11103,16 @@
         <f aca="false">Notes!$B$6</f>
         <v>10</v>
       </c>
-      <c r="G6" s="5" t="n">
-        <f aca="false">E6/C6</f>
+      <c r="G6" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(E6),E6/C6,"")</f>
         <v>2.66666666666667</v>
       </c>
       <c r="H6" s="16" t="str">
-        <f aca="false">IF(G6&gt;=1,"OK","&lt;1 period")</f>
+        <f aca="false">IF(ISNUMBER(G6),IF(G6&gt;=1,"OK","&lt;1 period"),"")</f>
         <v>OK</v>
       </c>
       <c r="I6" s="16" t="str">
-        <f aca="false">IF(ABS(G6-ROUND(G6,0))&lt;0.001,"yes","no")</f>
+        <f aca="false">IF(AND(ISNUMBER(G6),G6&gt;0),IF(ABS(G6-ROUND(G6,0))&lt;0.001,"yes","no"),"")</f>
         <v>no</v>
       </c>
       <c r="J6" s="7"/>
@@ -10951,7 +11121,7 @@
         <v>10</v>
       </c>
       <c r="M6" s="8" t="str">
-        <f aca="false">IF(AND(ISNUMBER(J6),ISNUMBER(K6),ISNUMBER(L6)),IF(AND(L6&gt;0,K6&gt;=J6),ROUNDUP((K6-J6)/L6,0)+1,""),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(J6),ISNUMBER(K6),ISNUMBER(L6)),IF(AND(L6&gt;0,K6&gt;=J6),ROUNDUP((K6-J6)/L6,0)+1,"check window"),"")</f>
         <v/>
       </c>
       <c r="N6" s="15"/>
@@ -10988,16 +11158,16 @@
         <f aca="false">Notes!$B$6</f>
         <v>10</v>
       </c>
-      <c r="G7" s="5" t="n">
-        <f aca="false">E7/C7</f>
+      <c r="G7" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(E7),E7/C7,"")</f>
         <v>2</v>
       </c>
       <c r="H7" s="16" t="str">
-        <f aca="false">IF(G7&gt;=1,"OK","&lt;1 period")</f>
+        <f aca="false">IF(ISNUMBER(G7),IF(G7&gt;=1,"OK","&lt;1 period"),"")</f>
         <v>OK</v>
       </c>
       <c r="I7" s="16" t="str">
-        <f aca="false">IF(ABS(G7-ROUND(G7,0))&lt;0.001,"yes","no")</f>
+        <f aca="false">IF(AND(ISNUMBER(G7),G7&gt;0),IF(ABS(G7-ROUND(G7,0))&lt;0.001,"yes","no"),"")</f>
         <v>yes</v>
       </c>
       <c r="J7" s="7"/>
@@ -11006,7 +11176,7 @@
         <v>10</v>
       </c>
       <c r="M7" s="8" t="str">
-        <f aca="false">IF(AND(ISNUMBER(J7),ISNUMBER(K7),ISNUMBER(L7)),IF(AND(L7&gt;0,K7&gt;=J7),ROUNDUP((K7-J7)/L7,0)+1,""),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(J7),ISNUMBER(K7),ISNUMBER(L7)),IF(AND(L7&gt;0,K7&gt;=J7),ROUNDUP((K7-J7)/L7,0)+1,"check window"),"")</f>
         <v/>
       </c>
       <c r="N7" s="15"/>
@@ -11043,16 +11213,16 @@
         <f aca="false">Notes!$B$6</f>
         <v>10</v>
       </c>
-      <c r="G8" s="5" t="n">
-        <f aca="false">E8/C8</f>
+      <c r="G8" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(E8),E8/C8,"")</f>
         <v>2.66666666666667</v>
       </c>
       <c r="H8" s="16" t="str">
-        <f aca="false">IF(G8&gt;=1,"OK","&lt;1 period")</f>
+        <f aca="false">IF(ISNUMBER(G8),IF(G8&gt;=1,"OK","&lt;1 period"),"")</f>
         <v>OK</v>
       </c>
       <c r="I8" s="16" t="str">
-        <f aca="false">IF(ABS(G8-ROUND(G8,0))&lt;0.001,"yes","no")</f>
+        <f aca="false">IF(AND(ISNUMBER(G8),G8&gt;0),IF(ABS(G8-ROUND(G8,0))&lt;0.001,"yes","no"),"")</f>
         <v>no</v>
       </c>
       <c r="J8" s="7"/>
@@ -11061,7 +11231,7 @@
         <v>10</v>
       </c>
       <c r="M8" s="8" t="str">
-        <f aca="false">IF(AND(ISNUMBER(J8),ISNUMBER(K8),ISNUMBER(L8)),IF(AND(L8&gt;0,K8&gt;=J8),ROUNDUP((K8-J8)/L8,0)+1,""),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(J8),ISNUMBER(K8),ISNUMBER(L8)),IF(AND(L8&gt;0,K8&gt;=J8),ROUNDUP((K8-J8)/L8,0)+1,"check window"),"")</f>
         <v/>
       </c>
       <c r="N8" s="15"/>
@@ -11098,16 +11268,16 @@
         <f aca="false">Notes!$B$6</f>
         <v>10</v>
       </c>
-      <c r="G9" s="5" t="n">
-        <f aca="false">E9/C9</f>
+      <c r="G9" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(E9),E9/C9,"")</f>
         <v>2.66666666666667</v>
       </c>
       <c r="H9" s="16" t="str">
-        <f aca="false">IF(G9&gt;=1,"OK","&lt;1 period")</f>
+        <f aca="false">IF(ISNUMBER(G9),IF(G9&gt;=1,"OK","&lt;1 period"),"")</f>
         <v>OK</v>
       </c>
       <c r="I9" s="16" t="str">
-        <f aca="false">IF(ABS(G9-ROUND(G9,0))&lt;0.001,"yes","no")</f>
+        <f aca="false">IF(AND(ISNUMBER(G9),G9&gt;0),IF(ABS(G9-ROUND(G9,0))&lt;0.001,"yes","no"),"")</f>
         <v>no</v>
       </c>
       <c r="J9" s="7"/>
@@ -11116,7 +11286,7 @@
         <v>10</v>
       </c>
       <c r="M9" s="8" t="str">
-        <f aca="false">IF(AND(ISNUMBER(J9),ISNUMBER(K9),ISNUMBER(L9)),IF(AND(L9&gt;0,K9&gt;=J9),ROUNDUP((K9-J9)/L9,0)+1,""),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(J9),ISNUMBER(K9),ISNUMBER(L9)),IF(AND(L9&gt;0,K9&gt;=J9),ROUNDUP((K9-J9)/L9,0)+1,"check window"),"")</f>
         <v/>
       </c>
       <c r="N9" s="15"/>
@@ -11153,16 +11323,16 @@
         <f aca="false">Notes!$B$6</f>
         <v>10</v>
       </c>
-      <c r="G10" s="5" t="n">
-        <f aca="false">E10/C10</f>
+      <c r="G10" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(E10),E10/C10,"")</f>
         <v>4</v>
       </c>
       <c r="H10" s="16" t="str">
-        <f aca="false">IF(G10&gt;=1,"OK","&lt;1 period")</f>
+        <f aca="false">IF(ISNUMBER(G10),IF(G10&gt;=1,"OK","&lt;1 period"),"")</f>
         <v>OK</v>
       </c>
       <c r="I10" s="16" t="str">
-        <f aca="false">IF(ABS(G10-ROUND(G10,0))&lt;0.001,"yes","no")</f>
+        <f aca="false">IF(AND(ISNUMBER(G10),G10&gt;0),IF(ABS(G10-ROUND(G10,0))&lt;0.001,"yes","no"),"")</f>
         <v>yes</v>
       </c>
       <c r="J10" s="7"/>
@@ -11171,7 +11341,7 @@
         <v>10</v>
       </c>
       <c r="M10" s="8" t="str">
-        <f aca="false">IF(AND(ISNUMBER(J10),ISNUMBER(K10),ISNUMBER(L10)),IF(AND(L10&gt;0,K10&gt;=J10),ROUNDUP((K10-J10)/L10,0)+1,""),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(J10),ISNUMBER(K10),ISNUMBER(L10)),IF(AND(L10&gt;0,K10&gt;=J10),ROUNDUP((K10-J10)/L10,0)+1,"check window"),"")</f>
         <v/>
       </c>
       <c r="N10" s="15"/>
@@ -11208,16 +11378,16 @@
         <f aca="false">Notes!$B$6</f>
         <v>10</v>
       </c>
-      <c r="G11" s="5" t="n">
-        <f aca="false">E11/C11</f>
+      <c r="G11" s="6" t="n">
+        <f aca="false">IF(ISNUMBER(E11),E11/C11,"")</f>
         <v>4</v>
       </c>
       <c r="H11" s="16" t="str">
-        <f aca="false">IF(G11&gt;=1,"OK","&lt;1 period")</f>
+        <f aca="false">IF(ISNUMBER(G11),IF(G11&gt;=1,"OK","&lt;1 period"),"")</f>
         <v>OK</v>
       </c>
       <c r="I11" s="16" t="str">
-        <f aca="false">IF(ABS(G11-ROUND(G11,0))&lt;0.001,"yes","no")</f>
+        <f aca="false">IF(AND(ISNUMBER(G11),G11&gt;0),IF(ABS(G11-ROUND(G11,0))&lt;0.001,"yes","no"),"")</f>
         <v>yes</v>
       </c>
       <c r="J11" s="7"/>
@@ -11226,7 +11396,7 @@
         <v>10</v>
       </c>
       <c r="M11" s="8" t="str">
-        <f aca="false">IF(AND(ISNUMBER(J11),ISNUMBER(K11),ISNUMBER(L11)),IF(AND(L11&gt;0,K11&gt;=J11),ROUNDUP((K11-J11)/L11,0)+1,""),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(J11),ISNUMBER(K11),ISNUMBER(L11)),IF(AND(L11&gt;0,K11&gt;=J11),ROUNDUP((K11-J11)/L11,0)+1,"check window"),"")</f>
         <v/>
       </c>
       <c r="N11" s="15"/>
@@ -11267,22 +11437,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="28" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="28" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="29" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -11303,7 +11473,7 @@
     <tabColor rgb="FF7F7F7F"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -11313,148 +11483,148 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="30" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="31" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="32" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="33" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B4" s="34" t="n">
         <v>640</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="33" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B5" s="34" t="n">
         <v>640</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="33" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B6" s="34" t="n">
         <v>10</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="35" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="36" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="37" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="38" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="33" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="39" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="39" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="39" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="39" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="39" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="39" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11462,7 +11632,7 @@
         <v>18</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11470,7 +11640,7 @@
         <v>19</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11478,47 +11648,47 @@
         <v>24</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="39" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="39" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="39" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="39" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="39" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11526,20 +11696,20 @@
         <v>1</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="33" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C32" s="33" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11600,66 +11770,80 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="32" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="33" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="33" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="33" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="33" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="33" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C46" s="33" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="33" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="33" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>142</v>
+        <v>145</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="33" t="s">
+        <v>138</v>
+      </c>
+      <c r="C49" s="33" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="false" error="Enter a number greater than 0." errorStyle="stop" errorTitle="Number needed" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B4:B6" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>